<commit_message>
update: add ASVS 5.0 Tracker and remove outdated mitigations document
</commit_message>
<xml_diff>
--- a/Deliverables/Phase_1/ASVS_5.0_Tracker.xlsx
+++ b/Deliverables/Phase_1/ASVS_5.0_Tracker.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24332"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mateus Fernandes\Desktop\ISEP\Mestrado\DESOFS\thu_crr_2\Deliverables\Phase_1\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Utilizador\Desktop\DESOFS\desofs2026-thu_crr_2\Deliverables\Phase_1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5A8E851-D22B-4E3F-8556-D5E844C41096}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B1366F7-E48A-4B1A-9830-CE29546F8FAE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1950" yWindow="1950" windowWidth="21600" windowHeight="11385" tabRatio="500" firstSheet="13" activeTab="14" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
@@ -41,8 +41,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
@@ -53,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2239" uniqueCount="985">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2337" uniqueCount="996">
   <si>
     <t>OWASP ASVS 5.0 – Compliance Tracker</t>
   </si>
@@ -3020,13 +3018,46 @@
   </si>
   <si>
     <t>Compliant</t>
+  </si>
+  <si>
+    <t>src/middlewares/errorHandler.ts generic 500 message to client; full detail to server logs only. Controllers sanitized to remove error.message leaks.</t>
+  </si>
+  <si>
+    <t>errorHandler.ts, index.ts - central handler catches all unhandled exceptions.</t>
+  </si>
+  <si>
+    <t>errorHandler.ts, index.ts - registered as last middleware via app.use(errorHandler).</t>
+  </si>
+  <si>
+    <t>errorHandler.ts — req.method and req.path stripped of \r\n before logging; %s format specifiers used to prevent log injection.</t>
+  </si>
+  <si>
+    <t>index.ts -  express.json({ limit: "1mb" }) set to reject oversized payloads before reaching controllers.</t>
+  </si>
+  <si>
+    <t>ApplicationRoutes.ts - multer limits.fileSize set to 5 MB; max 10 files per request.</t>
+  </si>
+  <si>
+    <t>validatePdfMagicBytes.ts, ApplicationController.ts - magic bytes (%PDF) checked after upload; invalid files deleted immediately.</t>
+  </si>
+  <si>
+    <t>sanitizeFilename.ts, ApplicationController.ts - filename sanitized and resolved path validated to stay within uploads/ directory; prevents path traversal.</t>
+  </si>
+  <si>
+    <t>index.ts - express.static for /uploads removed; files no longer publicly accessible.</t>
+  </si>
+  <si>
+    <t>ApplicationController.ts, authMiddleware.ts - getDocument checks ownership; only document owner (Visitor) or NetworkManager can access.</t>
+  </si>
+  <si>
+    <t>authMiddleware.ts - token read exclusively from Authorization header, never from query string.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -3091,6 +3122,14 @@
       <sz val="10"/>
       <color rgb="FF1F3864"/>
       <name val="Cambria"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <charset val="1"/>
     </font>
   </fonts>
@@ -3188,7 +3227,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -3263,6 +3302,10 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3499,7 +3542,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.25</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="5">
                   <c:v>0.15384615384615385</c:v>
@@ -3508,7 +3551,7 @@
                   <c:v>0.16666666666666666</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0</c:v>
+                  <c:v>0.25</c:v>
                 </c:pt>
                 <c:pt idx="8">
                   <c:v>0.5</c:v>
@@ -3526,7 +3569,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>0</c:v>
+                  <c:v>0.5</c:v>
                 </c:pt>
                 <c:pt idx="14">
                   <c:v>0</c:v>
@@ -3713,10 +3756,10 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>0</c:v>
+                  <c:v>0.1</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>0</c:v>
+                  <c:v>0.1875</c:v>
                 </c:pt>
                 <c:pt idx="16">
                   <c:v>0</c:v>
@@ -3900,7 +3943,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>0</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4048,7 +4091,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>7.6923076923076927E-2</c:v>
+                  <c:v>0.30769230769230771</c:v>
                 </c:pt>
                 <c:pt idx="5">
                   <c:v>8.5106382978723402E-2</c:v>
@@ -4057,7 +4100,7 @@
                   <c:v>5.2631578947368418E-2</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0</c:v>
+                  <c:v>7.6923076923076927E-2</c:v>
                 </c:pt>
                 <c:pt idx="8">
                   <c:v>0.2857142857142857</c:v>
@@ -4075,13 +4118,13 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>0</c:v>
+                  <c:v>7.6923076923076927E-2</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>0</c:v>
+                  <c:v>4.7619047619047616E-2</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>0</c:v>
+                  <c:v>0.23529411764705882</c:v>
                 </c:pt>
                 <c:pt idx="16">
                   <c:v>0</c:v>
@@ -4597,13 +4640,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:P23"/>
-  <sheetFormatPr defaultColWidth="8.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="34" customWidth="1"/>
     <col min="2" max="13" width="11" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="36" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:16" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="25" t="s">
         <v>0</v>
       </c>
@@ -4623,7 +4666,7 @@
       <c r="O1" s="25"/>
       <c r="P1" s="25"/>
     </row>
-    <row r="2" spans="1:16" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:16" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="26"/>
       <c r="B2" s="26"/>
       <c r="C2" s="26"/>
@@ -4641,7 +4684,7 @@
       <c r="O2" s="26"/>
       <c r="P2" s="26"/>
     </row>
-    <row r="3" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="27"/>
       <c r="B3" s="27"/>
       <c r="C3" s="1"/>
@@ -4652,7 +4695,7 @@
       <c r="M3" s="1"/>
       <c r="O3" s="1"/>
     </row>
-    <row r="5" spans="1:16" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:16" ht="31.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>1</v>
       </c>
@@ -4693,7 +4736,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="6" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>14</v>
       </c>
@@ -4742,7 +4785,7 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="7" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
         <v>15</v>
       </c>
@@ -4791,7 +4834,7 @@
         <v>7.6923076923076927E-2</v>
       </c>
     </row>
-    <row r="8" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>16</v>
       </c>
@@ -4840,7 +4883,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
         <v>17</v>
       </c>
@@ -4889,7 +4932,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>18</v>
       </c>
@@ -4901,11 +4944,11 @@
       </c>
       <c r="D10" s="4">
         <f>COUNTIFS('V5 - File Handling'!$F$2:$F$18,"Compliant",'V5 - File Handling'!$E$2:$E$18,1)</f>
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E10" s="5">
         <f t="shared" si="0"/>
-        <v>0.25</v>
+        <v>1</v>
       </c>
       <c r="F10" s="4">
         <v>5</v>
@@ -4931,14 +4974,14 @@
       </c>
       <c r="L10" s="4">
         <f>COUNTIF('V5 - File Handling'!$F$2:$F$18,"Compliant")</f>
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="M10" s="5">
         <f t="shared" si="3"/>
-        <v>7.6923076923076927E-2</v>
-      </c>
-    </row>
-    <row r="11" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+        <v>0.30769230769230771</v>
+      </c>
+    </row>
+    <row r="11" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="6" t="s">
         <v>19</v>
       </c>
@@ -4987,7 +5030,7 @@
         <v>8.5106382978723402E-2</v>
       </c>
     </row>
-    <row r="12" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>20</v>
       </c>
@@ -5036,7 +5079,7 @@
         <v>5.2631578947368418E-2</v>
       </c>
     </row>
-    <row r="13" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
         <v>21</v>
       </c>
@@ -5048,11 +5091,11 @@
       </c>
       <c r="D13" s="7">
         <f>COUNTIFS('V8 - Authorization'!$F$2:$F$18,"Compliant",'V8 - Authorization'!$E$2:$E$18,1)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E13" s="8">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="F13" s="7">
         <v>3</v>
@@ -5078,14 +5121,14 @@
       </c>
       <c r="L13" s="7">
         <f>COUNTIF('V8 - Authorization'!$F$2:$F$18,"Compliant")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M13" s="8">
         <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+        <v>7.6923076923076927E-2</v>
+      </c>
+    </row>
+    <row r="14" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>22</v>
       </c>
@@ -5132,7 +5175,7 @@
         <v>0.2857142857142857</v>
       </c>
     </row>
-    <row r="15" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="6" t="s">
         <v>24</v>
       </c>
@@ -5181,7 +5224,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>25</v>
       </c>
@@ -5230,7 +5273,7 @@
         <v>4.1666666666666664E-2</v>
       </c>
     </row>
-    <row r="17" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="6" t="s">
         <v>26</v>
       </c>
@@ -5279,7 +5322,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
         <v>27</v>
       </c>
@@ -5328,7 +5371,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="6" t="s">
         <v>28</v>
       </c>
@@ -5340,11 +5383,11 @@
       </c>
       <c r="D19" s="7">
         <f>COUNTIFS('V14 - Data Protection'!$F$2:$F$17,"Compliant",'V14 - Data Protection'!$E$2:$E$17,1)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E19" s="8">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="F19" s="7">
         <v>7</v>
@@ -5370,14 +5413,14 @@
       </c>
       <c r="L19" s="7">
         <f>COUNTIF('V14 - Data Protection'!$F$2:$F$17,"Compliant")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M19" s="8">
         <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="20" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+        <v>7.6923076923076927E-2</v>
+      </c>
+    </row>
+    <row r="20" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
         <v>29</v>
       </c>
@@ -5400,11 +5443,11 @@
       </c>
       <c r="G20" s="4">
         <f>COUNTIFS('V15 - Secure Coding and Archite'!$F$2:$F$26,"Compliant",'V15 - Secure Coding and Archite'!$E$2:$E$26,2)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H20" s="5">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="I20" s="4">
         <v>8</v>
@@ -5419,14 +5462,14 @@
       </c>
       <c r="L20" s="4">
         <f>COUNTIF('V15 - Secure Coding and Archite'!$F$2:$F$26,"Compliant")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M20" s="5">
         <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="21" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+        <v>4.7619047619047616E-2</v>
+      </c>
+    </row>
+    <row r="21" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="6" t="s">
         <v>30</v>
       </c>
@@ -5447,33 +5490,33 @@
       </c>
       <c r="G21" s="7">
         <f>COUNTIFS('V16 - Security Logging and Erro'!$F$2:$F$23,"Compliant",'V16 - Security Logging and Erro'!$E$2:$E$23,2)</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H21" s="8">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.1875</v>
       </c>
       <c r="I21" s="7">
         <v>1</v>
       </c>
       <c r="J21" s="7">
         <f>COUNTIFS('V16 - Security Logging and Erro'!$F$2:$F$23,"Compliant",'V16 - Security Logging and Erro'!$E$2:$E$23,3)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K21" s="8">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L21" s="7">
         <f>COUNTIF('V16 - Security Logging and Erro'!$F$2:$F$23,"Compliant")</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="M21" s="8">
         <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="22" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+        <v>0.23529411764705882</v>
+      </c>
+    </row>
+    <row r="22" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
         <v>31</v>
       </c>
@@ -5520,7 +5563,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:13" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:13" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="9" t="s">
         <v>32</v>
       </c>
@@ -5534,11 +5577,11 @@
       </c>
       <c r="D23" s="10">
         <f>SUM(D6:D22)</f>
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="E23" s="11">
         <f>IFERROR(AVERAGE(E6:E22),"")</f>
-        <v>0.13525641025641025</v>
+        <v>0.23525641025641025</v>
       </c>
       <c r="F23" s="10">
         <f>SUM(F6:F22)</f>
@@ -5546,11 +5589,11 @@
       </c>
       <c r="G23" s="10">
         <f>SUM(G6:G22)</f>
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="H23" s="11">
         <f>IFERROR(AVERAGE(H6:H22),"")</f>
-        <v>5.3475935828877011E-3</v>
+        <v>2.2259358288770053E-2</v>
       </c>
       <c r="I23" s="10">
         <f>SUM(I6:I22)</f>
@@ -5558,19 +5601,19 @@
       </c>
       <c r="J23" s="10">
         <f>SUM(J6:J22)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K23" s="11">
         <f>IFERROR(AVERAGE(K6:K22),"")</f>
-        <v>0</v>
+        <v>6.25E-2</v>
       </c>
       <c r="L23" s="10">
         <f>SUM(L6:L22)</f>
-        <v>13</v>
+        <v>23</v>
       </c>
       <c r="M23" s="11">
         <f>IFERROR(AVERAGE(M6:M22),"")</f>
-        <v>4.2292062832541055E-2</v>
+        <v>8.1558448119687599E-2</v>
       </c>
     </row>
   </sheetData>
@@ -5636,7 +5679,7 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
   <dimension ref="A1:H10"/>
-  <sheetFormatPr defaultColWidth="8.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
@@ -5648,7 +5691,7 @@
     <col min="8" max="8" width="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" ht="28.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="12" t="s">
         <v>33</v>
       </c>
@@ -5674,7 +5717,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="13" t="s">
         <v>490</v>
       </c>
@@ -5688,7 +5731,7 @@
       <c r="G2" s="13"/>
       <c r="H2" s="13"/>
     </row>
-    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
         <v>490</v>
       </c>
@@ -5710,7 +5753,7 @@
       <c r="G3" s="16"/>
       <c r="H3" s="16"/>
     </row>
-    <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="19" t="s">
         <v>490</v>
       </c>
@@ -5732,7 +5775,7 @@
       <c r="G4" s="21"/>
       <c r="H4" s="21"/>
     </row>
-    <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
         <v>490</v>
       </c>
@@ -5754,7 +5797,7 @@
       <c r="G5" s="16"/>
       <c r="H5" s="16"/>
     </row>
-    <row r="6" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="13" t="s">
         <v>498</v>
       </c>
@@ -5768,7 +5811,7 @@
       <c r="G6" s="13"/>
       <c r="H6" s="13"/>
     </row>
-    <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="14" t="s">
         <v>498</v>
       </c>
@@ -5790,7 +5833,7 @@
       <c r="G7" s="16"/>
       <c r="H7" s="16"/>
     </row>
-    <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="19" t="s">
         <v>498</v>
       </c>
@@ -5814,7 +5857,7 @@
         <v>910</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="14" t="s">
         <v>498</v>
       </c>
@@ -5838,7 +5881,7 @@
         <v>916</v>
       </c>
     </row>
-    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="19" t="s">
         <v>498</v>
       </c>
@@ -5888,7 +5931,7 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
   <dimension ref="A1:H44"/>
-  <sheetFormatPr defaultColWidth="8.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
@@ -5900,7 +5943,7 @@
     <col min="8" max="8" width="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" ht="28.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="12" t="s">
         <v>33</v>
       </c>
@@ -5926,7 +5969,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="13" t="s">
         <v>508</v>
       </c>
@@ -5940,7 +5983,7 @@
       <c r="G2" s="13"/>
       <c r="H2" s="13"/>
     </row>
-    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
         <v>508</v>
       </c>
@@ -5964,7 +6007,7 @@
         <v>910</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="19" t="s">
         <v>508</v>
       </c>
@@ -5988,7 +6031,7 @@
         <v>928</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="13" t="s">
         <v>514</v>
       </c>
@@ -6002,7 +6045,7 @@
       <c r="G5" s="13"/>
       <c r="H5" s="13"/>
     </row>
-    <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="14" t="s">
         <v>514</v>
       </c>
@@ -6026,7 +6069,7 @@
         <v>921</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="19" t="s">
         <v>514</v>
       </c>
@@ -6050,7 +6093,7 @@
         <v>910</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="14" t="s">
         <v>514</v>
       </c>
@@ -6072,7 +6115,7 @@
       <c r="G8" s="16"/>
       <c r="H8" s="16"/>
     </row>
-    <row r="9" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="13" t="s">
         <v>522</v>
       </c>
@@ -6086,7 +6129,7 @@
       <c r="G9" s="13"/>
       <c r="H9" s="13"/>
     </row>
-    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="14" t="s">
         <v>522</v>
       </c>
@@ -6110,7 +6153,7 @@
         <v>916</v>
       </c>
     </row>
-    <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="19" t="s">
         <v>522</v>
       </c>
@@ -6134,7 +6177,7 @@
         <v>916</v>
       </c>
     </row>
-    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="14" t="s">
         <v>522</v>
       </c>
@@ -6158,7 +6201,7 @@
         <v>929</v>
       </c>
     </row>
-    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="19" t="s">
         <v>522</v>
       </c>
@@ -6182,7 +6225,7 @@
         <v>916</v>
       </c>
     </row>
-    <row r="14" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="14" t="s">
         <v>522</v>
       </c>
@@ -6204,7 +6247,7 @@
       <c r="G14" s="16"/>
       <c r="H14" s="16"/>
     </row>
-    <row r="15" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="13" t="s">
         <v>534</v>
       </c>
@@ -6218,7 +6261,7 @@
       <c r="G15" s="13"/>
       <c r="H15" s="13"/>
     </row>
-    <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="14" t="s">
         <v>534</v>
       </c>
@@ -6240,7 +6283,7 @@
       <c r="G16" s="16"/>
       <c r="H16" s="16"/>
     </row>
-    <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="19" t="s">
         <v>534</v>
       </c>
@@ -6262,7 +6305,7 @@
       <c r="G17" s="21"/>
       <c r="H17" s="21"/>
     </row>
-    <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="14" t="s">
         <v>534</v>
       </c>
@@ -6284,7 +6327,7 @@
       <c r="G18" s="16"/>
       <c r="H18" s="16"/>
     </row>
-    <row r="19" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="19" t="s">
         <v>534</v>
       </c>
@@ -6306,7 +6349,7 @@
       <c r="G19" s="21"/>
       <c r="H19" s="21"/>
     </row>
-    <row r="20" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="14" t="s">
         <v>534</v>
       </c>
@@ -6328,7 +6371,7 @@
       <c r="G20" s="16"/>
       <c r="H20" s="16"/>
     </row>
-    <row r="21" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="19" t="s">
         <v>534</v>
       </c>
@@ -6352,7 +6395,7 @@
         <v>921</v>
       </c>
     </row>
-    <row r="22" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="14" t="s">
         <v>534</v>
       </c>
@@ -6376,7 +6419,7 @@
         <v>930</v>
       </c>
     </row>
-    <row r="23" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="19" t="s">
         <v>534</v>
       </c>
@@ -6400,7 +6443,7 @@
         <v>931</v>
       </c>
     </row>
-    <row r="24" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="14" t="s">
         <v>534</v>
       </c>
@@ -6424,7 +6467,7 @@
         <v>925</v>
       </c>
     </row>
-    <row r="25" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="19" t="s">
         <v>534</v>
       </c>
@@ -6448,7 +6491,7 @@
         <v>916</v>
       </c>
     </row>
-    <row r="26" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="14" t="s">
         <v>534</v>
       </c>
@@ -6472,7 +6515,7 @@
         <v>903</v>
       </c>
     </row>
-    <row r="27" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="19" t="s">
         <v>534</v>
       </c>
@@ -6494,7 +6537,7 @@
       <c r="G27" s="21"/>
       <c r="H27" s="21"/>
     </row>
-    <row r="28" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="14" t="s">
         <v>534</v>
       </c>
@@ -6516,7 +6559,7 @@
       <c r="G28" s="16"/>
       <c r="H28" s="16"/>
     </row>
-    <row r="29" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="19" t="s">
         <v>534</v>
       </c>
@@ -6538,7 +6581,7 @@
       <c r="G29" s="21"/>
       <c r="H29" s="21"/>
     </row>
-    <row r="30" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="14" t="s">
         <v>534</v>
       </c>
@@ -6560,7 +6603,7 @@
       <c r="G30" s="16"/>
       <c r="H30" s="16"/>
     </row>
-    <row r="31" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="19" t="s">
         <v>534</v>
       </c>
@@ -6582,7 +6625,7 @@
       <c r="G31" s="21"/>
       <c r="H31" s="21"/>
     </row>
-    <row r="32" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="13" t="s">
         <v>568</v>
       </c>
@@ -6596,7 +6639,7 @@
       <c r="G32" s="13"/>
       <c r="H32" s="13"/>
     </row>
-    <row r="33" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="14" t="s">
         <v>568</v>
       </c>
@@ -6620,7 +6663,7 @@
         <v>919</v>
       </c>
     </row>
-    <row r="34" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="19" t="s">
         <v>568</v>
       </c>
@@ -6644,7 +6687,7 @@
         <v>929</v>
       </c>
     </row>
-    <row r="35" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="14" t="s">
         <v>568</v>
       </c>
@@ -6668,7 +6711,7 @@
         <v>910</v>
       </c>
     </row>
-    <row r="36" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="19" t="s">
         <v>568</v>
       </c>
@@ -6692,7 +6735,7 @@
         <v>916</v>
       </c>
     </row>
-    <row r="37" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="14" t="s">
         <v>568</v>
       </c>
@@ -6716,7 +6759,7 @@
         <v>919</v>
       </c>
     </row>
-    <row r="38" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="13" t="s">
         <v>580</v>
       </c>
@@ -6730,7 +6773,7 @@
       <c r="G38" s="13"/>
       <c r="H38" s="13"/>
     </row>
-    <row r="39" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="14" t="s">
         <v>580</v>
       </c>
@@ -6754,7 +6797,7 @@
         <v>928</v>
       </c>
     </row>
-    <row r="40" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="19" t="s">
         <v>580</v>
       </c>
@@ -6778,7 +6821,7 @@
         <v>927</v>
       </c>
     </row>
-    <row r="41" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="13" t="s">
         <v>586</v>
       </c>
@@ -6792,7 +6835,7 @@
       <c r="G41" s="13"/>
       <c r="H41" s="13"/>
     </row>
-    <row r="42" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="14" t="s">
         <v>586</v>
       </c>
@@ -6816,7 +6859,7 @@
         <v>903</v>
       </c>
     </row>
-    <row r="43" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="19" t="s">
         <v>586</v>
       </c>
@@ -6840,7 +6883,7 @@
         <v>932</v>
       </c>
     </row>
-    <row r="44" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="14" t="s">
         <v>586</v>
       </c>
@@ -6890,7 +6933,7 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0B00-000000000000}">
   <dimension ref="A1:H32"/>
-  <sheetFormatPr defaultColWidth="8.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
@@ -6902,7 +6945,7 @@
     <col min="8" max="8" width="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" ht="28.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="12" t="s">
         <v>33</v>
       </c>
@@ -6928,7 +6971,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="13" t="s">
         <v>594</v>
       </c>
@@ -6942,7 +6985,7 @@
       <c r="G2" s="13"/>
       <c r="H2" s="13"/>
     </row>
-    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
         <v>594</v>
       </c>
@@ -6966,7 +7009,7 @@
         <v>933</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="19" t="s">
         <v>594</v>
       </c>
@@ -6990,7 +7033,7 @@
         <v>934</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
         <v>594</v>
       </c>
@@ -7012,7 +7055,7 @@
       <c r="G5" s="16"/>
       <c r="H5" s="16"/>
     </row>
-    <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="19" t="s">
         <v>594</v>
       </c>
@@ -7034,7 +7077,7 @@
       <c r="G6" s="21"/>
       <c r="H6" s="21"/>
     </row>
-    <row r="7" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="13" t="s">
         <v>604</v>
       </c>
@@ -7048,7 +7091,7 @@
       <c r="G7" s="13"/>
       <c r="H7" s="13"/>
     </row>
-    <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="14" t="s">
         <v>604</v>
       </c>
@@ -7072,7 +7115,7 @@
         <v>934</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="19" t="s">
         <v>604</v>
       </c>
@@ -7096,7 +7139,7 @@
         <v>934</v>
       </c>
     </row>
-    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="14" t="s">
         <v>604</v>
       </c>
@@ -7120,7 +7163,7 @@
         <v>934</v>
       </c>
     </row>
-    <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="19" t="s">
         <v>604</v>
       </c>
@@ -7142,7 +7185,7 @@
       <c r="G11" s="21"/>
       <c r="H11" s="21"/>
     </row>
-    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="14" t="s">
         <v>604</v>
       </c>
@@ -7164,7 +7207,7 @@
       <c r="G12" s="16"/>
       <c r="H12" s="16"/>
     </row>
-    <row r="13" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="13" t="s">
         <v>616</v>
       </c>
@@ -7178,7 +7221,7 @@
       <c r="G13" s="13"/>
       <c r="H13" s="13"/>
     </row>
-    <row r="14" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="14" t="s">
         <v>616</v>
       </c>
@@ -7200,7 +7243,7 @@
       <c r="G14" s="16"/>
       <c r="H14" s="16"/>
     </row>
-    <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="19" t="s">
         <v>616</v>
       </c>
@@ -7222,7 +7265,7 @@
       <c r="G15" s="21"/>
       <c r="H15" s="21"/>
     </row>
-    <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="14" t="s">
         <v>616</v>
       </c>
@@ -7246,7 +7289,7 @@
         <v>904</v>
       </c>
     </row>
-    <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="19" t="s">
         <v>616</v>
       </c>
@@ -7268,7 +7311,7 @@
       <c r="G17" s="21"/>
       <c r="H17" s="21"/>
     </row>
-    <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="14" t="s">
         <v>616</v>
       </c>
@@ -7290,7 +7333,7 @@
       <c r="G18" s="16"/>
       <c r="H18" s="16"/>
     </row>
-    <row r="19" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="13" t="s">
         <v>628</v>
       </c>
@@ -7304,7 +7347,7 @@
       <c r="G19" s="13"/>
       <c r="H19" s="13"/>
     </row>
-    <row r="20" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="14" t="s">
         <v>628</v>
       </c>
@@ -7326,7 +7369,7 @@
       <c r="G20" s="16"/>
       <c r="H20" s="16"/>
     </row>
-    <row r="21" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="19" t="s">
         <v>628</v>
       </c>
@@ -7350,7 +7393,7 @@
         <v>935</v>
       </c>
     </row>
-    <row r="22" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="14" t="s">
         <v>628</v>
       </c>
@@ -7374,7 +7417,7 @@
         <v>936</v>
       </c>
     </row>
-    <row r="23" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="19" t="s">
         <v>628</v>
       </c>
@@ -7398,7 +7441,7 @@
         <v>935</v>
       </c>
     </row>
-    <row r="24" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="13" t="s">
         <v>638</v>
       </c>
@@ -7412,7 +7455,7 @@
       <c r="G24" s="13"/>
       <c r="H24" s="13"/>
     </row>
-    <row r="25" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="14" t="s">
         <v>638</v>
       </c>
@@ -7436,7 +7479,7 @@
         <v>918</v>
       </c>
     </row>
-    <row r="26" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="19" t="s">
         <v>638</v>
       </c>
@@ -7458,7 +7501,7 @@
       <c r="G26" s="21"/>
       <c r="H26" s="21"/>
     </row>
-    <row r="27" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="13" t="s">
         <v>644</v>
       </c>
@@ -7472,7 +7515,7 @@
       <c r="G27" s="13"/>
       <c r="H27" s="13"/>
     </row>
-    <row r="28" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="14" t="s">
         <v>644</v>
       </c>
@@ -7496,7 +7539,7 @@
         <v>934</v>
       </c>
     </row>
-    <row r="29" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="19" t="s">
         <v>644</v>
       </c>
@@ -7518,7 +7561,7 @@
       <c r="G29" s="21"/>
       <c r="H29" s="21"/>
     </row>
-    <row r="30" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="13" t="s">
         <v>650</v>
       </c>
@@ -7532,7 +7575,7 @@
       <c r="G30" s="13"/>
       <c r="H30" s="13"/>
     </row>
-    <row r="31" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="14" t="s">
         <v>650</v>
       </c>
@@ -7554,7 +7597,7 @@
       <c r="G31" s="16"/>
       <c r="H31" s="16"/>
     </row>
-    <row r="32" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="19" t="s">
         <v>650</v>
       </c>
@@ -7602,7 +7645,7 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0C00-000000000000}">
   <dimension ref="A1:H16"/>
-  <sheetFormatPr defaultColWidth="8.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
@@ -7614,7 +7657,7 @@
     <col min="8" max="8" width="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" ht="28.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="12" t="s">
         <v>33</v>
       </c>
@@ -7640,7 +7683,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="13" t="s">
         <v>656</v>
       </c>
@@ -7654,7 +7697,7 @@
       <c r="G2" s="13"/>
       <c r="H2" s="13"/>
     </row>
-    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
         <v>656</v>
       </c>
@@ -7676,7 +7719,7 @@
       <c r="G3" s="16"/>
       <c r="H3" s="16"/>
     </row>
-    <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="19" t="s">
         <v>656</v>
       </c>
@@ -7700,7 +7743,7 @@
         <v>937</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
         <v>656</v>
       </c>
@@ -7724,7 +7767,7 @@
         <v>938</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="19" t="s">
         <v>656</v>
       </c>
@@ -7746,7 +7789,7 @@
       <c r="G6" s="21"/>
       <c r="H6" s="21"/>
     </row>
-    <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="14" t="s">
         <v>656</v>
       </c>
@@ -7768,7 +7811,7 @@
       <c r="G7" s="16"/>
       <c r="H7" s="16"/>
     </row>
-    <row r="8" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="13" t="s">
         <v>668</v>
       </c>
@@ -7782,7 +7825,7 @@
       <c r="G8" s="13"/>
       <c r="H8" s="13"/>
     </row>
-    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="14" t="s">
         <v>668</v>
       </c>
@@ -7804,7 +7847,7 @@
       <c r="G9" s="16"/>
       <c r="H9" s="16"/>
     </row>
-    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="19" t="s">
         <v>668</v>
       </c>
@@ -7826,7 +7869,7 @@
       <c r="G10" s="21"/>
       <c r="H10" s="21"/>
     </row>
-    <row r="11" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="13" t="s">
         <v>674</v>
       </c>
@@ -7840,7 +7883,7 @@
       <c r="G11" s="13"/>
       <c r="H11" s="13"/>
     </row>
-    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="14" t="s">
         <v>674</v>
       </c>
@@ -7864,7 +7907,7 @@
         <v>937</v>
       </c>
     </row>
-    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="19" t="s">
         <v>674</v>
       </c>
@@ -7888,7 +7931,7 @@
         <v>939</v>
       </c>
     </row>
-    <row r="14" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="14" t="s">
         <v>674</v>
       </c>
@@ -7912,7 +7955,7 @@
         <v>937</v>
       </c>
     </row>
-    <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="19" t="s">
         <v>674</v>
       </c>
@@ -7936,7 +7979,7 @@
         <v>940</v>
       </c>
     </row>
-    <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="14" t="s">
         <v>674</v>
       </c>
@@ -7984,7 +8027,7 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0D00-000000000000}">
   <dimension ref="A1:H26"/>
-  <sheetFormatPr defaultColWidth="8.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
@@ -7996,7 +8039,7 @@
     <col min="8" max="8" width="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" ht="28.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="12" t="s">
         <v>33</v>
       </c>
@@ -8022,7 +8065,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="13" t="s">
         <v>686</v>
       </c>
@@ -8036,7 +8079,7 @@
       <c r="G2" s="13"/>
       <c r="H2" s="13"/>
     </row>
-    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
         <v>686</v>
       </c>
@@ -8060,7 +8103,7 @@
         <v>941</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="19" t="s">
         <v>686</v>
       </c>
@@ -8082,7 +8125,7 @@
       <c r="G4" s="21"/>
       <c r="H4" s="21"/>
     </row>
-    <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
         <v>686</v>
       </c>
@@ -8104,7 +8147,7 @@
       <c r="G5" s="16"/>
       <c r="H5" s="16"/>
     </row>
-    <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="19" t="s">
         <v>686</v>
       </c>
@@ -8126,7 +8169,7 @@
       <c r="G6" s="21"/>
       <c r="H6" s="21"/>
     </row>
-    <row r="7" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="13" t="s">
         <v>696</v>
       </c>
@@ -8140,7 +8183,7 @@
       <c r="G7" s="13"/>
       <c r="H7" s="13"/>
     </row>
-    <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="14" t="s">
         <v>696</v>
       </c>
@@ -8164,7 +8207,7 @@
         <v>942</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="19" t="s">
         <v>696</v>
       </c>
@@ -8188,7 +8231,7 @@
         <v>901</v>
       </c>
     </row>
-    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="14" t="s">
         <v>696</v>
       </c>
@@ -8212,7 +8255,7 @@
         <v>943</v>
       </c>
     </row>
-    <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="19" t="s">
         <v>696</v>
       </c>
@@ -8236,7 +8279,7 @@
         <v>944</v>
       </c>
     </row>
-    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="14" t="s">
         <v>696</v>
       </c>
@@ -8260,7 +8303,7 @@
         <v>945</v>
       </c>
     </row>
-    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="19" t="s">
         <v>696</v>
       </c>
@@ -8282,7 +8325,7 @@
       <c r="G13" s="21"/>
       <c r="H13" s="21"/>
     </row>
-    <row r="14" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="13" t="s">
         <v>710</v>
       </c>
@@ -8296,7 +8339,7 @@
       <c r="G14" s="13"/>
       <c r="H14" s="13"/>
     </row>
-    <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="14" t="s">
         <v>710</v>
       </c>
@@ -8320,7 +8363,7 @@
         <v>946</v>
       </c>
     </row>
-    <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="19" t="s">
         <v>710</v>
       </c>
@@ -8344,7 +8387,7 @@
         <v>947</v>
       </c>
     </row>
-    <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="14" t="s">
         <v>710</v>
       </c>
@@ -8366,7 +8409,7 @@
       <c r="G17" s="16"/>
       <c r="H17" s="16"/>
     </row>
-    <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="19" t="s">
         <v>710</v>
       </c>
@@ -8388,7 +8431,7 @@
       <c r="G18" s="21"/>
       <c r="H18" s="21"/>
     </row>
-    <row r="19" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="13" t="s">
         <v>720</v>
       </c>
@@ -8402,7 +8445,7 @@
       <c r="G19" s="13"/>
       <c r="H19" s="13"/>
     </row>
-    <row r="20" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="14" t="s">
         <v>720</v>
       </c>
@@ -8424,7 +8467,7 @@
       <c r="G20" s="16"/>
       <c r="H20" s="16"/>
     </row>
-    <row r="21" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="19" t="s">
         <v>720</v>
       </c>
@@ -8448,7 +8491,7 @@
         <v>934</v>
       </c>
     </row>
-    <row r="22" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="14" t="s">
         <v>720</v>
       </c>
@@ -8472,7 +8515,7 @@
         <v>948</v>
       </c>
     </row>
-    <row r="23" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="19" t="s">
         <v>720</v>
       </c>
@@ -8496,7 +8539,7 @@
         <v>949</v>
       </c>
     </row>
-    <row r="24" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="14" t="s">
         <v>720</v>
       </c>
@@ -8520,7 +8563,7 @@
         <v>950</v>
       </c>
     </row>
-    <row r="25" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="19" t="s">
         <v>720</v>
       </c>
@@ -8542,7 +8585,7 @@
       <c r="G25" s="21"/>
       <c r="H25" s="21"/>
     </row>
-    <row r="26" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="14" t="s">
         <v>720</v>
       </c>
@@ -8590,7 +8633,7 @@
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0E00-000000000000}">
   <dimension ref="A1:H17"/>
-  <sheetFormatPr defaultColWidth="8.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
@@ -8602,7 +8645,7 @@
     <col min="8" max="8" width="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" ht="28.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="12" t="s">
         <v>33</v>
       </c>
@@ -8628,7 +8671,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="13" t="s">
         <v>736</v>
       </c>
@@ -8642,7 +8685,7 @@
       <c r="G2" s="13"/>
       <c r="H2" s="13"/>
     </row>
-    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
         <v>736</v>
       </c>
@@ -8666,7 +8709,7 @@
         <v>941</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="19" t="s">
         <v>736</v>
       </c>
@@ -8690,7 +8733,7 @@
         <v>951</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="13" t="s">
         <v>742</v>
       </c>
@@ -8704,7 +8747,7 @@
       <c r="G5" s="13"/>
       <c r="H5" s="13"/>
     </row>
-    <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="14" t="s">
         <v>742</v>
       </c>
@@ -8721,12 +8764,14 @@
         <v>1</v>
       </c>
       <c r="F6" s="18" t="s">
-        <v>983</v>
-      </c>
-      <c r="G6" s="16"/>
+        <v>984</v>
+      </c>
+      <c r="G6" s="16" t="s">
+        <v>995</v>
+      </c>
       <c r="H6" s="16"/>
     </row>
-    <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="19" t="s">
         <v>742</v>
       </c>
@@ -8750,7 +8795,7 @@
         <v>952</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="14" t="s">
         <v>742</v>
       </c>
@@ -8774,7 +8819,7 @@
         <v>953</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="19" t="s">
         <v>742</v>
       </c>
@@ -8798,7 +8843,7 @@
         <v>954</v>
       </c>
     </row>
-    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="14" t="s">
         <v>742</v>
       </c>
@@ -8820,7 +8865,7 @@
       <c r="G10" s="16"/>
       <c r="H10" s="16"/>
     </row>
-    <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="19" t="s">
         <v>742</v>
       </c>
@@ -8842,7 +8887,7 @@
       <c r="G11" s="21"/>
       <c r="H11" s="21"/>
     </row>
-    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="14" t="s">
         <v>742</v>
       </c>
@@ -8864,7 +8909,7 @@
       <c r="G12" s="16"/>
       <c r="H12" s="16"/>
     </row>
-    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="19" t="s">
         <v>742</v>
       </c>
@@ -8886,7 +8931,7 @@
       <c r="G13" s="21"/>
       <c r="H13" s="21"/>
     </row>
-    <row r="14" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="13" t="s">
         <v>760</v>
       </c>
@@ -8900,7 +8945,7 @@
       <c r="G14" s="13"/>
       <c r="H14" s="13"/>
     </row>
-    <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="14" t="s">
         <v>760</v>
       </c>
@@ -8922,7 +8967,7 @@
       <c r="G15" s="16"/>
       <c r="H15" s="16"/>
     </row>
-    <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="19" t="s">
         <v>760</v>
       </c>
@@ -8946,7 +8991,7 @@
         <v>955</v>
       </c>
     </row>
-    <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="14" t="s">
         <v>760</v>
       </c>
@@ -8996,7 +9041,7 @@
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0F00-000000000000}">
   <dimension ref="A1:H26"/>
-  <sheetFormatPr defaultColWidth="8.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
@@ -9008,7 +9053,7 @@
     <col min="8" max="8" width="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" ht="28.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="12" t="s">
         <v>33</v>
       </c>
@@ -9034,7 +9079,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="13" t="s">
         <v>768</v>
       </c>
@@ -9048,7 +9093,7 @@
       <c r="G2" s="13"/>
       <c r="H2" s="13"/>
     </row>
-    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
         <v>768</v>
       </c>
@@ -9070,7 +9115,7 @@
       <c r="G3" s="16"/>
       <c r="H3" s="16"/>
     </row>
-    <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="19" t="s">
         <v>768</v>
       </c>
@@ -9094,7 +9139,7 @@
         <v>957</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
         <v>768</v>
       </c>
@@ -9118,7 +9163,7 @@
         <v>958</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="19" t="s">
         <v>768</v>
       </c>
@@ -9140,7 +9185,7 @@
       <c r="G6" s="21"/>
       <c r="H6" s="21"/>
     </row>
-    <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="14" t="s">
         <v>768</v>
       </c>
@@ -9162,7 +9207,7 @@
       <c r="G7" s="16"/>
       <c r="H7" s="16"/>
     </row>
-    <row r="8" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="13" t="s">
         <v>780</v>
       </c>
@@ -9176,7 +9221,7 @@
       <c r="G8" s="13"/>
       <c r="H8" s="13"/>
     </row>
-    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="14" t="s">
         <v>780</v>
       </c>
@@ -9198,7 +9243,7 @@
       <c r="G9" s="16"/>
       <c r="H9" s="16"/>
     </row>
-    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="19" t="s">
         <v>780</v>
       </c>
@@ -9215,14 +9260,16 @@
         <v>2</v>
       </c>
       <c r="F10" s="18" t="s">
-        <v>983</v>
-      </c>
-      <c r="G10" s="21"/>
+        <v>984</v>
+      </c>
+      <c r="G10" s="21" t="s">
+        <v>989</v>
+      </c>
       <c r="H10" s="21" t="s">
         <v>959</v>
       </c>
     </row>
-    <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="14" t="s">
         <v>780</v>
       </c>
@@ -9246,7 +9293,7 @@
         <v>960</v>
       </c>
     </row>
-    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="19" t="s">
         <v>780</v>
       </c>
@@ -9265,10 +9312,10 @@
       <c r="F12" s="18" t="s">
         <v>45</v>
       </c>
-      <c r="G12" s="21"/>
+      <c r="G12" s="29"/>
       <c r="H12" s="21"/>
     </row>
-    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="14" t="s">
         <v>780</v>
       </c>
@@ -9290,7 +9337,7 @@
       <c r="G13" s="16"/>
       <c r="H13" s="16"/>
     </row>
-    <row r="14" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="13" t="s">
         <v>792</v>
       </c>
@@ -9304,7 +9351,7 @@
       <c r="G14" s="13"/>
       <c r="H14" s="13"/>
     </row>
-    <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="14" t="s">
         <v>792</v>
       </c>
@@ -9326,7 +9373,7 @@
       <c r="G15" s="16"/>
       <c r="H15" s="16"/>
     </row>
-    <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="19" t="s">
         <v>792</v>
       </c>
@@ -9350,7 +9397,7 @@
         <v>961</v>
       </c>
     </row>
-    <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="14" t="s">
         <v>792</v>
       </c>
@@ -9374,7 +9421,7 @@
         <v>962</v>
       </c>
     </row>
-    <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="19" t="s">
         <v>792</v>
       </c>
@@ -9398,7 +9445,7 @@
         <v>963</v>
       </c>
     </row>
-    <row r="19" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="14" t="s">
         <v>792</v>
       </c>
@@ -9422,7 +9469,7 @@
         <v>964</v>
       </c>
     </row>
-    <row r="20" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="19" t="s">
         <v>792</v>
       </c>
@@ -9446,7 +9493,7 @@
         <v>964</v>
       </c>
     </row>
-    <row r="21" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="14" t="s">
         <v>792</v>
       </c>
@@ -9470,7 +9517,7 @@
         <v>965</v>
       </c>
     </row>
-    <row r="22" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="13" t="s">
         <v>808</v>
       </c>
@@ -9484,7 +9531,7 @@
       <c r="G22" s="13"/>
       <c r="H22" s="13"/>
     </row>
-    <row r="23" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="14" t="s">
         <v>808</v>
       </c>
@@ -9506,7 +9553,7 @@
       <c r="G23" s="16"/>
       <c r="H23" s="16"/>
     </row>
-    <row r="24" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="19" t="s">
         <v>808</v>
       </c>
@@ -9528,7 +9575,7 @@
       <c r="G24" s="21"/>
       <c r="H24" s="21"/>
     </row>
-    <row r="25" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="14" t="s">
         <v>808</v>
       </c>
@@ -9550,7 +9597,7 @@
       <c r="G25" s="16"/>
       <c r="H25" s="16"/>
     </row>
-    <row r="26" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="19" t="s">
         <v>808</v>
       </c>
@@ -9597,8 +9644,8 @@
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1000-000000000000}">
-  <dimension ref="A1:H23"/>
-  <sheetFormatPr defaultColWidth="8.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:H26"/>
+  <sheetFormatPr defaultColWidth="8.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
@@ -9610,7 +9657,7 @@
     <col min="8" max="8" width="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" ht="28.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="12" t="s">
         <v>33</v>
       </c>
@@ -9636,7 +9683,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="13" t="s">
         <v>818</v>
       </c>
@@ -9650,7 +9697,7 @@
       <c r="G2" s="13"/>
       <c r="H2" s="13"/>
     </row>
-    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
         <v>818</v>
       </c>
@@ -9674,7 +9721,7 @@
         <v>966</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="13" t="s">
         <v>822</v>
       </c>
@@ -9688,7 +9735,7 @@
       <c r="G4" s="13"/>
       <c r="H4" s="13"/>
     </row>
-    <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
         <v>822</v>
       </c>
@@ -9712,7 +9759,7 @@
         <v>967</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="19" t="s">
         <v>822</v>
       </c>
@@ -9736,7 +9783,7 @@
         <v>968</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="14" t="s">
         <v>822</v>
       </c>
@@ -9760,7 +9807,7 @@
         <v>969</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="19" t="s">
         <v>822</v>
       </c>
@@ -9784,7 +9831,7 @@
         <v>967</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="14" t="s">
         <v>822</v>
       </c>
@@ -9808,7 +9855,7 @@
         <v>970</v>
       </c>
     </row>
-    <row r="10" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="13" t="s">
         <v>834</v>
       </c>
@@ -9822,7 +9869,7 @@
       <c r="G10" s="13"/>
       <c r="H10" s="13"/>
     </row>
-    <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="14" t="s">
         <v>834</v>
       </c>
@@ -9846,7 +9893,7 @@
         <v>971</v>
       </c>
     </row>
-    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="19" t="s">
         <v>834</v>
       </c>
@@ -9870,7 +9917,7 @@
         <v>972</v>
       </c>
     </row>
-    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="14" t="s">
         <v>834</v>
       </c>
@@ -9894,7 +9941,7 @@
         <v>973</v>
       </c>
     </row>
-    <row r="14" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="19" t="s">
         <v>834</v>
       </c>
@@ -9918,7 +9965,7 @@
         <v>974</v>
       </c>
     </row>
-    <row r="15" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="13" t="s">
         <v>844</v>
       </c>
@@ -9932,7 +9979,7 @@
       <c r="G15" s="13"/>
       <c r="H15" s="13"/>
     </row>
-    <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="14" t="s">
         <v>844</v>
       </c>
@@ -9956,7 +10003,7 @@
         <v>964</v>
       </c>
     </row>
-    <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="19" t="s">
         <v>844</v>
       </c>
@@ -9980,7 +10027,7 @@
         <v>975</v>
       </c>
     </row>
-    <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="14" t="s">
         <v>844</v>
       </c>
@@ -10004,7 +10051,7 @@
         <v>974</v>
       </c>
     </row>
-    <row r="19" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="13" t="s">
         <v>852</v>
       </c>
@@ -10018,7 +10065,7 @@
       <c r="G19" s="13"/>
       <c r="H19" s="13"/>
     </row>
-    <row r="20" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="14" t="s">
         <v>852</v>
       </c>
@@ -10035,14 +10082,16 @@
         <v>2</v>
       </c>
       <c r="F20" s="18" t="s">
-        <v>983</v>
-      </c>
-      <c r="G20" s="16"/>
+        <v>984</v>
+      </c>
+      <c r="G20" s="16" t="s">
+        <v>985</v>
+      </c>
       <c r="H20" s="16" t="s">
         <v>976</v>
       </c>
     </row>
-    <row r="21" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="19" t="s">
         <v>852</v>
       </c>
@@ -10059,14 +10108,16 @@
         <v>2</v>
       </c>
       <c r="F21" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G21" s="21"/>
+        <v>984</v>
+      </c>
+      <c r="G21" s="16" t="s">
+        <v>986</v>
+      </c>
       <c r="H21" s="21" t="s">
         <v>958</v>
       </c>
     </row>
-    <row r="22" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="14" t="s">
         <v>852</v>
       </c>
@@ -10083,14 +10134,16 @@
         <v>2</v>
       </c>
       <c r="F22" s="18" t="s">
-        <v>983</v>
-      </c>
-      <c r="G22" s="16"/>
+        <v>984</v>
+      </c>
+      <c r="G22" s="16" t="s">
+        <v>987</v>
+      </c>
       <c r="H22" s="16" t="s">
         <v>977</v>
       </c>
     </row>
-    <row r="23" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="19" t="s">
         <v>852</v>
       </c>
@@ -10107,10 +10160,18 @@
         <v>3</v>
       </c>
       <c r="F23" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G23" s="21"/>
+        <v>984</v>
+      </c>
+      <c r="G23" s="16" t="s">
+        <v>988</v>
+      </c>
       <c r="H23" s="21"/>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G25" s="28"/>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G26" s="28"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="F2:F23">
@@ -10131,14 +10192,14 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.51180555555555496" footer="0.51180555555555496"/>
-  <pageSetup firstPageNumber="0" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <pageSetup firstPageNumber="0" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1100-000000000000}">
   <dimension ref="A1:H16"/>
-  <sheetFormatPr defaultColWidth="8.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
@@ -10150,7 +10211,7 @@
     <col min="8" max="8" width="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" ht="28.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="12" t="s">
         <v>33</v>
       </c>
@@ -10176,7 +10237,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="13" t="s">
         <v>862</v>
       </c>
@@ -10190,7 +10251,7 @@
       <c r="G2" s="13"/>
       <c r="H2" s="13"/>
     </row>
-    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
         <v>862</v>
       </c>
@@ -10214,7 +10275,7 @@
         <v>978</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="19" t="s">
         <v>862</v>
       </c>
@@ -10236,7 +10297,7 @@
       <c r="G4" s="21"/>
       <c r="H4" s="21"/>
     </row>
-    <row r="5" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="13" t="s">
         <v>868</v>
       </c>
@@ -10250,7 +10311,7 @@
       <c r="G5" s="13"/>
       <c r="H5" s="13"/>
     </row>
-    <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="14" t="s">
         <v>868</v>
       </c>
@@ -10274,7 +10335,7 @@
         <v>979</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="19" t="s">
         <v>868</v>
       </c>
@@ -10298,7 +10359,7 @@
         <v>980</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="14" t="s">
         <v>868</v>
       </c>
@@ -10322,7 +10383,7 @@
         <v>981</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="19" t="s">
         <v>868</v>
       </c>
@@ -10346,7 +10407,7 @@
         <v>973</v>
       </c>
     </row>
-    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="14" t="s">
         <v>868</v>
       </c>
@@ -10368,7 +10429,7 @@
       <c r="G10" s="16"/>
       <c r="H10" s="16"/>
     </row>
-    <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="19" t="s">
         <v>868</v>
       </c>
@@ -10390,7 +10451,7 @@
       <c r="G11" s="21"/>
       <c r="H11" s="21"/>
     </row>
-    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="14" t="s">
         <v>868</v>
       </c>
@@ -10412,7 +10473,7 @@
       <c r="G12" s="16"/>
       <c r="H12" s="16"/>
     </row>
-    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="19" t="s">
         <v>868</v>
       </c>
@@ -10434,7 +10495,7 @@
       <c r="G13" s="21"/>
       <c r="H13" s="21"/>
     </row>
-    <row r="14" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="13" t="s">
         <v>886</v>
       </c>
@@ -10448,7 +10509,7 @@
       <c r="G14" s="13"/>
       <c r="H14" s="13"/>
     </row>
-    <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="14" t="s">
         <v>886</v>
       </c>
@@ -10472,7 +10533,7 @@
         <v>958</v>
       </c>
     </row>
-    <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="19" t="s">
         <v>886</v>
       </c>
@@ -10522,7 +10583,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:H36"/>
-  <sheetFormatPr defaultColWidth="8.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
@@ -10534,7 +10595,7 @@
     <col min="8" max="8" width="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" ht="28.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="12" t="s">
         <v>33</v>
       </c>
@@ -10560,7 +10621,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="13" t="s">
         <v>41</v>
       </c>
@@ -10574,7 +10635,7 @@
       <c r="G2" s="13"/>
       <c r="H2" s="13"/>
     </row>
-    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
         <v>41</v>
       </c>
@@ -10596,7 +10657,7 @@
       <c r="G3" s="16"/>
       <c r="H3" s="16"/>
     </row>
-    <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="19" t="s">
         <v>41</v>
       </c>
@@ -10618,7 +10679,7 @@
       <c r="G4" s="21"/>
       <c r="H4" s="21"/>
     </row>
-    <row r="5" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="13" t="s">
         <v>48</v>
       </c>
@@ -10632,7 +10693,7 @@
       <c r="G5" s="13"/>
       <c r="H5" s="13"/>
     </row>
-    <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="14" t="s">
         <v>48</v>
       </c>
@@ -10654,7 +10715,7 @@
       <c r="G6" s="16"/>
       <c r="H6" s="16"/>
     </row>
-    <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="19" t="s">
         <v>48</v>
       </c>
@@ -10676,7 +10737,7 @@
       <c r="G7" s="21"/>
       <c r="H7" s="21"/>
     </row>
-    <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="14" t="s">
         <v>48</v>
       </c>
@@ -10698,7 +10759,7 @@
       <c r="G8" s="16"/>
       <c r="H8" s="16"/>
     </row>
-    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="19" t="s">
         <v>48</v>
       </c>
@@ -10720,7 +10781,7 @@
       <c r="G9" s="21"/>
       <c r="H9" s="21"/>
     </row>
-    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="14" t="s">
         <v>48</v>
       </c>
@@ -10742,7 +10803,7 @@
       <c r="G10" s="16"/>
       <c r="H10" s="16"/>
     </row>
-    <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="19" t="s">
         <v>48</v>
       </c>
@@ -10766,7 +10827,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="14" t="s">
         <v>48</v>
       </c>
@@ -10790,7 +10851,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="19" t="s">
         <v>48</v>
       </c>
@@ -10814,7 +10875,7 @@
         <v>895</v>
       </c>
     </row>
-    <row r="14" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="14" t="s">
         <v>48</v>
       </c>
@@ -10836,7 +10897,7 @@
       <c r="G14" s="16"/>
       <c r="H14" s="16"/>
     </row>
-    <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="19" t="s">
         <v>48</v>
       </c>
@@ -10858,7 +10919,7 @@
       <c r="G15" s="21"/>
       <c r="H15" s="21"/>
     </row>
-    <row r="16" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="13" t="s">
         <v>70</v>
       </c>
@@ -10872,7 +10933,7 @@
       <c r="G16" s="13"/>
       <c r="H16" s="13"/>
     </row>
-    <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="14" t="s">
         <v>70</v>
       </c>
@@ -10894,7 +10955,7 @@
       <c r="G17" s="16"/>
       <c r="H17" s="16"/>
     </row>
-    <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="19" t="s">
         <v>70</v>
       </c>
@@ -10916,7 +10977,7 @@
       <c r="G18" s="21"/>
       <c r="H18" s="21"/>
     </row>
-    <row r="19" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="14" t="s">
         <v>70</v>
       </c>
@@ -10940,7 +11001,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="20" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="19" t="s">
         <v>70</v>
       </c>
@@ -10964,7 +11025,7 @@
         <v>895</v>
       </c>
     </row>
-    <row r="21" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="14" t="s">
         <v>70</v>
       </c>
@@ -10988,7 +11049,7 @@
         <v>896</v>
       </c>
     </row>
-    <row r="22" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="19" t="s">
         <v>70</v>
       </c>
@@ -11012,7 +11073,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="23" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="14" t="s">
         <v>70</v>
       </c>
@@ -11036,7 +11097,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="24" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="19" t="s">
         <v>70</v>
       </c>
@@ -11060,7 +11121,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="25" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="14" t="s">
         <v>70</v>
       </c>
@@ -11084,7 +11145,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="26" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="19" t="s">
         <v>70</v>
       </c>
@@ -11108,7 +11169,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="27" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="14" t="s">
         <v>70</v>
       </c>
@@ -11132,7 +11193,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="28" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="19" t="s">
         <v>70</v>
       </c>
@@ -11154,7 +11215,7 @@
       <c r="G28" s="21"/>
       <c r="H28" s="21"/>
     </row>
-    <row r="29" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="13" t="s">
         <v>96</v>
       </c>
@@ -11168,7 +11229,7 @@
       <c r="G29" s="13"/>
       <c r="H29" s="13"/>
     </row>
-    <row r="30" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="14" t="s">
         <v>96</v>
       </c>
@@ -11192,7 +11253,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="31" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="19" t="s">
         <v>96</v>
       </c>
@@ -11216,7 +11277,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="32" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="14" t="s">
         <v>96</v>
       </c>
@@ -11240,7 +11301,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="33" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="13" t="s">
         <v>104</v>
       </c>
@@ -11254,7 +11315,7 @@
       <c r="G33" s="13"/>
       <c r="H33" s="13"/>
     </row>
-    <row r="34" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="14" t="s">
         <v>104</v>
       </c>
@@ -11276,7 +11337,7 @@
       <c r="G34" s="16"/>
       <c r="H34" s="16"/>
     </row>
-    <row r="35" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="19" t="s">
         <v>104</v>
       </c>
@@ -11300,7 +11361,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="36" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="14" t="s">
         <v>104</v>
       </c>
@@ -11348,7 +11409,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:H18"/>
-  <sheetFormatPr defaultColWidth="8.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
@@ -11360,7 +11421,7 @@
     <col min="8" max="8" width="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" ht="28.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="12" t="s">
         <v>33</v>
       </c>
@@ -11386,7 +11447,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="13" t="s">
         <v>112</v>
       </c>
@@ -11400,7 +11461,7 @@
       <c r="G2" s="13"/>
       <c r="H2" s="13"/>
     </row>
-    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
         <v>112</v>
       </c>
@@ -11422,7 +11483,7 @@
       <c r="G3" s="16"/>
       <c r="H3" s="16"/>
     </row>
-    <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="19" t="s">
         <v>112</v>
       </c>
@@ -11446,7 +11507,7 @@
         <v>897</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
         <v>112</v>
       </c>
@@ -11470,7 +11531,7 @@
         <v>898</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="13" t="s">
         <v>120</v>
       </c>
@@ -11484,7 +11545,7 @@
       <c r="G6" s="13"/>
       <c r="H6" s="13"/>
     </row>
-    <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="14" t="s">
         <v>120</v>
       </c>
@@ -11506,7 +11567,7 @@
       <c r="G7" s="16"/>
       <c r="H7" s="16"/>
     </row>
-    <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="19" t="s">
         <v>120</v>
       </c>
@@ -11528,7 +11589,7 @@
       <c r="G8" s="21"/>
       <c r="H8" s="21"/>
     </row>
-    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="14" t="s">
         <v>120</v>
       </c>
@@ -11552,7 +11613,7 @@
         <v>897</v>
       </c>
     </row>
-    <row r="10" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="13" t="s">
         <v>128</v>
       </c>
@@ -11566,7 +11627,7 @@
       <c r="G10" s="13"/>
       <c r="H10" s="13"/>
     </row>
-    <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="14" t="s">
         <v>128</v>
       </c>
@@ -11588,7 +11649,7 @@
       <c r="G11" s="16"/>
       <c r="H11" s="16"/>
     </row>
-    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="19" t="s">
         <v>128</v>
       </c>
@@ -11612,7 +11673,7 @@
         <v>899</v>
       </c>
     </row>
-    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="14" t="s">
         <v>128</v>
       </c>
@@ -11636,7 +11697,7 @@
         <v>900</v>
       </c>
     </row>
-    <row r="14" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="19" t="s">
         <v>128</v>
       </c>
@@ -11660,7 +11721,7 @@
         <v>901</v>
       </c>
     </row>
-    <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="14" t="s">
         <v>128</v>
       </c>
@@ -11682,7 +11743,7 @@
       <c r="G15" s="16"/>
       <c r="H15" s="16"/>
     </row>
-    <row r="16" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="13" t="s">
         <v>140</v>
       </c>
@@ -11696,7 +11757,7 @@
       <c r="G16" s="13"/>
       <c r="H16" s="13"/>
     </row>
-    <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="14" t="s">
         <v>140</v>
       </c>
@@ -11720,7 +11781,7 @@
         <v>902</v>
       </c>
     </row>
-    <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="19" t="s">
         <v>140</v>
       </c>
@@ -11768,7 +11829,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:H39"/>
-  <sheetFormatPr defaultColWidth="8.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
@@ -11780,7 +11841,7 @@
     <col min="8" max="8" width="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" ht="28.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="12" t="s">
         <v>33</v>
       </c>
@@ -11806,7 +11867,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="13" t="s">
         <v>146</v>
       </c>
@@ -11820,7 +11881,7 @@
       <c r="G2" s="13"/>
       <c r="H2" s="13"/>
     </row>
-    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
         <v>146</v>
       </c>
@@ -11842,7 +11903,7 @@
       <c r="G3" s="16"/>
       <c r="H3" s="16"/>
     </row>
-    <row r="4" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="13" t="s">
         <v>150</v>
       </c>
@@ -11856,7 +11917,7 @@
       <c r="G4" s="13"/>
       <c r="H4" s="13"/>
     </row>
-    <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
         <v>150</v>
       </c>
@@ -11878,7 +11939,7 @@
       <c r="G5" s="16"/>
       <c r="H5" s="16"/>
     </row>
-    <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="19" t="s">
         <v>150</v>
       </c>
@@ -11900,7 +11961,7 @@
       <c r="G6" s="21"/>
       <c r="H6" s="21"/>
     </row>
-    <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="14" t="s">
         <v>150</v>
       </c>
@@ -11922,7 +11983,7 @@
       <c r="G7" s="16"/>
       <c r="H7" s="16"/>
     </row>
-    <row r="8" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="13" t="s">
         <v>158</v>
       </c>
@@ -11936,7 +11997,7 @@
       <c r="G8" s="13"/>
       <c r="H8" s="13"/>
     </row>
-    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="14" t="s">
         <v>158</v>
       </c>
@@ -11958,7 +12019,7 @@
       <c r="G9" s="16"/>
       <c r="H9" s="16"/>
     </row>
-    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="19" t="s">
         <v>158</v>
       </c>
@@ -11982,7 +12043,7 @@
         <v>896</v>
       </c>
     </row>
-    <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="14" t="s">
         <v>158</v>
       </c>
@@ -12006,7 +12067,7 @@
         <v>903</v>
       </c>
     </row>
-    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="19" t="s">
         <v>158</v>
       </c>
@@ -12030,7 +12091,7 @@
         <v>904</v>
       </c>
     </row>
-    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="14" t="s">
         <v>158</v>
       </c>
@@ -12052,7 +12113,7 @@
       <c r="G13" s="16"/>
       <c r="H13" s="16"/>
     </row>
-    <row r="14" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="13" t="s">
         <v>170</v>
       </c>
@@ -12066,7 +12127,7 @@
       <c r="G14" s="13"/>
       <c r="H14" s="13"/>
     </row>
-    <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="14" t="s">
         <v>170</v>
       </c>
@@ -12088,7 +12149,7 @@
       <c r="G15" s="16"/>
       <c r="H15" s="16"/>
     </row>
-    <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="19" t="s">
         <v>170</v>
       </c>
@@ -12110,7 +12171,7 @@
       <c r="G16" s="21"/>
       <c r="H16" s="21"/>
     </row>
-    <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="14" t="s">
         <v>170</v>
       </c>
@@ -12134,7 +12195,7 @@
         <v>905</v>
       </c>
     </row>
-    <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="19" t="s">
         <v>170</v>
       </c>
@@ -12158,7 +12219,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="19" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="14" t="s">
         <v>170</v>
       </c>
@@ -12182,7 +12243,7 @@
         <v>897</v>
       </c>
     </row>
-    <row r="20" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="19" t="s">
         <v>170</v>
       </c>
@@ -12206,7 +12267,7 @@
         <v>906</v>
       </c>
     </row>
-    <row r="21" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="14" t="s">
         <v>170</v>
       </c>
@@ -12228,7 +12289,7 @@
       <c r="G21" s="16"/>
       <c r="H21" s="16"/>
     </row>
-    <row r="22" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="19" t="s">
         <v>170</v>
       </c>
@@ -12250,7 +12311,7 @@
       <c r="G22" s="21"/>
       <c r="H22" s="21"/>
     </row>
-    <row r="23" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="13" t="s">
         <v>188</v>
       </c>
@@ -12264,7 +12325,7 @@
       <c r="G23" s="13"/>
       <c r="H23" s="13"/>
     </row>
-    <row r="24" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="14" t="s">
         <v>188</v>
       </c>
@@ -12286,7 +12347,7 @@
       <c r="G24" s="16"/>
       <c r="H24" s="16"/>
     </row>
-    <row r="25" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="19" t="s">
         <v>188</v>
       </c>
@@ -12308,7 +12369,7 @@
       <c r="G25" s="21"/>
       <c r="H25" s="21"/>
     </row>
-    <row r="26" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="14" t="s">
         <v>188</v>
       </c>
@@ -12330,7 +12391,7 @@
       <c r="G26" s="16"/>
       <c r="H26" s="16"/>
     </row>
-    <row r="27" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="19" t="s">
         <v>188</v>
       </c>
@@ -12354,7 +12415,7 @@
         <v>903</v>
       </c>
     </row>
-    <row r="28" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="14" t="s">
         <v>188</v>
       </c>
@@ -12378,7 +12439,7 @@
         <v>897</v>
       </c>
     </row>
-    <row r="29" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="19" t="s">
         <v>188</v>
       </c>
@@ -12400,7 +12461,7 @@
       <c r="G29" s="21"/>
       <c r="H29" s="21"/>
     </row>
-    <row r="30" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="14" t="s">
         <v>188</v>
       </c>
@@ -12422,7 +12483,7 @@
       <c r="G30" s="16"/>
       <c r="H30" s="16"/>
     </row>
-    <row r="31" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="19" t="s">
         <v>188</v>
       </c>
@@ -12444,7 +12505,7 @@
       <c r="G31" s="21"/>
       <c r="H31" s="21"/>
     </row>
-    <row r="32" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="13" t="s">
         <v>206</v>
       </c>
@@ -12458,7 +12519,7 @@
       <c r="G32" s="13"/>
       <c r="H32" s="13"/>
     </row>
-    <row r="33" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="14" t="s">
         <v>206</v>
       </c>
@@ -12480,7 +12541,7 @@
       <c r="G33" s="16"/>
       <c r="H33" s="16"/>
     </row>
-    <row r="34" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="13" t="s">
         <v>210</v>
       </c>
@@ -12494,7 +12555,7 @@
       <c r="G34" s="13"/>
       <c r="H34" s="13"/>
     </row>
-    <row r="35" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="14" t="s">
         <v>210</v>
       </c>
@@ -12518,7 +12579,7 @@
         <v>895</v>
       </c>
     </row>
-    <row r="36" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="19" t="s">
         <v>210</v>
       </c>
@@ -12542,7 +12603,7 @@
         <v>907</v>
       </c>
     </row>
-    <row r="37" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="14" t="s">
         <v>210</v>
       </c>
@@ -12564,7 +12625,7 @@
       <c r="G37" s="16"/>
       <c r="H37" s="16"/>
     </row>
-    <row r="38" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="19" t="s">
         <v>210</v>
       </c>
@@ -12586,7 +12647,7 @@
       <c r="G38" s="21"/>
       <c r="H38" s="21"/>
     </row>
-    <row r="39" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="14" t="s">
         <v>210</v>
       </c>
@@ -12634,7 +12695,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:H21"/>
-  <sheetFormatPr defaultColWidth="8.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
@@ -12646,7 +12707,7 @@
     <col min="8" max="8" width="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" ht="28.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="12" t="s">
         <v>33</v>
       </c>
@@ -12672,7 +12733,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="13" t="s">
         <v>222</v>
       </c>
@@ -12686,7 +12747,7 @@
       <c r="G2" s="13"/>
       <c r="H2" s="13"/>
     </row>
-    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
         <v>222</v>
       </c>
@@ -12708,7 +12769,7 @@
       <c r="G3" s="16"/>
       <c r="H3" s="16"/>
     </row>
-    <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="19" t="s">
         <v>222</v>
       </c>
@@ -12732,7 +12793,7 @@
         <v>908</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
         <v>222</v>
       </c>
@@ -12756,7 +12817,7 @@
         <v>897</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="19" t="s">
         <v>222</v>
       </c>
@@ -12778,7 +12839,7 @@
       <c r="G6" s="21"/>
       <c r="H6" s="21"/>
     </row>
-    <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="14" t="s">
         <v>222</v>
       </c>
@@ -12800,7 +12861,7 @@
       <c r="G7" s="16"/>
       <c r="H7" s="16"/>
     </row>
-    <row r="8" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="13" t="s">
         <v>234</v>
       </c>
@@ -12814,7 +12875,7 @@
       <c r="G8" s="13"/>
       <c r="H8" s="13"/>
     </row>
-    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="14" t="s">
         <v>234</v>
       </c>
@@ -12838,7 +12899,7 @@
         <v>909</v>
       </c>
     </row>
-    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="19" t="s">
         <v>234</v>
       </c>
@@ -12860,7 +12921,7 @@
       <c r="G10" s="21"/>
       <c r="H10" s="21"/>
     </row>
-    <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="14" t="s">
         <v>234</v>
       </c>
@@ -12882,7 +12943,7 @@
       <c r="G11" s="16"/>
       <c r="H11" s="16"/>
     </row>
-    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="19" t="s">
         <v>234</v>
       </c>
@@ -12904,7 +12965,7 @@
       <c r="G12" s="21"/>
       <c r="H12" s="21"/>
     </row>
-    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="14" t="s">
         <v>234</v>
       </c>
@@ -12926,7 +12987,7 @@
       <c r="G13" s="16"/>
       <c r="H13" s="16"/>
     </row>
-    <row r="14" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="13" t="s">
         <v>246</v>
       </c>
@@ -12940,7 +13001,7 @@
       <c r="G14" s="13"/>
       <c r="H14" s="13"/>
     </row>
-    <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="14" t="s">
         <v>246</v>
       </c>
@@ -12964,7 +13025,7 @@
         <v>902</v>
       </c>
     </row>
-    <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="19" t="s">
         <v>246</v>
       </c>
@@ -12988,7 +13049,7 @@
         <v>903</v>
       </c>
     </row>
-    <row r="17" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="13" t="s">
         <v>252</v>
       </c>
@@ -13002,7 +13063,7 @@
       <c r="G17" s="13"/>
       <c r="H17" s="13"/>
     </row>
-    <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="14" t="s">
         <v>252</v>
       </c>
@@ -13024,7 +13085,7 @@
       <c r="G18" s="16"/>
       <c r="H18" s="16"/>
     </row>
-    <row r="19" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="19" t="s">
         <v>252</v>
       </c>
@@ -13048,7 +13109,7 @@
         <v>897</v>
       </c>
     </row>
-    <row r="20" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="14" t="s">
         <v>252</v>
       </c>
@@ -13072,7 +13133,7 @@
         <v>910</v>
       </c>
     </row>
-    <row r="21" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="19" t="s">
         <v>252</v>
       </c>
@@ -13122,7 +13183,7 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:H18"/>
-  <sheetFormatPr defaultColWidth="8.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
@@ -13134,7 +13195,7 @@
     <col min="8" max="8" width="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" ht="28.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="12" t="s">
         <v>33</v>
       </c>
@@ -13160,7 +13221,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="13" t="s">
         <v>262</v>
       </c>
@@ -13174,7 +13235,7 @@
       <c r="G2" s="13"/>
       <c r="H2" s="13"/>
     </row>
-    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
         <v>262</v>
       </c>
@@ -13198,7 +13259,7 @@
         <v>912</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="13" t="s">
         <v>266</v>
       </c>
@@ -13212,7 +13273,7 @@
       <c r="G4" s="13"/>
       <c r="H4" s="13"/>
     </row>
-    <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
         <v>266</v>
       </c>
@@ -13229,12 +13290,14 @@
         <v>1</v>
       </c>
       <c r="F5" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G5" s="16"/>
+        <v>984</v>
+      </c>
+      <c r="G5" s="16" t="s">
+        <v>990</v>
+      </c>
       <c r="H5" s="16"/>
     </row>
-    <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="19" t="s">
         <v>266</v>
       </c>
@@ -13251,12 +13314,14 @@
         <v>1</v>
       </c>
       <c r="F6" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G6" s="21"/>
+        <v>984</v>
+      </c>
+      <c r="G6" s="21" t="s">
+        <v>991</v>
+      </c>
       <c r="H6" s="21"/>
     </row>
-    <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="14" t="s">
         <v>266</v>
       </c>
@@ -13280,7 +13345,7 @@
         <v>913</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="19" t="s">
         <v>266</v>
       </c>
@@ -13302,7 +13367,7 @@
       <c r="G8" s="21"/>
       <c r="H8" s="21"/>
     </row>
-    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="14" t="s">
         <v>266</v>
       </c>
@@ -13324,7 +13389,7 @@
       <c r="G9" s="16"/>
       <c r="H9" s="16"/>
     </row>
-    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="19" t="s">
         <v>266</v>
       </c>
@@ -13346,7 +13411,7 @@
       <c r="G10" s="21"/>
       <c r="H10" s="21"/>
     </row>
-    <row r="11" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="13" t="s">
         <v>280</v>
       </c>
@@ -13360,7 +13425,7 @@
       <c r="G11" s="13"/>
       <c r="H11" s="13"/>
     </row>
-    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="14" t="s">
         <v>280</v>
       </c>
@@ -13379,10 +13444,12 @@
       <c r="F12" s="18" t="s">
         <v>984</v>
       </c>
-      <c r="G12" s="16"/>
+      <c r="G12" s="16" t="s">
+        <v>993</v>
+      </c>
       <c r="H12" s="16"/>
     </row>
-    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="19" t="s">
         <v>280</v>
       </c>
@@ -13399,12 +13466,14 @@
         <v>1</v>
       </c>
       <c r="F13" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G13" s="21"/>
+        <v>984</v>
+      </c>
+      <c r="G13" s="21" t="s">
+        <v>992</v>
+      </c>
       <c r="H13" s="21"/>
     </row>
-    <row r="14" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="14" t="s">
         <v>280</v>
       </c>
@@ -13426,7 +13495,7 @@
       <c r="G14" s="16"/>
       <c r="H14" s="16"/>
     </row>
-    <row r="15" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="13" t="s">
         <v>288</v>
       </c>
@@ -13440,7 +13509,7 @@
       <c r="G15" s="13"/>
       <c r="H15" s="13"/>
     </row>
-    <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="14" t="s">
         <v>288</v>
       </c>
@@ -13464,7 +13533,7 @@
         <v>914</v>
       </c>
     </row>
-    <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="19" t="s">
         <v>288</v>
       </c>
@@ -13488,7 +13557,7 @@
         <v>896</v>
       </c>
     </row>
-    <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="14" t="s">
         <v>288</v>
       </c>
@@ -13538,7 +13607,7 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:H56"/>
-  <sheetFormatPr defaultColWidth="8.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
@@ -13550,7 +13619,7 @@
     <col min="8" max="8" width="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" ht="28.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="12" t="s">
         <v>33</v>
       </c>
@@ -13576,7 +13645,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="13" t="s">
         <v>296</v>
       </c>
@@ -13590,7 +13659,7 @@
       <c r="G2" s="13"/>
       <c r="H2" s="13"/>
     </row>
-    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
         <v>296</v>
       </c>
@@ -13612,7 +13681,7 @@
       <c r="G3" s="16"/>
       <c r="H3" s="16"/>
     </row>
-    <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="19" t="s">
         <v>296</v>
       </c>
@@ -13636,7 +13705,7 @@
         <v>915</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
         <v>296</v>
       </c>
@@ -13660,7 +13729,7 @@
         <v>916</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="13" t="s">
         <v>304</v>
       </c>
@@ -13674,7 +13743,7 @@
       <c r="G6" s="13"/>
       <c r="H6" s="13"/>
     </row>
-    <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="14" t="s">
         <v>304</v>
       </c>
@@ -13696,7 +13765,7 @@
       <c r="G7" s="16"/>
       <c r="H7" s="16"/>
     </row>
-    <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="19" t="s">
         <v>304</v>
       </c>
@@ -13718,7 +13787,7 @@
       <c r="G8" s="21"/>
       <c r="H8" s="21"/>
     </row>
-    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="14" t="s">
         <v>304</v>
       </c>
@@ -13740,7 +13809,7 @@
       <c r="G9" s="16"/>
       <c r="H9" s="16"/>
     </row>
-    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="19" t="s">
         <v>304</v>
       </c>
@@ -13762,7 +13831,7 @@
       <c r="G10" s="21"/>
       <c r="H10" s="21"/>
     </row>
-    <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="14" t="s">
         <v>304</v>
       </c>
@@ -13784,7 +13853,7 @@
       <c r="G11" s="16"/>
       <c r="H11" s="16"/>
     </row>
-    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="19" t="s">
         <v>304</v>
       </c>
@@ -13806,7 +13875,7 @@
       <c r="G12" s="21"/>
       <c r="H12" s="21"/>
     </row>
-    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="14" t="s">
         <v>304</v>
       </c>
@@ -13828,7 +13897,7 @@
       <c r="G13" s="16"/>
       <c r="H13" s="16"/>
     </row>
-    <row r="14" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="19" t="s">
         <v>304</v>
       </c>
@@ -13850,7 +13919,7 @@
       <c r="G14" s="21"/>
       <c r="H14" s="21"/>
     </row>
-    <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="14" t="s">
         <v>304</v>
       </c>
@@ -13874,7 +13943,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="19" t="s">
         <v>304</v>
       </c>
@@ -13898,7 +13967,7 @@
         <v>917</v>
       </c>
     </row>
-    <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="14" t="s">
         <v>304</v>
       </c>
@@ -13922,7 +13991,7 @@
         <v>915</v>
       </c>
     </row>
-    <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="19" t="s">
         <v>304</v>
       </c>
@@ -13946,7 +14015,7 @@
         <v>918</v>
       </c>
     </row>
-    <row r="19" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="13" t="s">
         <v>330</v>
       </c>
@@ -13960,7 +14029,7 @@
       <c r="G19" s="13"/>
       <c r="H19" s="13"/>
     </row>
-    <row r="20" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="14" t="s">
         <v>330</v>
       </c>
@@ -13982,7 +14051,7 @@
       <c r="G20" s="16"/>
       <c r="H20" s="16"/>
     </row>
-    <row r="21" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="19" t="s">
         <v>330</v>
       </c>
@@ -14004,7 +14073,7 @@
       <c r="G21" s="21"/>
       <c r="H21" s="21"/>
     </row>
-    <row r="22" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="14" t="s">
         <v>330</v>
       </c>
@@ -14028,7 +14097,7 @@
         <v>916</v>
       </c>
     </row>
-    <row r="23" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="19" t="s">
         <v>330</v>
       </c>
@@ -14052,7 +14121,7 @@
         <v>916</v>
       </c>
     </row>
-    <row r="24" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="14" t="s">
         <v>330</v>
       </c>
@@ -14074,7 +14143,7 @@
       <c r="G24" s="16"/>
       <c r="H24" s="16"/>
     </row>
-    <row r="25" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="19" t="s">
         <v>330</v>
       </c>
@@ -14096,7 +14165,7 @@
       <c r="G25" s="21"/>
       <c r="H25" s="21"/>
     </row>
-    <row r="26" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="14" t="s">
         <v>330</v>
       </c>
@@ -14118,7 +14187,7 @@
       <c r="G26" s="16"/>
       <c r="H26" s="16"/>
     </row>
-    <row r="27" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="19" t="s">
         <v>330</v>
       </c>
@@ -14140,7 +14209,7 @@
       <c r="G27" s="21"/>
       <c r="H27" s="21"/>
     </row>
-    <row r="28" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="13" t="s">
         <v>348</v>
       </c>
@@ -14154,7 +14223,7 @@
       <c r="G28" s="13"/>
       <c r="H28" s="13"/>
     </row>
-    <row r="29" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="14" t="s">
         <v>348</v>
       </c>
@@ -14176,7 +14245,7 @@
       <c r="G29" s="16"/>
       <c r="H29" s="16"/>
     </row>
-    <row r="30" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="19" t="s">
         <v>348</v>
       </c>
@@ -14198,7 +14267,7 @@
       <c r="G30" s="21"/>
       <c r="H30" s="21"/>
     </row>
-    <row r="31" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="14" t="s">
         <v>348</v>
       </c>
@@ -14222,7 +14291,7 @@
         <v>919</v>
       </c>
     </row>
-    <row r="32" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="19" t="s">
         <v>348</v>
       </c>
@@ -14246,7 +14315,7 @@
         <v>920</v>
       </c>
     </row>
-    <row r="33" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="14" t="s">
         <v>348</v>
       </c>
@@ -14268,7 +14337,7 @@
       <c r="G33" s="16"/>
       <c r="H33" s="16"/>
     </row>
-    <row r="34" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="19" t="s">
         <v>348</v>
       </c>
@@ -14290,7 +14359,7 @@
       <c r="G34" s="21"/>
       <c r="H34" s="21"/>
     </row>
-    <row r="35" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="13" t="s">
         <v>362</v>
       </c>
@@ -14304,7 +14373,7 @@
       <c r="G35" s="13"/>
       <c r="H35" s="13"/>
     </row>
-    <row r="36" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="14" t="s">
         <v>362</v>
       </c>
@@ -14328,7 +14397,7 @@
         <v>919</v>
       </c>
     </row>
-    <row r="37" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="19" t="s">
         <v>362</v>
       </c>
@@ -14352,7 +14421,7 @@
         <v>917</v>
       </c>
     </row>
-    <row r="38" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="14" t="s">
         <v>362</v>
       </c>
@@ -14376,7 +14445,7 @@
         <v>918</v>
       </c>
     </row>
-    <row r="39" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="19" t="s">
         <v>362</v>
       </c>
@@ -14400,7 +14469,7 @@
         <v>918</v>
       </c>
     </row>
-    <row r="40" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="14" t="s">
         <v>362</v>
       </c>
@@ -14424,7 +14493,7 @@
         <v>921</v>
       </c>
     </row>
-    <row r="41" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="19" t="s">
         <v>362</v>
       </c>
@@ -14446,7 +14515,7 @@
       <c r="G41" s="21"/>
       <c r="H41" s="21"/>
     </row>
-    <row r="42" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="14" t="s">
         <v>362</v>
       </c>
@@ -14468,7 +14537,7 @@
       <c r="G42" s="16"/>
       <c r="H42" s="16"/>
     </row>
-    <row r="43" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="19" t="s">
         <v>362</v>
       </c>
@@ -14490,7 +14559,7 @@
       <c r="G43" s="21"/>
       <c r="H43" s="21"/>
     </row>
-    <row r="44" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="13" t="s">
         <v>380</v>
       </c>
@@ -14504,7 +14573,7 @@
       <c r="G44" s="13"/>
       <c r="H44" s="13"/>
     </row>
-    <row r="45" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="14" t="s">
         <v>380</v>
       </c>
@@ -14528,7 +14597,7 @@
         <v>916</v>
       </c>
     </row>
-    <row r="46" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="19" t="s">
         <v>380</v>
       </c>
@@ -14552,7 +14621,7 @@
         <v>919</v>
       </c>
     </row>
-    <row r="47" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="14" t="s">
         <v>380</v>
       </c>
@@ -14576,7 +14645,7 @@
         <v>922</v>
       </c>
     </row>
-    <row r="48" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="19" t="s">
         <v>380</v>
       </c>
@@ -14598,7 +14667,7 @@
       <c r="G48" s="21"/>
       <c r="H48" s="21"/>
     </row>
-    <row r="49" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="13" t="s">
         <v>390</v>
       </c>
@@ -14612,7 +14681,7 @@
       <c r="G49" s="13"/>
       <c r="H49" s="13"/>
     </row>
-    <row r="50" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="14" t="s">
         <v>390</v>
       </c>
@@ -14634,7 +14703,7 @@
       <c r="G50" s="16"/>
       <c r="H50" s="16"/>
     </row>
-    <row r="51" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="19" t="s">
         <v>390</v>
       </c>
@@ -14656,7 +14725,7 @@
       <c r="G51" s="21"/>
       <c r="H51" s="21"/>
     </row>
-    <row r="52" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="13" t="s">
         <v>396</v>
       </c>
@@ -14670,7 +14739,7 @@
       <c r="G52" s="13"/>
       <c r="H52" s="13"/>
     </row>
-    <row r="53" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="14" t="s">
         <v>396</v>
       </c>
@@ -14694,7 +14763,7 @@
         <v>903</v>
       </c>
     </row>
-    <row r="54" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" s="19" t="s">
         <v>396</v>
       </c>
@@ -14718,7 +14787,7 @@
         <v>919</v>
       </c>
     </row>
-    <row r="55" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="14" t="s">
         <v>396</v>
       </c>
@@ -14742,7 +14811,7 @@
         <v>919</v>
       </c>
     </row>
-    <row r="56" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="19" t="s">
         <v>396</v>
       </c>
@@ -14792,7 +14861,7 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:H26"/>
-  <sheetFormatPr defaultColWidth="8.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
@@ -14804,7 +14873,7 @@
     <col min="8" max="8" width="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" ht="28.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="12" t="s">
         <v>33</v>
       </c>
@@ -14830,7 +14899,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="13" t="s">
         <v>406</v>
       </c>
@@ -14844,7 +14913,7 @@
       <c r="G2" s="13"/>
       <c r="H2" s="13"/>
     </row>
-    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
         <v>406</v>
       </c>
@@ -14868,7 +14937,7 @@
         <v>919</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="19" t="s">
         <v>406</v>
       </c>
@@ -14892,7 +14961,7 @@
         <v>923</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
         <v>406</v>
       </c>
@@ -14916,7 +14985,7 @@
         <v>924</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="13" t="s">
         <v>414</v>
       </c>
@@ -14930,7 +14999,7 @@
       <c r="G6" s="13"/>
       <c r="H6" s="13"/>
     </row>
-    <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="14" t="s">
         <v>414</v>
       </c>
@@ -14952,7 +15021,7 @@
       <c r="G7" s="16"/>
       <c r="H7" s="16"/>
     </row>
-    <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="19" t="s">
         <v>414</v>
       </c>
@@ -14974,7 +15043,7 @@
       <c r="G8" s="21"/>
       <c r="H8" s="21"/>
     </row>
-    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="14" t="s">
         <v>414</v>
       </c>
@@ -14996,7 +15065,7 @@
       <c r="G9" s="16"/>
       <c r="H9" s="16"/>
     </row>
-    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="19" t="s">
         <v>414</v>
       </c>
@@ -15018,7 +15087,7 @@
       <c r="G10" s="21"/>
       <c r="H10" s="21"/>
     </row>
-    <row r="11" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="13" t="s">
         <v>424</v>
       </c>
@@ -15032,7 +15101,7 @@
       <c r="G11" s="13"/>
       <c r="H11" s="13"/>
     </row>
-    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="14" t="s">
         <v>424</v>
       </c>
@@ -15056,7 +15125,7 @@
         <v>919</v>
       </c>
     </row>
-    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="19" t="s">
         <v>424</v>
       </c>
@@ -15080,7 +15149,7 @@
         <v>919</v>
       </c>
     </row>
-    <row r="14" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="13" t="s">
         <v>430</v>
       </c>
@@ -15094,7 +15163,7 @@
       <c r="G14" s="13"/>
       <c r="H14" s="13"/>
     </row>
-    <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="14" t="s">
         <v>430</v>
       </c>
@@ -15116,7 +15185,7 @@
       <c r="G15" s="16"/>
       <c r="H15" s="16"/>
     </row>
-    <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="19" t="s">
         <v>430</v>
       </c>
@@ -15138,7 +15207,7 @@
       <c r="G16" s="21"/>
       <c r="H16" s="21"/>
     </row>
-    <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="14" t="s">
         <v>430</v>
       </c>
@@ -15162,7 +15231,7 @@
         <v>925</v>
       </c>
     </row>
-    <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="19" t="s">
         <v>430</v>
       </c>
@@ -15186,7 +15255,7 @@
         <v>926</v>
       </c>
     </row>
-    <row r="19" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="14" t="s">
         <v>430</v>
       </c>
@@ -15210,7 +15279,7 @@
         <v>927</v>
       </c>
     </row>
-    <row r="20" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="13" t="s">
         <v>442</v>
       </c>
@@ -15224,7 +15293,7 @@
       <c r="G20" s="13"/>
       <c r="H20" s="13"/>
     </row>
-    <row r="21" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="14" t="s">
         <v>442</v>
       </c>
@@ -15248,7 +15317,7 @@
         <v>916</v>
       </c>
     </row>
-    <row r="22" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="19" t="s">
         <v>442</v>
       </c>
@@ -15272,7 +15341,7 @@
         <v>925</v>
       </c>
     </row>
-    <row r="23" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="14" t="s">
         <v>442</v>
       </c>
@@ -15294,7 +15363,7 @@
       <c r="G23" s="16"/>
       <c r="H23" s="16"/>
     </row>
-    <row r="24" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="13" t="s">
         <v>450</v>
       </c>
@@ -15308,7 +15377,7 @@
       <c r="G24" s="13"/>
       <c r="H24" s="13"/>
     </row>
-    <row r="25" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="14" t="s">
         <v>450</v>
       </c>
@@ -15332,7 +15401,7 @@
         <v>924</v>
       </c>
     </row>
-    <row r="26" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="19" t="s">
         <v>450</v>
       </c>
@@ -15382,7 +15451,7 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
   <dimension ref="A1:H18"/>
-  <sheetFormatPr defaultColWidth="8.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
@@ -15394,7 +15463,7 @@
     <col min="8" max="8" width="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" ht="28.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="12" t="s">
         <v>33</v>
       </c>
@@ -15420,7 +15489,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="13" t="s">
         <v>456</v>
       </c>
@@ -15434,7 +15503,7 @@
       <c r="G2" s="13"/>
       <c r="H2" s="13"/>
     </row>
-    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
         <v>456</v>
       </c>
@@ -15456,7 +15525,7 @@
       <c r="G3" s="16"/>
       <c r="H3" s="16"/>
     </row>
-    <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="19" t="s">
         <v>456</v>
       </c>
@@ -15480,7 +15549,7 @@
         <v>903</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
         <v>456</v>
       </c>
@@ -15502,7 +15571,7 @@
       <c r="G5" s="16"/>
       <c r="H5" s="16"/>
     </row>
-    <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="19" t="s">
         <v>456</v>
       </c>
@@ -15524,7 +15593,7 @@
       <c r="G6" s="21"/>
       <c r="H6" s="21"/>
     </row>
-    <row r="7" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="13" t="s">
         <v>466</v>
       </c>
@@ -15538,7 +15607,7 @@
       <c r="G7" s="13"/>
       <c r="H7" s="13"/>
     </row>
-    <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="14" t="s">
         <v>466</v>
       </c>
@@ -15560,7 +15629,7 @@
       <c r="G8" s="16"/>
       <c r="H8" s="16"/>
     </row>
-    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="19" t="s">
         <v>466</v>
       </c>
@@ -15577,12 +15646,14 @@
         <v>1</v>
       </c>
       <c r="F9" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G9" s="21"/>
+        <v>984</v>
+      </c>
+      <c r="G9" s="21" t="s">
+        <v>994</v>
+      </c>
       <c r="H9" s="21"/>
     </row>
-    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="14" t="s">
         <v>466</v>
       </c>
@@ -15606,7 +15677,7 @@
         <v>903</v>
       </c>
     </row>
-    <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="19" t="s">
         <v>466</v>
       </c>
@@ -15628,7 +15699,7 @@
       <c r="G11" s="21"/>
       <c r="H11" s="21"/>
     </row>
-    <row r="12" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="13" t="s">
         <v>476</v>
       </c>
@@ -15642,7 +15713,7 @@
       <c r="G12" s="13"/>
       <c r="H12" s="13"/>
     </row>
-    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="14" t="s">
         <v>476</v>
       </c>
@@ -15664,7 +15735,7 @@
       <c r="G13" s="16"/>
       <c r="H13" s="16"/>
     </row>
-    <row r="14" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="19" t="s">
         <v>476</v>
       </c>
@@ -15686,7 +15757,7 @@
       <c r="G14" s="21"/>
       <c r="H14" s="21"/>
     </row>
-    <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="14" t="s">
         <v>476</v>
       </c>
@@ -15708,7 +15779,7 @@
       <c r="G15" s="16"/>
       <c r="H15" s="16"/>
     </row>
-    <row r="16" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="13" t="s">
         <v>484</v>
       </c>
@@ -15722,7 +15793,7 @@
       <c r="G16" s="13"/>
       <c r="H16" s="13"/>
     </row>
-    <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="14" t="s">
         <v>484</v>
       </c>
@@ -15746,7 +15817,7 @@
         <v>901</v>
       </c>
     </row>
-    <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="19" t="s">
         <v>484</v>
       </c>

</xml_diff>

<commit_message>
docs: modify ASVS 5.0 Tracker file
</commit_message>
<xml_diff>
--- a/Deliverables/Phase_1/ASVS_5.0_Tracker.xlsx
+++ b/Deliverables/Phase_1/ASVS_5.0_Tracker.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Utilizador\Desktop\DESOFS\desofs2026-thu_crr_2\Deliverables\Phase_1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B1366F7-E48A-4B1A-9830-CE29546F8FAE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F114A21-7639-42EF-ADE5-2639FE0B64F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1950" yWindow="1950" windowWidth="21600" windowHeight="11385" tabRatio="500" firstSheet="13" activeTab="14" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="500" firstSheet="14" activeTab="14" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2337" uniqueCount="996">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2257" uniqueCount="1005">
   <si>
     <t>OWASP ASVS 5.0 – Compliance Tracker</t>
   </si>
@@ -2942,9 +2942,6 @@
     <t>SR-05, SR-10, SR-11</t>
   </si>
   <si>
-    <t>SR-03, SR-05, SR-10, SR-11</t>
-  </si>
-  <si>
     <t>SR-03, SR-05, SR-07</t>
   </si>
   <si>
@@ -2993,9 +2990,6 @@
     <t>SR-01, SR-03, SR-12</t>
   </si>
   <si>
-    <t>SR-05, SR-09, SR-14</t>
-  </si>
-  <si>
     <t>SR-03, SR-05, SR-08</t>
   </si>
   <si>
@@ -3051,6 +3045,39 @@
   </si>
   <si>
     <t>authMiddleware.ts - token read exclusively from Authorization header, never from query string.</t>
+  </si>
+  <si>
+    <t>SR-05, SR-10, SR-11, MT22(https://github.com/mei-desofs/desofs2026-thu_crr_2/pull/1)</t>
+  </si>
+  <si>
+    <t>SR-05, SR-09, SR-14, MT22, MT23, MT24 (https://github.com/mei-desofs/desofs2026-thu_crr_2/pull/1)</t>
+  </si>
+  <si>
+    <t>MT22 (https://github.com/mei-desofs/desofs2026-thu_crr_2/pull/1)</t>
+  </si>
+  <si>
+    <t>SR-08, SR-09, SR-14, MT22 (https://github.com/mei-desofs/desofs2026-thu_crr_2/pull/1)</t>
+  </si>
+  <si>
+    <t>SR-03, SR-05, SR-10, SR-11, MT19 (https://github.com/mei-desofs/desofs2026-thu_crr_2/pull/2)</t>
+  </si>
+  <si>
+    <t>MT17 (https://github.com/mei-desofs/desofs2026-thu_crr_2/pull/7)</t>
+  </si>
+  <si>
+    <t>MT16 (https://github.com/mei-desofs/desofs2026-thu_crr_2/pull/6)</t>
+  </si>
+  <si>
+    <t>MT15(https://github.com/mei-desofs/desofs2026-thu_crr_2/pull/5), MT16 (https://github.com/mei-desofs/desofs2026-thu_crr_2/pull/6)</t>
+  </si>
+  <si>
+    <t>MT13 (https://github.com/mei-desofs/desofs2026-thu_crr_2/pull/3)</t>
+  </si>
+  <si>
+    <t>MT14 (https://github.com/mei-desofs/desofs2026-thu_crr_2/pull/4)</t>
+  </si>
+  <si>
+    <t>MT16(https://github.com/mei-desofs/desofs2026-thu_crr_2/pull/6), MT14(https://github.com/mei-desofs/desofs2026-thu_crr_2/pull/4)</t>
   </si>
 </sst>
 </file>
@@ -3295,6 +3322,10 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -3302,10 +3333,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3759,7 +3786,7 @@
                   <c:v>0.1</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>0.1875</c:v>
+                  <c:v>0.25</c:v>
                 </c:pt>
                 <c:pt idx="16">
                   <c:v>0</c:v>
@@ -4124,7 +4151,7 @@
                   <c:v>4.7619047619047616E-2</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>0.23529411764705882</c:v>
+                  <c:v>0.29411764705882354</c:v>
                 </c:pt>
                 <c:pt idx="16">
                   <c:v>0</c:v>
@@ -4647,46 +4674,46 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="25" t="s">
+      <c r="A1" s="27" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="25"/>
-      <c r="C1" s="25"/>
-      <c r="D1" s="25"/>
-      <c r="E1" s="25"/>
-      <c r="F1" s="25"/>
-      <c r="G1" s="25"/>
-      <c r="H1" s="25"/>
-      <c r="I1" s="25"/>
-      <c r="J1" s="25"/>
-      <c r="K1" s="25"/>
-      <c r="L1" s="25"/>
-      <c r="M1" s="25"/>
-      <c r="N1" s="25"/>
-      <c r="O1" s="25"/>
-      <c r="P1" s="25"/>
+      <c r="B1" s="27"/>
+      <c r="C1" s="27"/>
+      <c r="D1" s="27"/>
+      <c r="E1" s="27"/>
+      <c r="F1" s="27"/>
+      <c r="G1" s="27"/>
+      <c r="H1" s="27"/>
+      <c r="I1" s="27"/>
+      <c r="J1" s="27"/>
+      <c r="K1" s="27"/>
+      <c r="L1" s="27"/>
+      <c r="M1" s="27"/>
+      <c r="N1" s="27"/>
+      <c r="O1" s="27"/>
+      <c r="P1" s="27"/>
     </row>
     <row r="2" spans="1:16" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="26"/>
-      <c r="B2" s="26"/>
-      <c r="C2" s="26"/>
-      <c r="D2" s="26"/>
-      <c r="E2" s="26"/>
-      <c r="F2" s="26"/>
-      <c r="G2" s="26"/>
-      <c r="H2" s="26"/>
-      <c r="I2" s="26"/>
-      <c r="J2" s="26"/>
-      <c r="K2" s="26"/>
-      <c r="L2" s="26"/>
-      <c r="M2" s="26"/>
-      <c r="N2" s="26"/>
-      <c r="O2" s="26"/>
-      <c r="P2" s="26"/>
+      <c r="A2" s="28"/>
+      <c r="B2" s="28"/>
+      <c r="C2" s="28"/>
+      <c r="D2" s="28"/>
+      <c r="E2" s="28"/>
+      <c r="F2" s="28"/>
+      <c r="G2" s="28"/>
+      <c r="H2" s="28"/>
+      <c r="I2" s="28"/>
+      <c r="J2" s="28"/>
+      <c r="K2" s="28"/>
+      <c r="L2" s="28"/>
+      <c r="M2" s="28"/>
+      <c r="N2" s="28"/>
+      <c r="O2" s="28"/>
+      <c r="P2" s="28"/>
     </row>
     <row r="3" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="27"/>
-      <c r="B3" s="27"/>
+      <c r="A3" s="29"/>
+      <c r="B3" s="29"/>
       <c r="C3" s="1"/>
       <c r="E3" s="1"/>
       <c r="G3" s="1"/>
@@ -5490,11 +5517,11 @@
       </c>
       <c r="G21" s="7">
         <f>COUNTIFS('V16 - Security Logging and Erro'!$F$2:$F$23,"Compliant",'V16 - Security Logging and Erro'!$E$2:$E$23,2)</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H21" s="8">
         <f t="shared" si="1"/>
-        <v>0.1875</v>
+        <v>0.25</v>
       </c>
       <c r="I21" s="7">
         <v>1</v>
@@ -5509,11 +5536,11 @@
       </c>
       <c r="L21" s="7">
         <f>COUNTIF('V16 - Security Logging and Erro'!$F$2:$F$23,"Compliant")</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M21" s="8">
         <f t="shared" si="3"/>
-        <v>0.23529411764705882</v>
+        <v>0.29411764705882354</v>
       </c>
     </row>
     <row r="22" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -5589,11 +5616,11 @@
       </c>
       <c r="G23" s="10">
         <f>SUM(G6:G22)</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H23" s="11">
         <f>IFERROR(AVERAGE(H6:H22),"")</f>
-        <v>2.2259358288770053E-2</v>
+        <v>2.5935828877005348E-2</v>
       </c>
       <c r="I23" s="10">
         <f>SUM(I6:I22)</f>
@@ -5609,11 +5636,11 @@
       </c>
       <c r="L23" s="10">
         <f>SUM(L6:L22)</f>
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="M23" s="11">
         <f>IFERROR(AVERAGE(M6:M22),"")</f>
-        <v>8.1558448119687599E-2</v>
+        <v>8.5018655732144344E-2</v>
       </c>
     </row>
   </sheetData>
@@ -5748,7 +5775,7 @@
         <v>1</v>
       </c>
       <c r="F3" s="18" t="s">
-        <v>984</v>
+        <v>982</v>
       </c>
       <c r="G3" s="16"/>
       <c r="H3" s="16"/>
@@ -5770,7 +5797,7 @@
         <v>1</v>
       </c>
       <c r="F4" s="18" t="s">
-        <v>983</v>
+        <v>981</v>
       </c>
       <c r="G4" s="21"/>
       <c r="H4" s="21"/>
@@ -5792,7 +5819,7 @@
         <v>1</v>
       </c>
       <c r="F5" s="18" t="s">
-        <v>984</v>
+        <v>982</v>
       </c>
       <c r="G5" s="16"/>
       <c r="H5" s="16"/>
@@ -5828,7 +5855,7 @@
         <v>1</v>
       </c>
       <c r="F7" s="18" t="s">
-        <v>983</v>
+        <v>981</v>
       </c>
       <c r="G7" s="16"/>
       <c r="H7" s="16"/>
@@ -5850,7 +5877,7 @@
         <v>2</v>
       </c>
       <c r="F8" s="18" t="s">
-        <v>983</v>
+        <v>981</v>
       </c>
       <c r="G8" s="21"/>
       <c r="H8" s="21" t="s">
@@ -7108,7 +7135,7 @@
         <v>2</v>
       </c>
       <c r="F8" s="18" t="s">
-        <v>983</v>
+        <v>981</v>
       </c>
       <c r="G8" s="16"/>
       <c r="H8" s="16" t="s">
@@ -7156,7 +7183,7 @@
         <v>2</v>
       </c>
       <c r="F10" s="18" t="s">
-        <v>983</v>
+        <v>981</v>
       </c>
       <c r="G10" s="16"/>
       <c r="H10" s="16" t="s">
@@ -7364,7 +7391,7 @@
         <v>1</v>
       </c>
       <c r="F20" s="18" t="s">
-        <v>984</v>
+        <v>982</v>
       </c>
       <c r="G20" s="16"/>
       <c r="H20" s="16"/>
@@ -7386,7 +7413,7 @@
         <v>2</v>
       </c>
       <c r="F21" s="18" t="s">
-        <v>983</v>
+        <v>981</v>
       </c>
       <c r="G21" s="21"/>
       <c r="H21" s="21" t="s">
@@ -7410,7 +7437,7 @@
         <v>2</v>
       </c>
       <c r="F22" s="18" t="s">
-        <v>983</v>
+        <v>981</v>
       </c>
       <c r="G22" s="16"/>
       <c r="H22" s="16" t="s">
@@ -7434,7 +7461,7 @@
         <v>2</v>
       </c>
       <c r="F23" s="18" t="s">
-        <v>983</v>
+        <v>981</v>
       </c>
       <c r="G23" s="21"/>
       <c r="H23" s="21" t="s">
@@ -7532,7 +7559,7 @@
         <v>2</v>
       </c>
       <c r="F28" s="18" t="s">
-        <v>983</v>
+        <v>981</v>
       </c>
       <c r="G28" s="16"/>
       <c r="H28" s="16" t="s">
@@ -8200,7 +8227,7 @@
         <v>2</v>
       </c>
       <c r="F8" s="18" t="s">
-        <v>983</v>
+        <v>981</v>
       </c>
       <c r="G8" s="16"/>
       <c r="H8" s="16" t="s">
@@ -8272,7 +8299,7 @@
         <v>2</v>
       </c>
       <c r="F11" s="18" t="s">
-        <v>983</v>
+        <v>981</v>
       </c>
       <c r="G11" s="21"/>
       <c r="H11" s="21" t="s">
@@ -8508,7 +8535,7 @@
         <v>2</v>
       </c>
       <c r="F22" s="18" t="s">
-        <v>983</v>
+        <v>981</v>
       </c>
       <c r="G22" s="16"/>
       <c r="H22" s="16" t="s">
@@ -8702,7 +8729,7 @@
         <v>2</v>
       </c>
       <c r="F3" s="18" t="s">
-        <v>983</v>
+        <v>981</v>
       </c>
       <c r="G3" s="16"/>
       <c r="H3" s="16" t="s">
@@ -8764,12 +8791,14 @@
         <v>1</v>
       </c>
       <c r="F6" s="18" t="s">
-        <v>984</v>
+        <v>982</v>
       </c>
       <c r="G6" s="16" t="s">
-        <v>995</v>
-      </c>
-      <c r="H6" s="16"/>
+        <v>993</v>
+      </c>
+      <c r="H6" s="16" t="s">
+        <v>1004</v>
+      </c>
     </row>
     <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="19" t="s">
@@ -9156,7 +9185,7 @@
         <v>2</v>
       </c>
       <c r="F5" s="18" t="s">
-        <v>983</v>
+        <v>981</v>
       </c>
       <c r="G5" s="16"/>
       <c r="H5" s="16" t="s">
@@ -9260,13 +9289,13 @@
         <v>2</v>
       </c>
       <c r="F10" s="18" t="s">
-        <v>984</v>
+        <v>982</v>
       </c>
       <c r="G10" s="21" t="s">
-        <v>989</v>
+        <v>987</v>
       </c>
       <c r="H10" s="21" t="s">
-        <v>959</v>
+        <v>998</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -9286,11 +9315,11 @@
         <v>2</v>
       </c>
       <c r="F11" s="18" t="s">
-        <v>983</v>
+        <v>981</v>
       </c>
       <c r="G11" s="16"/>
       <c r="H11" s="16" t="s">
-        <v>960</v>
+        <v>959</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -9312,7 +9341,7 @@
       <c r="F12" s="18" t="s">
         <v>45</v>
       </c>
-      <c r="G12" s="29"/>
+      <c r="G12" s="26"/>
       <c r="H12" s="21"/>
     </row>
     <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -9368,7 +9397,7 @@
         <v>1</v>
       </c>
       <c r="F15" s="18" t="s">
-        <v>983</v>
+        <v>981</v>
       </c>
       <c r="G15" s="16"/>
       <c r="H15" s="16"/>
@@ -9394,7 +9423,7 @@
       </c>
       <c r="G16" s="21"/>
       <c r="H16" s="21" t="s">
-        <v>961</v>
+        <v>960</v>
       </c>
     </row>
     <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -9414,11 +9443,11 @@
         <v>2</v>
       </c>
       <c r="F17" s="18" t="s">
-        <v>983</v>
+        <v>981</v>
       </c>
       <c r="G17" s="16"/>
       <c r="H17" s="16" t="s">
-        <v>962</v>
+        <v>961</v>
       </c>
     </row>
     <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -9442,7 +9471,7 @@
       </c>
       <c r="G18" s="21"/>
       <c r="H18" s="21" t="s">
-        <v>963</v>
+        <v>962</v>
       </c>
     </row>
     <row r="19" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -9462,11 +9491,11 @@
         <v>2</v>
       </c>
       <c r="F19" s="18" t="s">
-        <v>983</v>
+        <v>981</v>
       </c>
       <c r="G19" s="16"/>
       <c r="H19" s="16" t="s">
-        <v>964</v>
+        <v>963</v>
       </c>
     </row>
     <row r="20" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -9486,11 +9515,11 @@
         <v>2</v>
       </c>
       <c r="F20" s="18" t="s">
-        <v>983</v>
+        <v>981</v>
       </c>
       <c r="G20" s="21"/>
       <c r="H20" s="21" t="s">
-        <v>964</v>
+        <v>963</v>
       </c>
     </row>
     <row r="21" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -9514,7 +9543,7 @@
       </c>
       <c r="G21" s="16"/>
       <c r="H21" s="16" t="s">
-        <v>965</v>
+        <v>964</v>
       </c>
     </row>
     <row r="22" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -9718,7 +9747,7 @@
       </c>
       <c r="G3" s="16"/>
       <c r="H3" s="16" t="s">
-        <v>966</v>
+        <v>965</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -9756,7 +9785,7 @@
       </c>
       <c r="G5" s="16"/>
       <c r="H5" s="16" t="s">
-        <v>967</v>
+        <v>966</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -9780,7 +9809,7 @@
       </c>
       <c r="G6" s="21"/>
       <c r="H6" s="21" t="s">
-        <v>968</v>
+        <v>967</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -9804,7 +9833,7 @@
       </c>
       <c r="G7" s="16"/>
       <c r="H7" s="16" t="s">
-        <v>969</v>
+        <v>968</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -9828,7 +9857,7 @@
       </c>
       <c r="G8" s="21"/>
       <c r="H8" s="21" t="s">
-        <v>967</v>
+        <v>966</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -9852,7 +9881,7 @@
       </c>
       <c r="G9" s="16"/>
       <c r="H9" s="16" t="s">
-        <v>970</v>
+        <v>969</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -9890,7 +9919,7 @@
       </c>
       <c r="G11" s="16"/>
       <c r="H11" s="16" t="s">
-        <v>971</v>
+        <v>970</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -9914,7 +9943,7 @@
       </c>
       <c r="G12" s="21"/>
       <c r="H12" s="21" t="s">
-        <v>972</v>
+        <v>971</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -9938,7 +9967,7 @@
       </c>
       <c r="G13" s="16"/>
       <c r="H13" s="16" t="s">
-        <v>973</v>
+        <v>972</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -9962,7 +9991,7 @@
       </c>
       <c r="G14" s="21"/>
       <c r="H14" s="21" t="s">
-        <v>974</v>
+        <v>973</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -9996,11 +10025,11 @@
         <v>2</v>
       </c>
       <c r="F16" s="18" t="s">
-        <v>45</v>
+        <v>982</v>
       </c>
       <c r="G16" s="16"/>
       <c r="H16" s="16" t="s">
-        <v>964</v>
+        <v>997</v>
       </c>
     </row>
     <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -10024,7 +10053,7 @@
       </c>
       <c r="G17" s="21"/>
       <c r="H17" s="21" t="s">
-        <v>975</v>
+        <v>974</v>
       </c>
     </row>
     <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -10048,7 +10077,7 @@
       </c>
       <c r="G18" s="16"/>
       <c r="H18" s="16" t="s">
-        <v>974</v>
+        <v>973</v>
       </c>
     </row>
     <row r="19" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -10082,13 +10111,13 @@
         <v>2</v>
       </c>
       <c r="F20" s="18" t="s">
-        <v>984</v>
+        <v>982</v>
       </c>
       <c r="G20" s="16" t="s">
-        <v>985</v>
+        <v>983</v>
       </c>
       <c r="H20" s="16" t="s">
-        <v>976</v>
+        <v>995</v>
       </c>
     </row>
     <row r="21" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -10108,13 +10137,13 @@
         <v>2</v>
       </c>
       <c r="F21" s="18" t="s">
+        <v>982</v>
+      </c>
+      <c r="G21" s="16" t="s">
         <v>984</v>
       </c>
-      <c r="G21" s="16" t="s">
-        <v>986</v>
-      </c>
       <c r="H21" s="21" t="s">
-        <v>958</v>
+        <v>994</v>
       </c>
     </row>
     <row r="22" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -10134,13 +10163,13 @@
         <v>2</v>
       </c>
       <c r="F22" s="18" t="s">
-        <v>984</v>
+        <v>982</v>
       </c>
       <c r="G22" s="16" t="s">
-        <v>987</v>
+        <v>985</v>
       </c>
       <c r="H22" s="16" t="s">
-        <v>977</v>
+        <v>975</v>
       </c>
     </row>
     <row r="23" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -10160,18 +10189,20 @@
         <v>3</v>
       </c>
       <c r="F23" s="18" t="s">
-        <v>984</v>
+        <v>982</v>
       </c>
       <c r="G23" s="16" t="s">
-        <v>988</v>
-      </c>
-      <c r="H23" s="21"/>
+        <v>986</v>
+      </c>
+      <c r="H23" s="21" t="s">
+        <v>996</v>
+      </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="G25" s="28"/>
+      <c r="G25" s="25"/>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="G26" s="28"/>
+      <c r="G26" s="25"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="F2:F23">
@@ -10272,7 +10303,7 @@
       </c>
       <c r="G3" s="16"/>
       <c r="H3" s="16" t="s">
-        <v>978</v>
+        <v>976</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -10332,7 +10363,7 @@
       </c>
       <c r="G6" s="16"/>
       <c r="H6" s="16" t="s">
-        <v>979</v>
+        <v>977</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -10356,7 +10387,7 @@
       </c>
       <c r="G7" s="21"/>
       <c r="H7" s="21" t="s">
-        <v>980</v>
+        <v>978</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -10380,7 +10411,7 @@
       </c>
       <c r="G8" s="16"/>
       <c r="H8" s="16" t="s">
-        <v>981</v>
+        <v>979</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -10404,7 +10435,7 @@
       </c>
       <c r="G9" s="21"/>
       <c r="H9" s="21" t="s">
-        <v>973</v>
+        <v>972</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -10554,7 +10585,7 @@
       </c>
       <c r="G16" s="21"/>
       <c r="H16" s="21" t="s">
-        <v>982</v>
+        <v>980</v>
       </c>
     </row>
   </sheetData>
@@ -10652,7 +10683,7 @@
         <v>2</v>
       </c>
       <c r="F3" s="18" t="s">
-        <v>983</v>
+        <v>981</v>
       </c>
       <c r="G3" s="16"/>
       <c r="H3" s="16"/>
@@ -10674,7 +10705,7 @@
         <v>2</v>
       </c>
       <c r="F4" s="18" t="s">
-        <v>983</v>
+        <v>981</v>
       </c>
       <c r="G4" s="21"/>
       <c r="H4" s="21"/>
@@ -10776,7 +10807,7 @@
         <v>1</v>
       </c>
       <c r="F9" s="18" t="s">
-        <v>984</v>
+        <v>982</v>
       </c>
       <c r="G9" s="21"/>
       <c r="H9" s="21"/>
@@ -10798,7 +10829,7 @@
         <v>1</v>
       </c>
       <c r="F10" s="18" t="s">
-        <v>984</v>
+        <v>982</v>
       </c>
       <c r="G10" s="16"/>
       <c r="H10" s="16"/>
@@ -10972,7 +11003,7 @@
         <v>1</v>
       </c>
       <c r="F18" s="18" t="s">
-        <v>984</v>
+        <v>982</v>
       </c>
       <c r="G18" s="21"/>
       <c r="H18" s="21"/>
@@ -10994,7 +11025,7 @@
         <v>2</v>
       </c>
       <c r="F19" s="18" t="s">
-        <v>983</v>
+        <v>981</v>
       </c>
       <c r="G19" s="16"/>
       <c r="H19" s="16" t="s">
@@ -11270,7 +11301,7 @@
         <v>2</v>
       </c>
       <c r="F31" s="18" t="s">
-        <v>983</v>
+        <v>981</v>
       </c>
       <c r="G31" s="21"/>
       <c r="H31" s="21" t="s">
@@ -11354,7 +11385,7 @@
         <v>2</v>
       </c>
       <c r="F35" s="18" t="s">
-        <v>983</v>
+        <v>981</v>
       </c>
       <c r="G35" s="21"/>
       <c r="H35" s="21" t="s">
@@ -11478,7 +11509,7 @@
         <v>1</v>
       </c>
       <c r="F3" s="18" t="s">
-        <v>983</v>
+        <v>981</v>
       </c>
       <c r="G3" s="16"/>
       <c r="H3" s="16"/>
@@ -11562,7 +11593,7 @@
         <v>1</v>
       </c>
       <c r="F7" s="18" t="s">
-        <v>983</v>
+        <v>981</v>
       </c>
       <c r="G7" s="16"/>
       <c r="H7" s="16"/>
@@ -11584,7 +11615,7 @@
         <v>1</v>
       </c>
       <c r="F8" s="18" t="s">
-        <v>984</v>
+        <v>982</v>
       </c>
       <c r="G8" s="21"/>
       <c r="H8" s="21"/>
@@ -11606,7 +11637,7 @@
         <v>2</v>
       </c>
       <c r="F9" s="18" t="s">
-        <v>983</v>
+        <v>981</v>
       </c>
       <c r="G9" s="16"/>
       <c r="H9" s="16" t="s">
@@ -12166,7 +12197,7 @@
         <v>1</v>
       </c>
       <c r="F16" s="18" t="s">
-        <v>983</v>
+        <v>981</v>
       </c>
       <c r="G16" s="21"/>
       <c r="H16" s="21"/>
@@ -12342,7 +12373,7 @@
         <v>1</v>
       </c>
       <c r="F24" s="18" t="s">
-        <v>983</v>
+        <v>981</v>
       </c>
       <c r="G24" s="16"/>
       <c r="H24" s="16"/>
@@ -12364,7 +12395,7 @@
         <v>1</v>
       </c>
       <c r="F25" s="18" t="s">
-        <v>983</v>
+        <v>981</v>
       </c>
       <c r="G25" s="21"/>
       <c r="H25" s="21"/>
@@ -12386,7 +12417,7 @@
         <v>1</v>
       </c>
       <c r="F26" s="18" t="s">
-        <v>983</v>
+        <v>981</v>
       </c>
       <c r="G26" s="16"/>
       <c r="H26" s="16"/>
@@ -12408,7 +12439,7 @@
         <v>2</v>
       </c>
       <c r="F27" s="18" t="s">
-        <v>983</v>
+        <v>981</v>
       </c>
       <c r="G27" s="21"/>
       <c r="H27" s="21" t="s">
@@ -12764,7 +12795,7 @@
         <v>1</v>
       </c>
       <c r="F3" s="18" t="s">
-        <v>983</v>
+        <v>981</v>
       </c>
       <c r="G3" s="16"/>
       <c r="H3" s="16"/>
@@ -12892,7 +12923,7 @@
         <v>2</v>
       </c>
       <c r="F9" s="18" t="s">
-        <v>983</v>
+        <v>981</v>
       </c>
       <c r="G9" s="16"/>
       <c r="H9" s="16" t="s">
@@ -13018,7 +13049,7 @@
         <v>2</v>
       </c>
       <c r="F15" s="18" t="s">
-        <v>983</v>
+        <v>981</v>
       </c>
       <c r="G15" s="16"/>
       <c r="H15" s="16" t="s">
@@ -13252,7 +13283,7 @@
         <v>2</v>
       </c>
       <c r="F3" s="18" t="s">
-        <v>983</v>
+        <v>981</v>
       </c>
       <c r="G3" s="16"/>
       <c r="H3" s="16" t="s">
@@ -13290,12 +13321,14 @@
         <v>1</v>
       </c>
       <c r="F5" s="18" t="s">
-        <v>984</v>
+        <v>982</v>
       </c>
       <c r="G5" s="16" t="s">
-        <v>990</v>
-      </c>
-      <c r="H5" s="16"/>
+        <v>988</v>
+      </c>
+      <c r="H5" s="16" t="s">
+        <v>999</v>
+      </c>
     </row>
     <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="19" t="s">
@@ -13314,12 +13347,14 @@
         <v>1</v>
       </c>
       <c r="F6" s="18" t="s">
-        <v>984</v>
+        <v>982</v>
       </c>
       <c r="G6" s="21" t="s">
-        <v>991</v>
-      </c>
-      <c r="H6" s="21"/>
+        <v>989</v>
+      </c>
+      <c r="H6" s="21" t="s">
+        <v>1000</v>
+      </c>
     </row>
     <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="14" t="s">
@@ -13442,12 +13477,14 @@
         <v>1</v>
       </c>
       <c r="F12" s="18" t="s">
-        <v>984</v>
+        <v>982</v>
       </c>
       <c r="G12" s="16" t="s">
-        <v>993</v>
-      </c>
-      <c r="H12" s="16"/>
+        <v>991</v>
+      </c>
+      <c r="H12" s="16" t="s">
+        <v>1002</v>
+      </c>
     </row>
     <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="19" t="s">
@@ -13466,12 +13503,14 @@
         <v>1</v>
       </c>
       <c r="F13" s="18" t="s">
-        <v>984</v>
+        <v>982</v>
       </c>
       <c r="G13" s="21" t="s">
-        <v>992</v>
-      </c>
-      <c r="H13" s="21"/>
+        <v>990</v>
+      </c>
+      <c r="H13" s="21" t="s">
+        <v>1001</v>
+      </c>
     </row>
     <row r="14" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="14" t="s">
@@ -13526,7 +13565,7 @@
         <v>2</v>
       </c>
       <c r="F16" s="18" t="s">
-        <v>983</v>
+        <v>981</v>
       </c>
       <c r="G16" s="16"/>
       <c r="H16" s="16" t="s">
@@ -13676,7 +13715,7 @@
         <v>1</v>
       </c>
       <c r="F3" s="18" t="s">
-        <v>983</v>
+        <v>981</v>
       </c>
       <c r="G3" s="16"/>
       <c r="H3" s="16"/>
@@ -13848,7 +13887,7 @@
         <v>1</v>
       </c>
       <c r="F11" s="18" t="s">
-        <v>984</v>
+        <v>982</v>
       </c>
       <c r="G11" s="16"/>
       <c r="H11" s="16"/>
@@ -13914,7 +13953,7 @@
         <v>1</v>
       </c>
       <c r="F14" s="18" t="s">
-        <v>983</v>
+        <v>981</v>
       </c>
       <c r="G14" s="21"/>
       <c r="H14" s="21"/>
@@ -13936,7 +13975,7 @@
         <v>2</v>
       </c>
       <c r="F15" s="18" t="s">
-        <v>983</v>
+        <v>981</v>
       </c>
       <c r="G15" s="16"/>
       <c r="H15" s="16" t="s">
@@ -13960,7 +13999,7 @@
         <v>2</v>
       </c>
       <c r="F16" s="18" t="s">
-        <v>984</v>
+        <v>982</v>
       </c>
       <c r="G16" s="21"/>
       <c r="H16" s="21" t="s">
@@ -14068,7 +14107,7 @@
         <v>1</v>
       </c>
       <c r="F21" s="18" t="s">
-        <v>983</v>
+        <v>981</v>
       </c>
       <c r="G21" s="21"/>
       <c r="H21" s="21"/>
@@ -14114,7 +14153,7 @@
         <v>2</v>
       </c>
       <c r="F23" s="18" t="s">
-        <v>984</v>
+        <v>982</v>
       </c>
       <c r="G23" s="21"/>
       <c r="H23" s="21" t="s">
@@ -14262,7 +14301,7 @@
         <v>1</v>
       </c>
       <c r="F30" s="18" t="s">
-        <v>984</v>
+        <v>982</v>
       </c>
       <c r="G30" s="21"/>
       <c r="H30" s="21"/>
@@ -14780,7 +14819,7 @@
         <v>2</v>
       </c>
       <c r="F54" s="18" t="s">
-        <v>983</v>
+        <v>981</v>
       </c>
       <c r="G54" s="21"/>
       <c r="H54" s="21" t="s">
@@ -15016,7 +15055,7 @@
         <v>1</v>
       </c>
       <c r="F7" s="18" t="s">
-        <v>983</v>
+        <v>981</v>
       </c>
       <c r="G7" s="16"/>
       <c r="H7" s="16"/>
@@ -15038,7 +15077,7 @@
         <v>1</v>
       </c>
       <c r="F8" s="18" t="s">
-        <v>984</v>
+        <v>982</v>
       </c>
       <c r="G8" s="21"/>
       <c r="H8" s="21"/>
@@ -15142,7 +15181,7 @@
         <v>2</v>
       </c>
       <c r="F13" s="18" t="s">
-        <v>983</v>
+        <v>981</v>
       </c>
       <c r="G13" s="21"/>
       <c r="H13" s="21" t="s">
@@ -15418,7 +15457,7 @@
         <v>2</v>
       </c>
       <c r="F26" s="18" t="s">
-        <v>983</v>
+        <v>981</v>
       </c>
       <c r="G26" s="21"/>
       <c r="H26" s="21" t="s">
@@ -15520,7 +15559,7 @@
         <v>1</v>
       </c>
       <c r="F3" s="18" t="s">
-        <v>983</v>
+        <v>981</v>
       </c>
       <c r="G3" s="16"/>
       <c r="H3" s="16"/>
@@ -15646,12 +15685,14 @@
         <v>1</v>
       </c>
       <c r="F9" s="18" t="s">
-        <v>984</v>
+        <v>982</v>
       </c>
       <c r="G9" s="21" t="s">
-        <v>994</v>
-      </c>
-      <c r="H9" s="21"/>
+        <v>992</v>
+      </c>
+      <c r="H9" s="21" t="s">
+        <v>1003</v>
+      </c>
     </row>
     <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="14" t="s">
@@ -15730,7 +15771,7 @@
         <v>1</v>
       </c>
       <c r="F13" s="18" t="s">
-        <v>983</v>
+        <v>981</v>
       </c>
       <c r="G13" s="16"/>
       <c r="H13" s="16"/>

</xml_diff>

<commit_message>
chore: update ASVS_5.0_Tracker.xlsx with new data
</commit_message>
<xml_diff>
--- a/Deliverables/Phase_1/ASVS_5.0_Tracker.xlsx
+++ b/Deliverables/Phase_1/ASVS_5.0_Tracker.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24332"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\joaod\Desktop\repos\desofs2026-thu_crr_2\Deliverables\Phase_1\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Utilizador\Desktop\DESOFS\desofs2026-thu_crr_2\Deliverables\Phase_1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18C11AB1-81A9-4672-910D-AFB76E92CE7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8DF1C60A-0940-4656-9DCF-B1F6AE87E08F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="500" firstSheet="15" activeTab="16" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="500" firstSheet="13" activeTab="13" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2270" uniqueCount="1013">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2278" uniqueCount="1021">
   <si>
     <t>OWASP ASVS 5.0 – Compliance Tracker</t>
   </si>
@@ -3102,13 +3102,57 @@
   </si>
   <si>
     <t>SR-05, SR-09, SR-14, SR-15, MT25 (https://github.com/mei-desofs/desofs2026-thu_crr_2/pull/13)</t>
+  </si>
+  <si>
+    <t>httpLogger e securityLogger incluem timestamp, method, path, IP, status</t>
+  </si>
+  <si>
+    <t>Winston timestamp() usa UTC por omissão, Render captura em UTC</t>
+  </si>
+  <si>
+    <t>Apenas Console transport → stdout → Render</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Formato </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>lineFormat</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> consistente com JSON para metadata</t>
+    </r>
+  </si>
+  <si>
+    <t>loginLogger loga AUTH:LOGIN_SUCCESS e AUTH:LOGIN_FAILED; onRateLimitHit loga brute-force</t>
+  </si>
+  <si>
+    <t>authorizeRoles loga SECURITY:ACCESS_DENIED e SECURITY:UNAUTHENTICATED_ACCESS</t>
+  </si>
+  <si>
+    <t>securityLogger deteta e loga XSS, SQLi, path traversal</t>
+  </si>
+  <si>
+    <t>errorHandler loga UNHANDLED_ERROR com stack; httpLogger loga 5xx como error</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -3182,6 +3226,11 @@
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial Unicode MS"/>
     </font>
   </fonts>
   <fills count="10">
@@ -3278,7 +3327,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -3350,6 +3399,9 @@
     <xf numFmtId="0" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -3357,9 +3409,7 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3813,7 +3863,7 @@
                   <c:v>0.1</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>0.25</c:v>
+                  <c:v>0.875</c:v>
                 </c:pt>
                 <c:pt idx="16">
                   <c:v>0</c:v>
@@ -4178,7 +4228,7 @@
                   <c:v>4.7619047619047616E-2</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>0.29411764705882354</c:v>
+                  <c:v>0.88235294117647056</c:v>
                 </c:pt>
                 <c:pt idx="16">
                   <c:v>0</c:v>
@@ -4694,53 +4744,53 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:P23"/>
-  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="34" customWidth="1"/>
     <col min="2" max="13" width="11" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="36" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="27" t="s">
+    <row r="1" spans="1:16" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="28" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="27"/>
-      <c r="C1" s="27"/>
-      <c r="D1" s="27"/>
-      <c r="E1" s="27"/>
-      <c r="F1" s="27"/>
-      <c r="G1" s="27"/>
-      <c r="H1" s="27"/>
-      <c r="I1" s="27"/>
-      <c r="J1" s="27"/>
-      <c r="K1" s="27"/>
-      <c r="L1" s="27"/>
-      <c r="M1" s="27"/>
-      <c r="N1" s="27"/>
-      <c r="O1" s="27"/>
-      <c r="P1" s="27"/>
-    </row>
-    <row r="2" spans="1:16" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="28"/>
-      <c r="B2" s="28"/>
-      <c r="C2" s="28"/>
-      <c r="D2" s="28"/>
-      <c r="E2" s="28"/>
-      <c r="F2" s="28"/>
-      <c r="G2" s="28"/>
-      <c r="H2" s="28"/>
-      <c r="I2" s="28"/>
-      <c r="J2" s="28"/>
-      <c r="K2" s="28"/>
-      <c r="L2" s="28"/>
-      <c r="M2" s="28"/>
-      <c r="N2" s="28"/>
-      <c r="O2" s="28"/>
-      <c r="P2" s="28"/>
-    </row>
-    <row r="3" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="29"/>
-      <c r="B3" s="29"/>
+      <c r="B1" s="28"/>
+      <c r="C1" s="28"/>
+      <c r="D1" s="28"/>
+      <c r="E1" s="28"/>
+      <c r="F1" s="28"/>
+      <c r="G1" s="28"/>
+      <c r="H1" s="28"/>
+      <c r="I1" s="28"/>
+      <c r="J1" s="28"/>
+      <c r="K1" s="28"/>
+      <c r="L1" s="28"/>
+      <c r="M1" s="28"/>
+      <c r="N1" s="28"/>
+      <c r="O1" s="28"/>
+      <c r="P1" s="28"/>
+    </row>
+    <row r="2" spans="1:16" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="29"/>
+      <c r="B2" s="29"/>
+      <c r="C2" s="29"/>
+      <c r="D2" s="29"/>
+      <c r="E2" s="29"/>
+      <c r="F2" s="29"/>
+      <c r="G2" s="29"/>
+      <c r="H2" s="29"/>
+      <c r="I2" s="29"/>
+      <c r="J2" s="29"/>
+      <c r="K2" s="29"/>
+      <c r="L2" s="29"/>
+      <c r="M2" s="29"/>
+      <c r="N2" s="29"/>
+      <c r="O2" s="29"/>
+      <c r="P2" s="29"/>
+    </row>
+    <row r="3" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="30"/>
+      <c r="B3" s="30"/>
       <c r="C3" s="1"/>
       <c r="E3" s="1"/>
       <c r="G3" s="1"/>
@@ -4749,7 +4799,7 @@
       <c r="M3" s="1"/>
       <c r="O3" s="1"/>
     </row>
-    <row r="5" spans="1:16" ht="31.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:16" ht="31.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>1</v>
       </c>
@@ -4790,7 +4840,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="6" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>14</v>
       </c>
@@ -4839,7 +4889,7 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="7" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
         <v>15</v>
       </c>
@@ -4888,7 +4938,7 @@
         <v>7.6923076923076927E-2</v>
       </c>
     </row>
-    <row r="8" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>16</v>
       </c>
@@ -4937,7 +4987,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
         <v>17</v>
       </c>
@@ -4986,7 +5036,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>18</v>
       </c>
@@ -5035,7 +5085,7 @@
         <v>0.30769230769230771</v>
       </c>
     </row>
-    <row r="11" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="6" t="s">
         <v>19</v>
       </c>
@@ -5084,7 +5134,7 @@
         <v>0.1276595744680851</v>
       </c>
     </row>
-    <row r="12" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>20</v>
       </c>
@@ -5133,7 +5183,7 @@
         <v>5.2631578947368418E-2</v>
       </c>
     </row>
-    <row r="13" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
         <v>21</v>
       </c>
@@ -5182,7 +5232,7 @@
         <v>0.23076923076923078</v>
       </c>
     </row>
-    <row r="14" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>22</v>
       </c>
@@ -5229,7 +5279,7 @@
         <v>0.42857142857142855</v>
       </c>
     </row>
-    <row r="15" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="6" t="s">
         <v>24</v>
       </c>
@@ -5278,7 +5328,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>25</v>
       </c>
@@ -5327,7 +5377,7 @@
         <v>4.1666666666666664E-2</v>
       </c>
     </row>
-    <row r="17" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="6" t="s">
         <v>26</v>
       </c>
@@ -5376,7 +5426,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
         <v>27</v>
       </c>
@@ -5425,7 +5475,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="6" t="s">
         <v>28</v>
       </c>
@@ -5474,7 +5524,7 @@
         <v>7.6923076923076927E-2</v>
       </c>
     </row>
-    <row r="20" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
         <v>29</v>
       </c>
@@ -5523,7 +5573,7 @@
         <v>4.7619047619047616E-2</v>
       </c>
     </row>
-    <row r="21" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="6" t="s">
         <v>30</v>
       </c>
@@ -5544,11 +5594,11 @@
       </c>
       <c r="G21" s="7">
         <f>COUNTIFS('V16 - Security Logging and Erro'!$F$2:$F$23,"Compliant",'V16 - Security Logging and Erro'!$E$2:$E$23,2)</f>
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="H21" s="8">
         <f t="shared" si="1"/>
-        <v>0.25</v>
+        <v>0.875</v>
       </c>
       <c r="I21" s="7">
         <v>1</v>
@@ -5563,14 +5613,14 @@
       </c>
       <c r="L21" s="7">
         <f>COUNTIF('V16 - Security Logging and Erro'!$F$2:$F$23,"Compliant")</f>
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="M21" s="8">
         <f t="shared" si="3"/>
-        <v>0.29411764705882354</v>
-      </c>
-    </row>
-    <row r="22" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+        <v>0.88235294117647056</v>
+      </c>
+    </row>
+    <row r="22" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
         <v>31</v>
       </c>
@@ -5617,7 +5667,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:13" ht="22.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:13" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="9" t="s">
         <v>32</v>
       </c>
@@ -5643,11 +5693,11 @@
       </c>
       <c r="G23" s="10">
         <f>SUM(G6:G22)</f>
-        <v>7</v>
+        <v>17</v>
       </c>
       <c r="H23" s="11">
         <f>IFERROR(AVERAGE(H6:H22),"")</f>
-        <v>2.5935828877005348E-2</v>
+        <v>6.2700534759358287E-2</v>
       </c>
       <c r="I23" s="10">
         <f>SUM(I6:I22)</f>
@@ -5663,11 +5713,11 @@
       </c>
       <c r="L23" s="10">
         <f>SUM(L6:L22)</f>
-        <v>29</v>
+        <v>39</v>
       </c>
       <c r="M23" s="11">
         <f>IFERROR(AVERAGE(M6:M22),"")</f>
-        <v>0.1049749197434772</v>
+        <v>0.13957699586804467</v>
       </c>
     </row>
   </sheetData>
@@ -5733,7 +5783,7 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
   <dimension ref="A1:H10"/>
-  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
@@ -5745,7 +5795,7 @@
     <col min="8" max="8" width="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="28.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:8" ht="28.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="12" t="s">
         <v>33</v>
       </c>
@@ -5771,7 +5821,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="13" t="s">
         <v>490</v>
       </c>
@@ -5785,7 +5835,7 @@
       <c r="G2" s="13"/>
       <c r="H2" s="13"/>
     </row>
-    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
         <v>490</v>
       </c>
@@ -5811,7 +5861,7 @@
         <v>1007</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="19" t="s">
         <v>490</v>
       </c>
@@ -5837,7 +5887,7 @@
         <v>1007</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
         <v>490</v>
       </c>
@@ -5859,7 +5909,7 @@
       <c r="G5" s="16"/>
       <c r="H5" s="16"/>
     </row>
-    <row r="6" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="13" t="s">
         <v>498</v>
       </c>
@@ -5873,7 +5923,7 @@
       <c r="G6" s="13"/>
       <c r="H6" s="13"/>
     </row>
-    <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="14" t="s">
         <v>498</v>
       </c>
@@ -5895,7 +5945,7 @@
       <c r="G7" s="16"/>
       <c r="H7" s="16"/>
     </row>
-    <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="19" t="s">
         <v>498</v>
       </c>
@@ -5919,7 +5969,7 @@
         <v>910</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="14" t="s">
         <v>498</v>
       </c>
@@ -5943,7 +5993,7 @@
         <v>916</v>
       </c>
     </row>
-    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="19" t="s">
         <v>498</v>
       </c>
@@ -5993,7 +6043,7 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
   <dimension ref="A1:H44"/>
-  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
@@ -6005,7 +6055,7 @@
     <col min="8" max="8" width="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="28.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:8" ht="28.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="12" t="s">
         <v>33</v>
       </c>
@@ -6031,7 +6081,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="13" t="s">
         <v>508</v>
       </c>
@@ -6045,7 +6095,7 @@
       <c r="G2" s="13"/>
       <c r="H2" s="13"/>
     </row>
-    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
         <v>508</v>
       </c>
@@ -6069,7 +6119,7 @@
         <v>910</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="19" t="s">
         <v>508</v>
       </c>
@@ -6093,7 +6143,7 @@
         <v>928</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="13" t="s">
         <v>514</v>
       </c>
@@ -6107,7 +6157,7 @@
       <c r="G5" s="13"/>
       <c r="H5" s="13"/>
     </row>
-    <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="14" t="s">
         <v>514</v>
       </c>
@@ -6131,7 +6181,7 @@
         <v>921</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="19" t="s">
         <v>514</v>
       </c>
@@ -6155,7 +6205,7 @@
         <v>910</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="14" t="s">
         <v>514</v>
       </c>
@@ -6177,7 +6227,7 @@
       <c r="G8" s="16"/>
       <c r="H8" s="16"/>
     </row>
-    <row r="9" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="13" t="s">
         <v>522</v>
       </c>
@@ -6191,7 +6241,7 @@
       <c r="G9" s="13"/>
       <c r="H9" s="13"/>
     </row>
-    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="14" t="s">
         <v>522</v>
       </c>
@@ -6215,7 +6265,7 @@
         <v>916</v>
       </c>
     </row>
-    <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="19" t="s">
         <v>522</v>
       </c>
@@ -6239,7 +6289,7 @@
         <v>916</v>
       </c>
     </row>
-    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="14" t="s">
         <v>522</v>
       </c>
@@ -6263,7 +6313,7 @@
         <v>929</v>
       </c>
     </row>
-    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="19" t="s">
         <v>522</v>
       </c>
@@ -6287,7 +6337,7 @@
         <v>916</v>
       </c>
     </row>
-    <row r="14" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="14" t="s">
         <v>522</v>
       </c>
@@ -6309,7 +6359,7 @@
       <c r="G14" s="16"/>
       <c r="H14" s="16"/>
     </row>
-    <row r="15" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="13" t="s">
         <v>534</v>
       </c>
@@ -6323,7 +6373,7 @@
       <c r="G15" s="13"/>
       <c r="H15" s="13"/>
     </row>
-    <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="14" t="s">
         <v>534</v>
       </c>
@@ -6345,7 +6395,7 @@
       <c r="G16" s="16"/>
       <c r="H16" s="16"/>
     </row>
-    <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="19" t="s">
         <v>534</v>
       </c>
@@ -6367,7 +6417,7 @@
       <c r="G17" s="21"/>
       <c r="H17" s="21"/>
     </row>
-    <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="14" t="s">
         <v>534</v>
       </c>
@@ -6389,7 +6439,7 @@
       <c r="G18" s="16"/>
       <c r="H18" s="16"/>
     </row>
-    <row r="19" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="19" t="s">
         <v>534</v>
       </c>
@@ -6411,7 +6461,7 @@
       <c r="G19" s="21"/>
       <c r="H19" s="21"/>
     </row>
-    <row r="20" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="14" t="s">
         <v>534</v>
       </c>
@@ -6433,7 +6483,7 @@
       <c r="G20" s="16"/>
       <c r="H20" s="16"/>
     </row>
-    <row r="21" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="19" t="s">
         <v>534</v>
       </c>
@@ -6457,7 +6507,7 @@
         <v>921</v>
       </c>
     </row>
-    <row r="22" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="14" t="s">
         <v>534</v>
       </c>
@@ -6481,7 +6531,7 @@
         <v>930</v>
       </c>
     </row>
-    <row r="23" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="19" t="s">
         <v>534</v>
       </c>
@@ -6505,7 +6555,7 @@
         <v>931</v>
       </c>
     </row>
-    <row r="24" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="14" t="s">
         <v>534</v>
       </c>
@@ -6529,7 +6579,7 @@
         <v>925</v>
       </c>
     </row>
-    <row r="25" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="19" t="s">
         <v>534</v>
       </c>
@@ -6553,7 +6603,7 @@
         <v>916</v>
       </c>
     </row>
-    <row r="26" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="14" t="s">
         <v>534</v>
       </c>
@@ -6577,7 +6627,7 @@
         <v>903</v>
       </c>
     </row>
-    <row r="27" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="19" t="s">
         <v>534</v>
       </c>
@@ -6599,7 +6649,7 @@
       <c r="G27" s="21"/>
       <c r="H27" s="21"/>
     </row>
-    <row r="28" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="14" t="s">
         <v>534</v>
       </c>
@@ -6621,7 +6671,7 @@
       <c r="G28" s="16"/>
       <c r="H28" s="16"/>
     </row>
-    <row r="29" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="19" t="s">
         <v>534</v>
       </c>
@@ -6643,7 +6693,7 @@
       <c r="G29" s="21"/>
       <c r="H29" s="21"/>
     </row>
-    <row r="30" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="14" t="s">
         <v>534</v>
       </c>
@@ -6665,7 +6715,7 @@
       <c r="G30" s="16"/>
       <c r="H30" s="16"/>
     </row>
-    <row r="31" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="19" t="s">
         <v>534</v>
       </c>
@@ -6687,7 +6737,7 @@
       <c r="G31" s="21"/>
       <c r="H31" s="21"/>
     </row>
-    <row r="32" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="13" t="s">
         <v>568</v>
       </c>
@@ -6701,7 +6751,7 @@
       <c r="G32" s="13"/>
       <c r="H32" s="13"/>
     </row>
-    <row r="33" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="14" t="s">
         <v>568</v>
       </c>
@@ -6725,7 +6775,7 @@
         <v>919</v>
       </c>
     </row>
-    <row r="34" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="19" t="s">
         <v>568</v>
       </c>
@@ -6749,7 +6799,7 @@
         <v>929</v>
       </c>
     </row>
-    <row r="35" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="14" t="s">
         <v>568</v>
       </c>
@@ -6773,7 +6823,7 @@
         <v>910</v>
       </c>
     </row>
-    <row r="36" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="19" t="s">
         <v>568</v>
       </c>
@@ -6797,7 +6847,7 @@
         <v>916</v>
       </c>
     </row>
-    <row r="37" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="14" t="s">
         <v>568</v>
       </c>
@@ -6821,7 +6871,7 @@
         <v>919</v>
       </c>
     </row>
-    <row r="38" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="13" t="s">
         <v>580</v>
       </c>
@@ -6835,7 +6885,7 @@
       <c r="G38" s="13"/>
       <c r="H38" s="13"/>
     </row>
-    <row r="39" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="14" t="s">
         <v>580</v>
       </c>
@@ -6859,7 +6909,7 @@
         <v>928</v>
       </c>
     </row>
-    <row r="40" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="19" t="s">
         <v>580</v>
       </c>
@@ -6883,7 +6933,7 @@
         <v>927</v>
       </c>
     </row>
-    <row r="41" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="13" t="s">
         <v>586</v>
       </c>
@@ -6897,7 +6947,7 @@
       <c r="G41" s="13"/>
       <c r="H41" s="13"/>
     </row>
-    <row r="42" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="14" t="s">
         <v>586</v>
       </c>
@@ -6921,7 +6971,7 @@
         <v>903</v>
       </c>
     </row>
-    <row r="43" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="19" t="s">
         <v>586</v>
       </c>
@@ -6945,7 +6995,7 @@
         <v>932</v>
       </c>
     </row>
-    <row r="44" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="14" t="s">
         <v>586</v>
       </c>
@@ -6995,7 +7045,7 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0B00-000000000000}">
   <dimension ref="A1:H32"/>
-  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
@@ -7007,7 +7057,7 @@
     <col min="8" max="8" width="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="28.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:8" ht="28.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="12" t="s">
         <v>33</v>
       </c>
@@ -7033,7 +7083,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="13" t="s">
         <v>594</v>
       </c>
@@ -7047,7 +7097,7 @@
       <c r="G2" s="13"/>
       <c r="H2" s="13"/>
     </row>
-    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
         <v>594</v>
       </c>
@@ -7071,7 +7121,7 @@
         <v>933</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="19" t="s">
         <v>594</v>
       </c>
@@ -7095,7 +7145,7 @@
         <v>934</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
         <v>594</v>
       </c>
@@ -7117,7 +7167,7 @@
       <c r="G5" s="16"/>
       <c r="H5" s="16"/>
     </row>
-    <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="19" t="s">
         <v>594</v>
       </c>
@@ -7139,7 +7189,7 @@
       <c r="G6" s="21"/>
       <c r="H6" s="21"/>
     </row>
-    <row r="7" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="13" t="s">
         <v>604</v>
       </c>
@@ -7153,7 +7203,7 @@
       <c r="G7" s="13"/>
       <c r="H7" s="13"/>
     </row>
-    <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="14" t="s">
         <v>604</v>
       </c>
@@ -7177,7 +7227,7 @@
         <v>934</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="19" t="s">
         <v>604</v>
       </c>
@@ -7201,7 +7251,7 @@
         <v>934</v>
       </c>
     </row>
-    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="14" t="s">
         <v>604</v>
       </c>
@@ -7225,7 +7275,7 @@
         <v>934</v>
       </c>
     </row>
-    <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="19" t="s">
         <v>604</v>
       </c>
@@ -7247,7 +7297,7 @@
       <c r="G11" s="21"/>
       <c r="H11" s="21"/>
     </row>
-    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="14" t="s">
         <v>604</v>
       </c>
@@ -7269,7 +7319,7 @@
       <c r="G12" s="16"/>
       <c r="H12" s="16"/>
     </row>
-    <row r="13" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="13" t="s">
         <v>616</v>
       </c>
@@ -7283,7 +7333,7 @@
       <c r="G13" s="13"/>
       <c r="H13" s="13"/>
     </row>
-    <row r="14" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="14" t="s">
         <v>616</v>
       </c>
@@ -7305,7 +7355,7 @@
       <c r="G14" s="16"/>
       <c r="H14" s="16"/>
     </row>
-    <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="19" t="s">
         <v>616</v>
       </c>
@@ -7327,7 +7377,7 @@
       <c r="G15" s="21"/>
       <c r="H15" s="21"/>
     </row>
-    <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="14" t="s">
         <v>616</v>
       </c>
@@ -7351,7 +7401,7 @@
         <v>904</v>
       </c>
     </row>
-    <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="19" t="s">
         <v>616</v>
       </c>
@@ -7373,7 +7423,7 @@
       <c r="G17" s="21"/>
       <c r="H17" s="21"/>
     </row>
-    <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="14" t="s">
         <v>616</v>
       </c>
@@ -7395,7 +7445,7 @@
       <c r="G18" s="16"/>
       <c r="H18" s="16"/>
     </row>
-    <row r="19" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="13" t="s">
         <v>628</v>
       </c>
@@ -7409,7 +7459,7 @@
       <c r="G19" s="13"/>
       <c r="H19" s="13"/>
     </row>
-    <row r="20" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="14" t="s">
         <v>628</v>
       </c>
@@ -7431,7 +7481,7 @@
       <c r="G20" s="16"/>
       <c r="H20" s="16"/>
     </row>
-    <row r="21" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="19" t="s">
         <v>628</v>
       </c>
@@ -7455,7 +7505,7 @@
         <v>935</v>
       </c>
     </row>
-    <row r="22" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="14" t="s">
         <v>628</v>
       </c>
@@ -7479,7 +7529,7 @@
         <v>936</v>
       </c>
     </row>
-    <row r="23" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="19" t="s">
         <v>628</v>
       </c>
@@ -7503,7 +7553,7 @@
         <v>935</v>
       </c>
     </row>
-    <row r="24" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="13" t="s">
         <v>638</v>
       </c>
@@ -7517,7 +7567,7 @@
       <c r="G24" s="13"/>
       <c r="H24" s="13"/>
     </row>
-    <row r="25" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="14" t="s">
         <v>638</v>
       </c>
@@ -7541,7 +7591,7 @@
         <v>918</v>
       </c>
     </row>
-    <row r="26" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="19" t="s">
         <v>638</v>
       </c>
@@ -7563,7 +7613,7 @@
       <c r="G26" s="21"/>
       <c r="H26" s="21"/>
     </row>
-    <row r="27" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="13" t="s">
         <v>644</v>
       </c>
@@ -7577,7 +7627,7 @@
       <c r="G27" s="13"/>
       <c r="H27" s="13"/>
     </row>
-    <row r="28" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="14" t="s">
         <v>644</v>
       </c>
@@ -7601,7 +7651,7 @@
         <v>934</v>
       </c>
     </row>
-    <row r="29" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="19" t="s">
         <v>644</v>
       </c>
@@ -7623,7 +7673,7 @@
       <c r="G29" s="21"/>
       <c r="H29" s="21"/>
     </row>
-    <row r="30" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="13" t="s">
         <v>650</v>
       </c>
@@ -7637,7 +7687,7 @@
       <c r="G30" s="13"/>
       <c r="H30" s="13"/>
     </row>
-    <row r="31" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="14" t="s">
         <v>650</v>
       </c>
@@ -7659,7 +7709,7 @@
       <c r="G31" s="16"/>
       <c r="H31" s="16"/>
     </row>
-    <row r="32" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="19" t="s">
         <v>650</v>
       </c>
@@ -7707,7 +7757,7 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0C00-000000000000}">
   <dimension ref="A1:H16"/>
-  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
@@ -7719,7 +7769,7 @@
     <col min="8" max="8" width="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="28.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:8" ht="28.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="12" t="s">
         <v>33</v>
       </c>
@@ -7745,7 +7795,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="13" t="s">
         <v>656</v>
       </c>
@@ -7759,7 +7809,7 @@
       <c r="G2" s="13"/>
       <c r="H2" s="13"/>
     </row>
-    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
         <v>656</v>
       </c>
@@ -7781,7 +7831,7 @@
       <c r="G3" s="16"/>
       <c r="H3" s="16"/>
     </row>
-    <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="19" t="s">
         <v>656</v>
       </c>
@@ -7805,7 +7855,7 @@
         <v>937</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
         <v>656</v>
       </c>
@@ -7829,7 +7879,7 @@
         <v>938</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="19" t="s">
         <v>656</v>
       </c>
@@ -7851,7 +7901,7 @@
       <c r="G6" s="21"/>
       <c r="H6" s="21"/>
     </row>
-    <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="14" t="s">
         <v>656</v>
       </c>
@@ -7873,7 +7923,7 @@
       <c r="G7" s="16"/>
       <c r="H7" s="16"/>
     </row>
-    <row r="8" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="13" t="s">
         <v>668</v>
       </c>
@@ -7887,7 +7937,7 @@
       <c r="G8" s="13"/>
       <c r="H8" s="13"/>
     </row>
-    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="14" t="s">
         <v>668</v>
       </c>
@@ -7909,7 +7959,7 @@
       <c r="G9" s="16"/>
       <c r="H9" s="16"/>
     </row>
-    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="19" t="s">
         <v>668</v>
       </c>
@@ -7931,7 +7981,7 @@
       <c r="G10" s="21"/>
       <c r="H10" s="21"/>
     </row>
-    <row r="11" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="13" t="s">
         <v>674</v>
       </c>
@@ -7945,7 +7995,7 @@
       <c r="G11" s="13"/>
       <c r="H11" s="13"/>
     </row>
-    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="14" t="s">
         <v>674</v>
       </c>
@@ -7969,7 +8019,7 @@
         <v>937</v>
       </c>
     </row>
-    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="19" t="s">
         <v>674</v>
       </c>
@@ -7993,7 +8043,7 @@
         <v>939</v>
       </c>
     </row>
-    <row r="14" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="14" t="s">
         <v>674</v>
       </c>
@@ -8017,7 +8067,7 @@
         <v>937</v>
       </c>
     </row>
-    <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="19" t="s">
         <v>674</v>
       </c>
@@ -8041,7 +8091,7 @@
         <v>940</v>
       </c>
     </row>
-    <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="14" t="s">
         <v>674</v>
       </c>
@@ -8089,7 +8139,7 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0D00-000000000000}">
   <dimension ref="A1:H26"/>
-  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
@@ -8101,7 +8151,7 @@
     <col min="8" max="8" width="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="28.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:8" ht="28.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="12" t="s">
         <v>33</v>
       </c>
@@ -8127,7 +8177,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="13" t="s">
         <v>686</v>
       </c>
@@ -8141,7 +8191,7 @@
       <c r="G2" s="13"/>
       <c r="H2" s="13"/>
     </row>
-    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
         <v>686</v>
       </c>
@@ -8165,7 +8215,7 @@
         <v>941</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="19" t="s">
         <v>686</v>
       </c>
@@ -8187,7 +8237,7 @@
       <c r="G4" s="21"/>
       <c r="H4" s="21"/>
     </row>
-    <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
         <v>686</v>
       </c>
@@ -8209,7 +8259,7 @@
       <c r="G5" s="16"/>
       <c r="H5" s="16"/>
     </row>
-    <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="19" t="s">
         <v>686</v>
       </c>
@@ -8231,7 +8281,7 @@
       <c r="G6" s="21"/>
       <c r="H6" s="21"/>
     </row>
-    <row r="7" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="13" t="s">
         <v>696</v>
       </c>
@@ -8245,7 +8295,7 @@
       <c r="G7" s="13"/>
       <c r="H7" s="13"/>
     </row>
-    <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="14" t="s">
         <v>696</v>
       </c>
@@ -8269,7 +8319,7 @@
         <v>942</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="19" t="s">
         <v>696</v>
       </c>
@@ -8293,7 +8343,7 @@
         <v>901</v>
       </c>
     </row>
-    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="14" t="s">
         <v>696</v>
       </c>
@@ -8317,7 +8367,7 @@
         <v>943</v>
       </c>
     </row>
-    <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="19" t="s">
         <v>696</v>
       </c>
@@ -8341,7 +8391,7 @@
         <v>944</v>
       </c>
     </row>
-    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="14" t="s">
         <v>696</v>
       </c>
@@ -8365,7 +8415,7 @@
         <v>945</v>
       </c>
     </row>
-    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="19" t="s">
         <v>696</v>
       </c>
@@ -8387,7 +8437,7 @@
       <c r="G13" s="21"/>
       <c r="H13" s="21"/>
     </row>
-    <row r="14" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="13" t="s">
         <v>710</v>
       </c>
@@ -8401,7 +8451,7 @@
       <c r="G14" s="13"/>
       <c r="H14" s="13"/>
     </row>
-    <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="14" t="s">
         <v>710</v>
       </c>
@@ -8425,7 +8475,7 @@
         <v>946</v>
       </c>
     </row>
-    <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="19" t="s">
         <v>710</v>
       </c>
@@ -8449,7 +8499,7 @@
         <v>947</v>
       </c>
     </row>
-    <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="14" t="s">
         <v>710</v>
       </c>
@@ -8471,7 +8521,7 @@
       <c r="G17" s="16"/>
       <c r="H17" s="16"/>
     </row>
-    <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="19" t="s">
         <v>710</v>
       </c>
@@ -8493,7 +8543,7 @@
       <c r="G18" s="21"/>
       <c r="H18" s="21"/>
     </row>
-    <row r="19" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="13" t="s">
         <v>720</v>
       </c>
@@ -8507,7 +8557,7 @@
       <c r="G19" s="13"/>
       <c r="H19" s="13"/>
     </row>
-    <row r="20" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="14" t="s">
         <v>720</v>
       </c>
@@ -8529,7 +8579,7 @@
       <c r="G20" s="16"/>
       <c r="H20" s="16"/>
     </row>
-    <row r="21" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="19" t="s">
         <v>720</v>
       </c>
@@ -8553,7 +8603,7 @@
         <v>934</v>
       </c>
     </row>
-    <row r="22" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="14" t="s">
         <v>720</v>
       </c>
@@ -8577,7 +8627,7 @@
         <v>948</v>
       </c>
     </row>
-    <row r="23" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="19" t="s">
         <v>720</v>
       </c>
@@ -8601,7 +8651,7 @@
         <v>949</v>
       </c>
     </row>
-    <row r="24" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="14" t="s">
         <v>720</v>
       </c>
@@ -8625,7 +8675,7 @@
         <v>950</v>
       </c>
     </row>
-    <row r="25" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="19" t="s">
         <v>720</v>
       </c>
@@ -8647,7 +8697,7 @@
       <c r="G25" s="21"/>
       <c r="H25" s="21"/>
     </row>
-    <row r="26" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="14" t="s">
         <v>720</v>
       </c>
@@ -8695,7 +8745,7 @@
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0E00-000000000000}">
   <dimension ref="A1:H17"/>
-  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
@@ -8707,7 +8757,7 @@
     <col min="8" max="8" width="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="28.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:8" ht="28.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="12" t="s">
         <v>33</v>
       </c>
@@ -8733,7 +8783,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="13" t="s">
         <v>736</v>
       </c>
@@ -8747,7 +8797,7 @@
       <c r="G2" s="13"/>
       <c r="H2" s="13"/>
     </row>
-    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
         <v>736</v>
       </c>
@@ -8771,7 +8821,7 @@
         <v>941</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="19" t="s">
         <v>736</v>
       </c>
@@ -8795,7 +8845,7 @@
         <v>951</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="13" t="s">
         <v>742</v>
       </c>
@@ -8809,7 +8859,7 @@
       <c r="G5" s="13"/>
       <c r="H5" s="13"/>
     </row>
-    <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="14" t="s">
         <v>742</v>
       </c>
@@ -8835,7 +8885,7 @@
         <v>1003</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="19" t="s">
         <v>742</v>
       </c>
@@ -8859,7 +8909,7 @@
         <v>952</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="14" t="s">
         <v>742</v>
       </c>
@@ -8883,7 +8933,7 @@
         <v>953</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="19" t="s">
         <v>742</v>
       </c>
@@ -8907,7 +8957,7 @@
         <v>954</v>
       </c>
     </row>
-    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="14" t="s">
         <v>742</v>
       </c>
@@ -8929,7 +8979,7 @@
       <c r="G10" s="16"/>
       <c r="H10" s="16"/>
     </row>
-    <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="19" t="s">
         <v>742</v>
       </c>
@@ -8951,7 +9001,7 @@
       <c r="G11" s="21"/>
       <c r="H11" s="21"/>
     </row>
-    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="14" t="s">
         <v>742</v>
       </c>
@@ -8973,7 +9023,7 @@
       <c r="G12" s="16"/>
       <c r="H12" s="16"/>
     </row>
-    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="19" t="s">
         <v>742</v>
       </c>
@@ -8995,7 +9045,7 @@
       <c r="G13" s="21"/>
       <c r="H13" s="21"/>
     </row>
-    <row r="14" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="13" t="s">
         <v>760</v>
       </c>
@@ -9009,7 +9059,7 @@
       <c r="G14" s="13"/>
       <c r="H14" s="13"/>
     </row>
-    <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="14" t="s">
         <v>760</v>
       </c>
@@ -9031,7 +9081,7 @@
       <c r="G15" s="16"/>
       <c r="H15" s="16"/>
     </row>
-    <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="19" t="s">
         <v>760</v>
       </c>
@@ -9055,7 +9105,7 @@
         <v>955</v>
       </c>
     </row>
-    <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="14" t="s">
         <v>760</v>
       </c>
@@ -9105,7 +9155,7 @@
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0F00-000000000000}">
   <dimension ref="A1:H26"/>
-  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
@@ -9117,7 +9167,7 @@
     <col min="8" max="8" width="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="28.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:8" ht="28.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="12" t="s">
         <v>33</v>
       </c>
@@ -9143,7 +9193,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="13" t="s">
         <v>768</v>
       </c>
@@ -9157,7 +9207,7 @@
       <c r="G2" s="13"/>
       <c r="H2" s="13"/>
     </row>
-    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
         <v>768</v>
       </c>
@@ -9179,7 +9229,7 @@
       <c r="G3" s="16"/>
       <c r="H3" s="16"/>
     </row>
-    <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="19" t="s">
         <v>768</v>
       </c>
@@ -9203,7 +9253,7 @@
         <v>957</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
         <v>768</v>
       </c>
@@ -9227,7 +9277,7 @@
         <v>958</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="19" t="s">
         <v>768</v>
       </c>
@@ -9249,7 +9299,7 @@
       <c r="G6" s="21"/>
       <c r="H6" s="21"/>
     </row>
-    <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="14" t="s">
         <v>768</v>
       </c>
@@ -9271,7 +9321,7 @@
       <c r="G7" s="16"/>
       <c r="H7" s="16"/>
     </row>
-    <row r="8" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="13" t="s">
         <v>780</v>
       </c>
@@ -9285,7 +9335,7 @@
       <c r="G8" s="13"/>
       <c r="H8" s="13"/>
     </row>
-    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="14" t="s">
         <v>780</v>
       </c>
@@ -9307,7 +9357,7 @@
       <c r="G9" s="16"/>
       <c r="H9" s="16"/>
     </row>
-    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="19" t="s">
         <v>780</v>
       </c>
@@ -9333,7 +9383,7 @@
         <v>997</v>
       </c>
     </row>
-    <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="14" t="s">
         <v>780</v>
       </c>
@@ -9357,7 +9407,7 @@
         <v>959</v>
       </c>
     </row>
-    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="19" t="s">
         <v>780</v>
       </c>
@@ -9379,7 +9429,7 @@
       <c r="G12" s="26"/>
       <c r="H12" s="21"/>
     </row>
-    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="14" t="s">
         <v>780</v>
       </c>
@@ -9401,7 +9451,7 @@
       <c r="G13" s="16"/>
       <c r="H13" s="16"/>
     </row>
-    <row r="14" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="13" t="s">
         <v>792</v>
       </c>
@@ -9415,7 +9465,7 @@
       <c r="G14" s="13"/>
       <c r="H14" s="13"/>
     </row>
-    <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="14" t="s">
         <v>792</v>
       </c>
@@ -9437,7 +9487,7 @@
       <c r="G15" s="16"/>
       <c r="H15" s="16"/>
     </row>
-    <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="19" t="s">
         <v>792</v>
       </c>
@@ -9461,7 +9511,7 @@
         <v>960</v>
       </c>
     </row>
-    <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="14" t="s">
         <v>792</v>
       </c>
@@ -9485,7 +9535,7 @@
         <v>961</v>
       </c>
     </row>
-    <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="19" t="s">
         <v>792</v>
       </c>
@@ -9509,7 +9559,7 @@
         <v>962</v>
       </c>
     </row>
-    <row r="19" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="14" t="s">
         <v>792</v>
       </c>
@@ -9533,7 +9583,7 @@
         <v>963</v>
       </c>
     </row>
-    <row r="20" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="19" t="s">
         <v>792</v>
       </c>
@@ -9557,7 +9607,7 @@
         <v>963</v>
       </c>
     </row>
-    <row r="21" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="14" t="s">
         <v>792</v>
       </c>
@@ -9581,7 +9631,7 @@
         <v>964</v>
       </c>
     </row>
-    <row r="22" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="13" t="s">
         <v>808</v>
       </c>
@@ -9595,7 +9645,7 @@
       <c r="G22" s="13"/>
       <c r="H22" s="13"/>
     </row>
-    <row r="23" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="14" t="s">
         <v>808</v>
       </c>
@@ -9617,7 +9667,7 @@
       <c r="G23" s="16"/>
       <c r="H23" s="16"/>
     </row>
-    <row r="24" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="19" t="s">
         <v>808</v>
       </c>
@@ -9639,7 +9689,7 @@
       <c r="G24" s="21"/>
       <c r="H24" s="21"/>
     </row>
-    <row r="25" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="14" t="s">
         <v>808</v>
       </c>
@@ -9661,7 +9711,7 @@
       <c r="G25" s="16"/>
       <c r="H25" s="16"/>
     </row>
-    <row r="26" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="19" t="s">
         <v>808</v>
       </c>
@@ -9709,7 +9759,7 @@
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1000-000000000000}">
   <dimension ref="A1:M26"/>
-  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
@@ -9721,7 +9771,7 @@
     <col min="8" max="8" width="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="28.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:13" ht="28.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="12" t="s">
         <v>33</v>
       </c>
@@ -9747,7 +9797,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="13" t="s">
         <v>818</v>
       </c>
@@ -9761,7 +9811,7 @@
       <c r="G2" s="13"/>
       <c r="H2" s="13"/>
     </row>
-    <row r="3" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
         <v>818</v>
       </c>
@@ -9778,14 +9828,14 @@
         <v>2</v>
       </c>
       <c r="F3" s="18" t="s">
-        <v>45</v>
+        <v>981</v>
       </c>
       <c r="G3" s="16"/>
       <c r="H3" s="16" t="s">
         <v>965</v>
       </c>
     </row>
-    <row r="4" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="13" t="s">
         <v>822</v>
       </c>
@@ -9799,7 +9849,7 @@
       <c r="G4" s="13"/>
       <c r="H4" s="13"/>
     </row>
-    <row r="5" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
         <v>822</v>
       </c>
@@ -9816,14 +9866,16 @@
         <v>2</v>
       </c>
       <c r="F5" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G5" s="16"/>
+        <v>981</v>
+      </c>
+      <c r="G5" s="16" t="s">
+        <v>1013</v>
+      </c>
       <c r="H5" s="16" t="s">
         <v>966</v>
       </c>
     </row>
-    <row r="6" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="19" t="s">
         <v>822</v>
       </c>
@@ -9840,15 +9892,17 @@
         <v>2</v>
       </c>
       <c r="F6" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G6" s="21"/>
+        <v>981</v>
+      </c>
+      <c r="G6" s="21" t="s">
+        <v>1014</v>
+      </c>
       <c r="H6" s="21" t="s">
         <v>967</v>
       </c>
       <c r="M6" s="25"/>
     </row>
-    <row r="7" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="14" t="s">
         <v>822</v>
       </c>
@@ -9865,14 +9919,16 @@
         <v>2</v>
       </c>
       <c r="F7" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G7" s="16"/>
+        <v>981</v>
+      </c>
+      <c r="G7" s="16" t="s">
+        <v>1015</v>
+      </c>
       <c r="H7" s="16" t="s">
         <v>968</v>
       </c>
     </row>
-    <row r="8" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="19" t="s">
         <v>822</v>
       </c>
@@ -9889,14 +9945,16 @@
         <v>2</v>
       </c>
       <c r="F8" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G8" s="21"/>
+        <v>981</v>
+      </c>
+      <c r="G8" t="s">
+        <v>1016</v>
+      </c>
       <c r="H8" s="21" t="s">
         <v>966</v>
       </c>
     </row>
-    <row r="9" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="14" t="s">
         <v>822</v>
       </c>
@@ -9913,7 +9971,7 @@
         <v>2</v>
       </c>
       <c r="F9" s="18" t="s">
-        <v>45</v>
+        <v>981</v>
       </c>
       <c r="G9" s="16" t="s">
         <v>1011</v>
@@ -9922,7 +9980,7 @@
         <v>1012</v>
       </c>
     </row>
-    <row r="10" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="13" t="s">
         <v>834</v>
       </c>
@@ -9936,7 +9994,7 @@
       <c r="G10" s="13"/>
       <c r="H10" s="13"/>
     </row>
-    <row r="11" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="14" t="s">
         <v>834</v>
       </c>
@@ -9953,14 +10011,16 @@
         <v>2</v>
       </c>
       <c r="F11" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G11" s="16"/>
+        <v>981</v>
+      </c>
+      <c r="G11" s="31" t="s">
+        <v>1017</v>
+      </c>
       <c r="H11" s="16" t="s">
         <v>969</v>
       </c>
     </row>
-    <row r="12" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="19" t="s">
         <v>834</v>
       </c>
@@ -9977,14 +10037,16 @@
         <v>2</v>
       </c>
       <c r="F12" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G12" s="21"/>
+        <v>981</v>
+      </c>
+      <c r="G12" s="21" t="s">
+        <v>1018</v>
+      </c>
       <c r="H12" s="21" t="s">
         <v>970</v>
       </c>
     </row>
-    <row r="13" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="14" t="s">
         <v>834</v>
       </c>
@@ -10001,14 +10063,16 @@
         <v>2</v>
       </c>
       <c r="F13" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G13" s="16"/>
+        <v>981</v>
+      </c>
+      <c r="G13" s="16" t="s">
+        <v>1019</v>
+      </c>
       <c r="H13" s="16" t="s">
         <v>971</v>
       </c>
     </row>
-    <row r="14" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="19" t="s">
         <v>834</v>
       </c>
@@ -10025,14 +10089,16 @@
         <v>2</v>
       </c>
       <c r="F14" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G14" s="21"/>
+        <v>981</v>
+      </c>
+      <c r="G14" s="21" t="s">
+        <v>1020</v>
+      </c>
       <c r="H14" s="21" t="s">
         <v>972</v>
       </c>
     </row>
-    <row r="15" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="13" t="s">
         <v>844</v>
       </c>
@@ -10046,7 +10112,7 @@
       <c r="G15" s="13"/>
       <c r="H15" s="13"/>
     </row>
-    <row r="16" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="14" t="s">
         <v>844</v>
       </c>
@@ -10070,7 +10136,7 @@
         <v>996</v>
       </c>
     </row>
-    <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="19" t="s">
         <v>844</v>
       </c>
@@ -10094,7 +10160,7 @@
         <v>973</v>
       </c>
     </row>
-    <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="14" t="s">
         <v>844</v>
       </c>
@@ -10118,7 +10184,7 @@
         <v>972</v>
       </c>
     </row>
-    <row r="19" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="13" t="s">
         <v>852</v>
       </c>
@@ -10132,7 +10198,7 @@
       <c r="G19" s="13"/>
       <c r="H19" s="13"/>
     </row>
-    <row r="20" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="14" t="s">
         <v>852</v>
       </c>
@@ -10158,7 +10224,7 @@
         <v>994</v>
       </c>
     </row>
-    <row r="21" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="19" t="s">
         <v>852</v>
       </c>
@@ -10184,7 +10250,7 @@
         <v>993</v>
       </c>
     </row>
-    <row r="22" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="14" t="s">
         <v>852</v>
       </c>
@@ -10210,7 +10276,7 @@
         <v>974</v>
       </c>
     </row>
-    <row r="23" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="19" t="s">
         <v>852</v>
       </c>
@@ -10236,10 +10302,10 @@
         <v>995</v>
       </c>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="G25" s="25"/>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="G26" s="25"/>
     </row>
   </sheetData>
@@ -10268,7 +10334,7 @@
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1100-000000000000}">
   <dimension ref="A1:H16"/>
-  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
@@ -10280,7 +10346,7 @@
     <col min="8" max="8" width="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="28.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:8" ht="28.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="12" t="s">
         <v>33</v>
       </c>
@@ -10306,7 +10372,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="13" t="s">
         <v>862</v>
       </c>
@@ -10320,7 +10386,7 @@
       <c r="G2" s="13"/>
       <c r="H2" s="13"/>
     </row>
-    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
         <v>862</v>
       </c>
@@ -10344,7 +10410,7 @@
         <v>975</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="19" t="s">
         <v>862</v>
       </c>
@@ -10366,7 +10432,7 @@
       <c r="G4" s="21"/>
       <c r="H4" s="21"/>
     </row>
-    <row r="5" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="13" t="s">
         <v>868</v>
       </c>
@@ -10380,7 +10446,7 @@
       <c r="G5" s="13"/>
       <c r="H5" s="13"/>
     </row>
-    <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="14" t="s">
         <v>868</v>
       </c>
@@ -10404,7 +10470,7 @@
         <v>976</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="19" t="s">
         <v>868</v>
       </c>
@@ -10428,7 +10494,7 @@
         <v>977</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="14" t="s">
         <v>868</v>
       </c>
@@ -10452,7 +10518,7 @@
         <v>978</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="19" t="s">
         <v>868</v>
       </c>
@@ -10476,7 +10542,7 @@
         <v>971</v>
       </c>
     </row>
-    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="14" t="s">
         <v>868</v>
       </c>
@@ -10498,7 +10564,7 @@
       <c r="G10" s="16"/>
       <c r="H10" s="16"/>
     </row>
-    <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="19" t="s">
         <v>868</v>
       </c>
@@ -10520,7 +10586,7 @@
       <c r="G11" s="21"/>
       <c r="H11" s="21"/>
     </row>
-    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="14" t="s">
         <v>868</v>
       </c>
@@ -10542,7 +10608,7 @@
       <c r="G12" s="16"/>
       <c r="H12" s="16"/>
     </row>
-    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="19" t="s">
         <v>868</v>
       </c>
@@ -10564,7 +10630,7 @@
       <c r="G13" s="21"/>
       <c r="H13" s="21"/>
     </row>
-    <row r="14" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="13" t="s">
         <v>886</v>
       </c>
@@ -10578,7 +10644,7 @@
       <c r="G14" s="13"/>
       <c r="H14" s="13"/>
     </row>
-    <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="14" t="s">
         <v>886</v>
       </c>
@@ -10602,7 +10668,7 @@
         <v>958</v>
       </c>
     </row>
-    <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="19" t="s">
         <v>886</v>
       </c>
@@ -10652,7 +10718,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:H36"/>
-  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
@@ -10664,7 +10730,7 @@
     <col min="8" max="8" width="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="28.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:8" ht="28.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="12" t="s">
         <v>33</v>
       </c>
@@ -10690,7 +10756,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="13" t="s">
         <v>41</v>
       </c>
@@ -10704,7 +10770,7 @@
       <c r="G2" s="13"/>
       <c r="H2" s="13"/>
     </row>
-    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
         <v>41</v>
       </c>
@@ -10726,7 +10792,7 @@
       <c r="G3" s="16"/>
       <c r="H3" s="16"/>
     </row>
-    <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="19" t="s">
         <v>41</v>
       </c>
@@ -10748,7 +10814,7 @@
       <c r="G4" s="21"/>
       <c r="H4" s="21"/>
     </row>
-    <row r="5" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="13" t="s">
         <v>48</v>
       </c>
@@ -10762,7 +10828,7 @@
       <c r="G5" s="13"/>
       <c r="H5" s="13"/>
     </row>
-    <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="14" t="s">
         <v>48</v>
       </c>
@@ -10784,7 +10850,7 @@
       <c r="G6" s="16"/>
       <c r="H6" s="16"/>
     </row>
-    <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="19" t="s">
         <v>48</v>
       </c>
@@ -10806,7 +10872,7 @@
       <c r="G7" s="21"/>
       <c r="H7" s="21"/>
     </row>
-    <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="14" t="s">
         <v>48</v>
       </c>
@@ -10828,7 +10894,7 @@
       <c r="G8" s="16"/>
       <c r="H8" s="16"/>
     </row>
-    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="19" t="s">
         <v>48</v>
       </c>
@@ -10850,7 +10916,7 @@
       <c r="G9" s="21"/>
       <c r="H9" s="21"/>
     </row>
-    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="14" t="s">
         <v>48</v>
       </c>
@@ -10872,7 +10938,7 @@
       <c r="G10" s="16"/>
       <c r="H10" s="16"/>
     </row>
-    <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="19" t="s">
         <v>48</v>
       </c>
@@ -10896,7 +10962,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="14" t="s">
         <v>48</v>
       </c>
@@ -10920,7 +10986,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="19" t="s">
         <v>48</v>
       </c>
@@ -10944,7 +11010,7 @@
         <v>895</v>
       </c>
     </row>
-    <row r="14" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="14" t="s">
         <v>48</v>
       </c>
@@ -10966,7 +11032,7 @@
       <c r="G14" s="16"/>
       <c r="H14" s="16"/>
     </row>
-    <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="19" t="s">
         <v>48</v>
       </c>
@@ -10988,7 +11054,7 @@
       <c r="G15" s="21"/>
       <c r="H15" s="21"/>
     </row>
-    <row r="16" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="13" t="s">
         <v>70</v>
       </c>
@@ -11002,7 +11068,7 @@
       <c r="G16" s="13"/>
       <c r="H16" s="13"/>
     </row>
-    <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="14" t="s">
         <v>70</v>
       </c>
@@ -11024,7 +11090,7 @@
       <c r="G17" s="16"/>
       <c r="H17" s="16"/>
     </row>
-    <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="19" t="s">
         <v>70</v>
       </c>
@@ -11046,7 +11112,7 @@
       <c r="G18" s="21"/>
       <c r="H18" s="21"/>
     </row>
-    <row r="19" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="14" t="s">
         <v>70</v>
       </c>
@@ -11070,7 +11136,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="20" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="19" t="s">
         <v>70</v>
       </c>
@@ -11094,7 +11160,7 @@
         <v>895</v>
       </c>
     </row>
-    <row r="21" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="14" t="s">
         <v>70</v>
       </c>
@@ -11118,7 +11184,7 @@
         <v>896</v>
       </c>
     </row>
-    <row r="22" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="19" t="s">
         <v>70</v>
       </c>
@@ -11142,7 +11208,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="23" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="14" t="s">
         <v>70</v>
       </c>
@@ -11166,7 +11232,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="24" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="19" t="s">
         <v>70</v>
       </c>
@@ -11190,7 +11256,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="25" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="14" t="s">
         <v>70</v>
       </c>
@@ -11214,7 +11280,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="26" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="19" t="s">
         <v>70</v>
       </c>
@@ -11238,7 +11304,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="27" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="14" t="s">
         <v>70</v>
       </c>
@@ -11262,7 +11328,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="28" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="19" t="s">
         <v>70</v>
       </c>
@@ -11284,7 +11350,7 @@
       <c r="G28" s="21"/>
       <c r="H28" s="21"/>
     </row>
-    <row r="29" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="13" t="s">
         <v>96</v>
       </c>
@@ -11298,7 +11364,7 @@
       <c r="G29" s="13"/>
       <c r="H29" s="13"/>
     </row>
-    <row r="30" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="14" t="s">
         <v>96</v>
       </c>
@@ -11322,7 +11388,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="31" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="19" t="s">
         <v>96</v>
       </c>
@@ -11346,7 +11412,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="32" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="14" t="s">
         <v>96</v>
       </c>
@@ -11370,7 +11436,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="33" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="13" t="s">
         <v>104</v>
       </c>
@@ -11384,7 +11450,7 @@
       <c r="G33" s="13"/>
       <c r="H33" s="13"/>
     </row>
-    <row r="34" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="14" t="s">
         <v>104</v>
       </c>
@@ -11406,7 +11472,7 @@
       <c r="G34" s="16"/>
       <c r="H34" s="16"/>
     </row>
-    <row r="35" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="19" t="s">
         <v>104</v>
       </c>
@@ -11430,7 +11496,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="36" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="14" t="s">
         <v>104</v>
       </c>
@@ -11478,7 +11544,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:H18"/>
-  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
@@ -11490,7 +11556,7 @@
     <col min="8" max="8" width="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="28.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:8" ht="28.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="12" t="s">
         <v>33</v>
       </c>
@@ -11516,7 +11582,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="13" t="s">
         <v>112</v>
       </c>
@@ -11530,7 +11596,7 @@
       <c r="G2" s="13"/>
       <c r="H2" s="13"/>
     </row>
-    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
         <v>112</v>
       </c>
@@ -11552,7 +11618,7 @@
       <c r="G3" s="16"/>
       <c r="H3" s="16"/>
     </row>
-    <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="19" t="s">
         <v>112</v>
       </c>
@@ -11576,7 +11642,7 @@
         <v>897</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
         <v>112</v>
       </c>
@@ -11600,7 +11666,7 @@
         <v>898</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="13" t="s">
         <v>120</v>
       </c>
@@ -11614,7 +11680,7 @@
       <c r="G6" s="13"/>
       <c r="H6" s="13"/>
     </row>
-    <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="14" t="s">
         <v>120</v>
       </c>
@@ -11636,7 +11702,7 @@
       <c r="G7" s="16"/>
       <c r="H7" s="16"/>
     </row>
-    <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="19" t="s">
         <v>120</v>
       </c>
@@ -11658,7 +11724,7 @@
       <c r="G8" s="21"/>
       <c r="H8" s="21"/>
     </row>
-    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="14" t="s">
         <v>120</v>
       </c>
@@ -11682,7 +11748,7 @@
         <v>897</v>
       </c>
     </row>
-    <row r="10" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="13" t="s">
         <v>128</v>
       </c>
@@ -11696,7 +11762,7 @@
       <c r="G10" s="13"/>
       <c r="H10" s="13"/>
     </row>
-    <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="14" t="s">
         <v>128</v>
       </c>
@@ -11718,7 +11784,7 @@
       <c r="G11" s="16"/>
       <c r="H11" s="16"/>
     </row>
-    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="19" t="s">
         <v>128</v>
       </c>
@@ -11742,7 +11808,7 @@
         <v>899</v>
       </c>
     </row>
-    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="14" t="s">
         <v>128</v>
       </c>
@@ -11766,7 +11832,7 @@
         <v>900</v>
       </c>
     </row>
-    <row r="14" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="19" t="s">
         <v>128</v>
       </c>
@@ -11790,7 +11856,7 @@
         <v>901</v>
       </c>
     </row>
-    <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="14" t="s">
         <v>128</v>
       </c>
@@ -11812,7 +11878,7 @@
       <c r="G15" s="16"/>
       <c r="H15" s="16"/>
     </row>
-    <row r="16" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="13" t="s">
         <v>140</v>
       </c>
@@ -11826,7 +11892,7 @@
       <c r="G16" s="13"/>
       <c r="H16" s="13"/>
     </row>
-    <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="14" t="s">
         <v>140</v>
       </c>
@@ -11850,7 +11916,7 @@
         <v>902</v>
       </c>
     </row>
-    <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="19" t="s">
         <v>140</v>
       </c>
@@ -11898,7 +11964,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:H39"/>
-  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
@@ -11910,7 +11976,7 @@
     <col min="8" max="8" width="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="28.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:8" ht="28.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="12" t="s">
         <v>33</v>
       </c>
@@ -11936,7 +12002,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="13" t="s">
         <v>146</v>
       </c>
@@ -11950,7 +12016,7 @@
       <c r="G2" s="13"/>
       <c r="H2" s="13"/>
     </row>
-    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
         <v>146</v>
       </c>
@@ -11972,7 +12038,7 @@
       <c r="G3" s="16"/>
       <c r="H3" s="16"/>
     </row>
-    <row r="4" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="13" t="s">
         <v>150</v>
       </c>
@@ -11986,7 +12052,7 @@
       <c r="G4" s="13"/>
       <c r="H4" s="13"/>
     </row>
-    <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
         <v>150</v>
       </c>
@@ -12008,7 +12074,7 @@
       <c r="G5" s="16"/>
       <c r="H5" s="16"/>
     </row>
-    <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="19" t="s">
         <v>150</v>
       </c>
@@ -12030,7 +12096,7 @@
       <c r="G6" s="21"/>
       <c r="H6" s="21"/>
     </row>
-    <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="14" t="s">
         <v>150</v>
       </c>
@@ -12052,7 +12118,7 @@
       <c r="G7" s="16"/>
       <c r="H7" s="16"/>
     </row>
-    <row r="8" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="13" t="s">
         <v>158</v>
       </c>
@@ -12066,7 +12132,7 @@
       <c r="G8" s="13"/>
       <c r="H8" s="13"/>
     </row>
-    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="14" t="s">
         <v>158</v>
       </c>
@@ -12088,7 +12154,7 @@
       <c r="G9" s="16"/>
       <c r="H9" s="16"/>
     </row>
-    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="19" t="s">
         <v>158</v>
       </c>
@@ -12112,7 +12178,7 @@
         <v>896</v>
       </c>
     </row>
-    <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="14" t="s">
         <v>158</v>
       </c>
@@ -12136,7 +12202,7 @@
         <v>903</v>
       </c>
     </row>
-    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="19" t="s">
         <v>158</v>
       </c>
@@ -12160,7 +12226,7 @@
         <v>904</v>
       </c>
     </row>
-    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="14" t="s">
         <v>158</v>
       </c>
@@ -12182,7 +12248,7 @@
       <c r="G13" s="16"/>
       <c r="H13" s="16"/>
     </row>
-    <row r="14" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="13" t="s">
         <v>170</v>
       </c>
@@ -12196,7 +12262,7 @@
       <c r="G14" s="13"/>
       <c r="H14" s="13"/>
     </row>
-    <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="14" t="s">
         <v>170</v>
       </c>
@@ -12218,7 +12284,7 @@
       <c r="G15" s="16"/>
       <c r="H15" s="16"/>
     </row>
-    <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="19" t="s">
         <v>170</v>
       </c>
@@ -12240,7 +12306,7 @@
       <c r="G16" s="21"/>
       <c r="H16" s="21"/>
     </row>
-    <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="14" t="s">
         <v>170</v>
       </c>
@@ -12264,7 +12330,7 @@
         <v>905</v>
       </c>
     </row>
-    <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="19" t="s">
         <v>170</v>
       </c>
@@ -12288,7 +12354,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="19" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="14" t="s">
         <v>170</v>
       </c>
@@ -12312,7 +12378,7 @@
         <v>897</v>
       </c>
     </row>
-    <row r="20" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="19" t="s">
         <v>170</v>
       </c>
@@ -12336,7 +12402,7 @@
         <v>906</v>
       </c>
     </row>
-    <row r="21" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="14" t="s">
         <v>170</v>
       </c>
@@ -12358,7 +12424,7 @@
       <c r="G21" s="16"/>
       <c r="H21" s="16"/>
     </row>
-    <row r="22" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="19" t="s">
         <v>170</v>
       </c>
@@ -12380,7 +12446,7 @@
       <c r="G22" s="21"/>
       <c r="H22" s="21"/>
     </row>
-    <row r="23" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="13" t="s">
         <v>188</v>
       </c>
@@ -12394,7 +12460,7 @@
       <c r="G23" s="13"/>
       <c r="H23" s="13"/>
     </row>
-    <row r="24" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="14" t="s">
         <v>188</v>
       </c>
@@ -12416,7 +12482,7 @@
       <c r="G24" s="16"/>
       <c r="H24" s="16"/>
     </row>
-    <row r="25" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="19" t="s">
         <v>188</v>
       </c>
@@ -12438,7 +12504,7 @@
       <c r="G25" s="21"/>
       <c r="H25" s="21"/>
     </row>
-    <row r="26" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="14" t="s">
         <v>188</v>
       </c>
@@ -12460,7 +12526,7 @@
       <c r="G26" s="16"/>
       <c r="H26" s="16"/>
     </row>
-    <row r="27" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="19" t="s">
         <v>188</v>
       </c>
@@ -12484,7 +12550,7 @@
         <v>903</v>
       </c>
     </row>
-    <row r="28" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="14" t="s">
         <v>188</v>
       </c>
@@ -12508,7 +12574,7 @@
         <v>897</v>
       </c>
     </row>
-    <row r="29" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="19" t="s">
         <v>188</v>
       </c>
@@ -12530,7 +12596,7 @@
       <c r="G29" s="21"/>
       <c r="H29" s="21"/>
     </row>
-    <row r="30" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="14" t="s">
         <v>188</v>
       </c>
@@ -12552,7 +12618,7 @@
       <c r="G30" s="16"/>
       <c r="H30" s="16"/>
     </row>
-    <row r="31" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="19" t="s">
         <v>188</v>
       </c>
@@ -12574,7 +12640,7 @@
       <c r="G31" s="21"/>
       <c r="H31" s="21"/>
     </row>
-    <row r="32" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="13" t="s">
         <v>206</v>
       </c>
@@ -12588,7 +12654,7 @@
       <c r="G32" s="13"/>
       <c r="H32" s="13"/>
     </row>
-    <row r="33" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="14" t="s">
         <v>206</v>
       </c>
@@ -12610,7 +12676,7 @@
       <c r="G33" s="16"/>
       <c r="H33" s="16"/>
     </row>
-    <row r="34" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="13" t="s">
         <v>210</v>
       </c>
@@ -12624,7 +12690,7 @@
       <c r="G34" s="13"/>
       <c r="H34" s="13"/>
     </row>
-    <row r="35" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="14" t="s">
         <v>210</v>
       </c>
@@ -12648,7 +12714,7 @@
         <v>895</v>
       </c>
     </row>
-    <row r="36" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="19" t="s">
         <v>210</v>
       </c>
@@ -12672,7 +12738,7 @@
         <v>907</v>
       </c>
     </row>
-    <row r="37" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="14" t="s">
         <v>210</v>
       </c>
@@ -12694,7 +12760,7 @@
       <c r="G37" s="16"/>
       <c r="H37" s="16"/>
     </row>
-    <row r="38" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="19" t="s">
         <v>210</v>
       </c>
@@ -12716,7 +12782,7 @@
       <c r="G38" s="21"/>
       <c r="H38" s="21"/>
     </row>
-    <row r="39" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="14" t="s">
         <v>210</v>
       </c>
@@ -12764,7 +12830,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:H21"/>
-  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
@@ -12776,7 +12842,7 @@
     <col min="8" max="8" width="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="28.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:8" ht="28.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="12" t="s">
         <v>33</v>
       </c>
@@ -12802,7 +12868,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="13" t="s">
         <v>222</v>
       </c>
@@ -12816,7 +12882,7 @@
       <c r="G2" s="13"/>
       <c r="H2" s="13"/>
     </row>
-    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
         <v>222</v>
       </c>
@@ -12838,7 +12904,7 @@
       <c r="G3" s="16"/>
       <c r="H3" s="16"/>
     </row>
-    <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="19" t="s">
         <v>222</v>
       </c>
@@ -12862,7 +12928,7 @@
         <v>908</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
         <v>222</v>
       </c>
@@ -12886,7 +12952,7 @@
         <v>897</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="19" t="s">
         <v>222</v>
       </c>
@@ -12908,7 +12974,7 @@
       <c r="G6" s="21"/>
       <c r="H6" s="21"/>
     </row>
-    <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="14" t="s">
         <v>222</v>
       </c>
@@ -12930,7 +12996,7 @@
       <c r="G7" s="16"/>
       <c r="H7" s="16"/>
     </row>
-    <row r="8" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="13" t="s">
         <v>234</v>
       </c>
@@ -12944,7 +13010,7 @@
       <c r="G8" s="13"/>
       <c r="H8" s="13"/>
     </row>
-    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="14" t="s">
         <v>234</v>
       </c>
@@ -12968,7 +13034,7 @@
         <v>909</v>
       </c>
     </row>
-    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="19" t="s">
         <v>234</v>
       </c>
@@ -12990,7 +13056,7 @@
       <c r="G10" s="21"/>
       <c r="H10" s="21"/>
     </row>
-    <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="14" t="s">
         <v>234</v>
       </c>
@@ -13012,7 +13078,7 @@
       <c r="G11" s="16"/>
       <c r="H11" s="16"/>
     </row>
-    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="19" t="s">
         <v>234</v>
       </c>
@@ -13034,7 +13100,7 @@
       <c r="G12" s="21"/>
       <c r="H12" s="21"/>
     </row>
-    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="14" t="s">
         <v>234</v>
       </c>
@@ -13056,7 +13122,7 @@
       <c r="G13" s="16"/>
       <c r="H13" s="16"/>
     </row>
-    <row r="14" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="13" t="s">
         <v>246</v>
       </c>
@@ -13070,7 +13136,7 @@
       <c r="G14" s="13"/>
       <c r="H14" s="13"/>
     </row>
-    <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="14" t="s">
         <v>246</v>
       </c>
@@ -13094,7 +13160,7 @@
         <v>902</v>
       </c>
     </row>
-    <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="19" t="s">
         <v>246</v>
       </c>
@@ -13118,7 +13184,7 @@
         <v>903</v>
       </c>
     </row>
-    <row r="17" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="13" t="s">
         <v>252</v>
       </c>
@@ -13132,7 +13198,7 @@
       <c r="G17" s="13"/>
       <c r="H17" s="13"/>
     </row>
-    <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="14" t="s">
         <v>252</v>
       </c>
@@ -13154,7 +13220,7 @@
       <c r="G18" s="16"/>
       <c r="H18" s="16"/>
     </row>
-    <row r="19" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="19" t="s">
         <v>252</v>
       </c>
@@ -13178,7 +13244,7 @@
         <v>897</v>
       </c>
     </row>
-    <row r="20" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="14" t="s">
         <v>252</v>
       </c>
@@ -13202,7 +13268,7 @@
         <v>910</v>
       </c>
     </row>
-    <row r="21" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="19" t="s">
         <v>252</v>
       </c>
@@ -13252,7 +13318,7 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:H18"/>
-  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
@@ -13264,7 +13330,7 @@
     <col min="8" max="8" width="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="28.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:8" ht="28.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="12" t="s">
         <v>33</v>
       </c>
@@ -13290,7 +13356,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="13" t="s">
         <v>262</v>
       </c>
@@ -13304,7 +13370,7 @@
       <c r="G2" s="13"/>
       <c r="H2" s="13"/>
     </row>
-    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
         <v>262</v>
       </c>
@@ -13328,7 +13394,7 @@
         <v>912</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="13" t="s">
         <v>266</v>
       </c>
@@ -13342,7 +13408,7 @@
       <c r="G4" s="13"/>
       <c r="H4" s="13"/>
     </row>
-    <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
         <v>266</v>
       </c>
@@ -13368,7 +13434,7 @@
         <v>998</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="19" t="s">
         <v>266</v>
       </c>
@@ -13394,7 +13460,7 @@
         <v>999</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="14" t="s">
         <v>266</v>
       </c>
@@ -13418,7 +13484,7 @@
         <v>913</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="19" t="s">
         <v>266</v>
       </c>
@@ -13440,7 +13506,7 @@
       <c r="G8" s="21"/>
       <c r="H8" s="21"/>
     </row>
-    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="14" t="s">
         <v>266</v>
       </c>
@@ -13462,7 +13528,7 @@
       <c r="G9" s="16"/>
       <c r="H9" s="16"/>
     </row>
-    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="19" t="s">
         <v>266</v>
       </c>
@@ -13484,7 +13550,7 @@
       <c r="G10" s="21"/>
       <c r="H10" s="21"/>
     </row>
-    <row r="11" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="13" t="s">
         <v>280</v>
       </c>
@@ -13498,7 +13564,7 @@
       <c r="G11" s="13"/>
       <c r="H11" s="13"/>
     </row>
-    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="14" t="s">
         <v>280</v>
       </c>
@@ -13524,7 +13590,7 @@
         <v>1001</v>
       </c>
     </row>
-    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="19" t="s">
         <v>280</v>
       </c>
@@ -13550,7 +13616,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="14" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="14" t="s">
         <v>280</v>
       </c>
@@ -13572,7 +13638,7 @@
       <c r="G14" s="16"/>
       <c r="H14" s="16"/>
     </row>
-    <row r="15" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="13" t="s">
         <v>288</v>
       </c>
@@ -13586,7 +13652,7 @@
       <c r="G15" s="13"/>
       <c r="H15" s="13"/>
     </row>
-    <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="14" t="s">
         <v>288</v>
       </c>
@@ -13610,7 +13676,7 @@
         <v>914</v>
       </c>
     </row>
-    <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="19" t="s">
         <v>288</v>
       </c>
@@ -13634,7 +13700,7 @@
         <v>896</v>
       </c>
     </row>
-    <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="14" t="s">
         <v>288</v>
       </c>
@@ -13684,7 +13750,7 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:H56"/>
-  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
@@ -13696,7 +13762,7 @@
     <col min="8" max="8" width="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="28.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:8" ht="28.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="12" t="s">
         <v>33</v>
       </c>
@@ -13722,7 +13788,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="13" t="s">
         <v>296</v>
       </c>
@@ -13736,7 +13802,7 @@
       <c r="G2" s="13"/>
       <c r="H2" s="13"/>
     </row>
-    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
         <v>296</v>
       </c>
@@ -13762,7 +13828,7 @@
         <v>1008</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="19" t="s">
         <v>296</v>
       </c>
@@ -13786,7 +13852,7 @@
         <v>915</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
         <v>296</v>
       </c>
@@ -13810,7 +13876,7 @@
         <v>916</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="13" t="s">
         <v>304</v>
       </c>
@@ -13824,7 +13890,7 @@
       <c r="G6" s="13"/>
       <c r="H6" s="13"/>
     </row>
-    <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="14" t="s">
         <v>304</v>
       </c>
@@ -13846,7 +13912,7 @@
       <c r="G7" s="16"/>
       <c r="H7" s="16"/>
     </row>
-    <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="19" t="s">
         <v>304</v>
       </c>
@@ -13868,7 +13934,7 @@
       <c r="G8" s="21"/>
       <c r="H8" s="21"/>
     </row>
-    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="14" t="s">
         <v>304</v>
       </c>
@@ -13890,7 +13956,7 @@
       <c r="G9" s="16"/>
       <c r="H9" s="16"/>
     </row>
-    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="19" t="s">
         <v>304</v>
       </c>
@@ -13912,7 +13978,7 @@
       <c r="G10" s="21"/>
       <c r="H10" s="21"/>
     </row>
-    <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="14" t="s">
         <v>304</v>
       </c>
@@ -13934,7 +14000,7 @@
       <c r="G11" s="16"/>
       <c r="H11" s="16"/>
     </row>
-    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="19" t="s">
         <v>304</v>
       </c>
@@ -13956,7 +14022,7 @@
       <c r="G12" s="21"/>
       <c r="H12" s="21"/>
     </row>
-    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="14" t="s">
         <v>304</v>
       </c>
@@ -13978,7 +14044,7 @@
       <c r="G13" s="16"/>
       <c r="H13" s="16"/>
     </row>
-    <row r="14" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="19" t="s">
         <v>304</v>
       </c>
@@ -14000,7 +14066,7 @@
       <c r="G14" s="21"/>
       <c r="H14" s="21"/>
     </row>
-    <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="14" t="s">
         <v>304</v>
       </c>
@@ -14024,7 +14090,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="19" t="s">
         <v>304</v>
       </c>
@@ -14048,7 +14114,7 @@
         <v>917</v>
       </c>
     </row>
-    <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="14" t="s">
         <v>304</v>
       </c>
@@ -14072,7 +14138,7 @@
         <v>915</v>
       </c>
     </row>
-    <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="19" t="s">
         <v>304</v>
       </c>
@@ -14096,7 +14162,7 @@
         <v>918</v>
       </c>
     </row>
-    <row r="19" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="13" t="s">
         <v>330</v>
       </c>
@@ -14110,7 +14176,7 @@
       <c r="G19" s="16"/>
       <c r="H19" s="13"/>
     </row>
-    <row r="20" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="14" t="s">
         <v>330</v>
       </c>
@@ -14129,14 +14195,14 @@
       <c r="F20" s="18" t="s">
         <v>981</v>
       </c>
-      <c r="G20" s="30" t="s">
+      <c r="G20" s="27" t="s">
         <v>1010</v>
       </c>
       <c r="H20" s="16" t="s">
         <v>1008</v>
       </c>
     </row>
-    <row r="21" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="19" t="s">
         <v>330</v>
       </c>
@@ -14158,7 +14224,7 @@
       <c r="G21" s="21"/>
       <c r="H21" s="21"/>
     </row>
-    <row r="22" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="14" t="s">
         <v>330</v>
       </c>
@@ -14182,7 +14248,7 @@
         <v>916</v>
       </c>
     </row>
-    <row r="23" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="19" t="s">
         <v>330</v>
       </c>
@@ -14206,7 +14272,7 @@
         <v>916</v>
       </c>
     </row>
-    <row r="24" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="14" t="s">
         <v>330</v>
       </c>
@@ -14228,7 +14294,7 @@
       <c r="G24" s="16"/>
       <c r="H24" s="16"/>
     </row>
-    <row r="25" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="19" t="s">
         <v>330</v>
       </c>
@@ -14250,7 +14316,7 @@
       <c r="G25" s="21"/>
       <c r="H25" s="21"/>
     </row>
-    <row r="26" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="14" t="s">
         <v>330</v>
       </c>
@@ -14272,7 +14338,7 @@
       <c r="G26" s="16"/>
       <c r="H26" s="16"/>
     </row>
-    <row r="27" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="19" t="s">
         <v>330</v>
       </c>
@@ -14294,7 +14360,7 @@
       <c r="G27" s="21"/>
       <c r="H27" s="21"/>
     </row>
-    <row r="28" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="13" t="s">
         <v>348</v>
       </c>
@@ -14308,7 +14374,7 @@
       <c r="G28" s="13"/>
       <c r="H28" s="13"/>
     </row>
-    <row r="29" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="14" t="s">
         <v>348</v>
       </c>
@@ -14330,7 +14396,7 @@
       <c r="G29" s="16"/>
       <c r="H29" s="16"/>
     </row>
-    <row r="30" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="19" t="s">
         <v>348</v>
       </c>
@@ -14352,7 +14418,7 @@
       <c r="G30" s="21"/>
       <c r="H30" s="21"/>
     </row>
-    <row r="31" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="14" t="s">
         <v>348</v>
       </c>
@@ -14376,7 +14442,7 @@
         <v>919</v>
       </c>
     </row>
-    <row r="32" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="19" t="s">
         <v>348</v>
       </c>
@@ -14400,7 +14466,7 @@
         <v>920</v>
       </c>
     </row>
-    <row r="33" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="14" t="s">
         <v>348</v>
       </c>
@@ -14422,7 +14488,7 @@
       <c r="G33" s="16"/>
       <c r="H33" s="16"/>
     </row>
-    <row r="34" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="19" t="s">
         <v>348</v>
       </c>
@@ -14444,7 +14510,7 @@
       <c r="G34" s="21"/>
       <c r="H34" s="21"/>
     </row>
-    <row r="35" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="13" t="s">
         <v>362</v>
       </c>
@@ -14458,7 +14524,7 @@
       <c r="G35" s="13"/>
       <c r="H35" s="13"/>
     </row>
-    <row r="36" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="14" t="s">
         <v>362</v>
       </c>
@@ -14482,7 +14548,7 @@
         <v>919</v>
       </c>
     </row>
-    <row r="37" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="19" t="s">
         <v>362</v>
       </c>
@@ -14506,7 +14572,7 @@
         <v>917</v>
       </c>
     </row>
-    <row r="38" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="14" t="s">
         <v>362</v>
       </c>
@@ -14530,7 +14596,7 @@
         <v>918</v>
       </c>
     </row>
-    <row r="39" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="19" t="s">
         <v>362</v>
       </c>
@@ -14554,7 +14620,7 @@
         <v>918</v>
       </c>
     </row>
-    <row r="40" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="14" t="s">
         <v>362</v>
       </c>
@@ -14578,7 +14644,7 @@
         <v>921</v>
       </c>
     </row>
-    <row r="41" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="19" t="s">
         <v>362</v>
       </c>
@@ -14600,7 +14666,7 @@
       <c r="G41" s="21"/>
       <c r="H41" s="21"/>
     </row>
-    <row r="42" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="14" t="s">
         <v>362</v>
       </c>
@@ -14622,7 +14688,7 @@
       <c r="G42" s="16"/>
       <c r="H42" s="16"/>
     </row>
-    <row r="43" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="19" t="s">
         <v>362</v>
       </c>
@@ -14644,7 +14710,7 @@
       <c r="G43" s="21"/>
       <c r="H43" s="21"/>
     </row>
-    <row r="44" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="13" t="s">
         <v>380</v>
       </c>
@@ -14658,7 +14724,7 @@
       <c r="G44" s="13"/>
       <c r="H44" s="13"/>
     </row>
-    <row r="45" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="14" t="s">
         <v>380</v>
       </c>
@@ -14682,7 +14748,7 @@
         <v>916</v>
       </c>
     </row>
-    <row r="46" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="19" t="s">
         <v>380</v>
       </c>
@@ -14706,7 +14772,7 @@
         <v>919</v>
       </c>
     </row>
-    <row r="47" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="14" t="s">
         <v>380</v>
       </c>
@@ -14730,7 +14796,7 @@
         <v>922</v>
       </c>
     </row>
-    <row r="48" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="19" t="s">
         <v>380</v>
       </c>
@@ -14752,7 +14818,7 @@
       <c r="G48" s="21"/>
       <c r="H48" s="21"/>
     </row>
-    <row r="49" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="13" t="s">
         <v>390</v>
       </c>
@@ -14766,7 +14832,7 @@
       <c r="G49" s="13"/>
       <c r="H49" s="13"/>
     </row>
-    <row r="50" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="14" t="s">
         <v>390</v>
       </c>
@@ -14788,7 +14854,7 @@
       <c r="G50" s="16"/>
       <c r="H50" s="16"/>
     </row>
-    <row r="51" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="19" t="s">
         <v>390</v>
       </c>
@@ -14810,7 +14876,7 @@
       <c r="G51" s="21"/>
       <c r="H51" s="21"/>
     </row>
-    <row r="52" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="13" t="s">
         <v>396</v>
       </c>
@@ -14824,7 +14890,7 @@
       <c r="G52" s="13"/>
       <c r="H52" s="13"/>
     </row>
-    <row r="53" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="14" t="s">
         <v>396</v>
       </c>
@@ -14848,7 +14914,7 @@
         <v>903</v>
       </c>
     </row>
-    <row r="54" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" s="19" t="s">
         <v>396</v>
       </c>
@@ -14872,7 +14938,7 @@
         <v>919</v>
       </c>
     </row>
-    <row r="55" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="14" t="s">
         <v>396</v>
       </c>
@@ -14896,7 +14962,7 @@
         <v>919</v>
       </c>
     </row>
-    <row r="56" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="19" t="s">
         <v>396</v>
       </c>
@@ -14946,7 +15012,7 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:H26"/>
-  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
@@ -14958,7 +15024,7 @@
     <col min="8" max="8" width="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="28.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:8" ht="28.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="12" t="s">
         <v>33</v>
       </c>
@@ -14984,7 +15050,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="13" t="s">
         <v>406</v>
       </c>
@@ -14998,7 +15064,7 @@
       <c r="G2" s="13"/>
       <c r="H2" s="13"/>
     </row>
-    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
         <v>406</v>
       </c>
@@ -15022,7 +15088,7 @@
         <v>919</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="19" t="s">
         <v>406</v>
       </c>
@@ -15046,7 +15112,7 @@
         <v>923</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
         <v>406</v>
       </c>
@@ -15070,7 +15136,7 @@
         <v>924</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="13" t="s">
         <v>414</v>
       </c>
@@ -15084,7 +15150,7 @@
       <c r="G6" s="13"/>
       <c r="H6" s="13"/>
     </row>
-    <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="14" t="s">
         <v>414</v>
       </c>
@@ -15106,7 +15172,7 @@
       <c r="G7" s="16"/>
       <c r="H7" s="16"/>
     </row>
-    <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="19" t="s">
         <v>414</v>
       </c>
@@ -15128,7 +15194,7 @@
       <c r="G8" s="21"/>
       <c r="H8" s="21"/>
     </row>
-    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="14" t="s">
         <v>414</v>
       </c>
@@ -15150,7 +15216,7 @@
       <c r="G9" s="16"/>
       <c r="H9" s="16"/>
     </row>
-    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="19" t="s">
         <v>414</v>
       </c>
@@ -15172,7 +15238,7 @@
       <c r="G10" s="21"/>
       <c r="H10" s="21"/>
     </row>
-    <row r="11" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="13" t="s">
         <v>424</v>
       </c>
@@ -15186,7 +15252,7 @@
       <c r="G11" s="13"/>
       <c r="H11" s="13"/>
     </row>
-    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="14" t="s">
         <v>424</v>
       </c>
@@ -15210,7 +15276,7 @@
         <v>919</v>
       </c>
     </row>
-    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="19" t="s">
         <v>424</v>
       </c>
@@ -15234,7 +15300,7 @@
         <v>919</v>
       </c>
     </row>
-    <row r="14" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="13" t="s">
         <v>430</v>
       </c>
@@ -15248,7 +15314,7 @@
       <c r="G14" s="13"/>
       <c r="H14" s="13"/>
     </row>
-    <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="14" t="s">
         <v>430</v>
       </c>
@@ -15270,7 +15336,7 @@
       <c r="G15" s="16"/>
       <c r="H15" s="16"/>
     </row>
-    <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="19" t="s">
         <v>430</v>
       </c>
@@ -15292,7 +15358,7 @@
       <c r="G16" s="21"/>
       <c r="H16" s="21"/>
     </row>
-    <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="14" t="s">
         <v>430</v>
       </c>
@@ -15316,7 +15382,7 @@
         <v>925</v>
       </c>
     </row>
-    <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="19" t="s">
         <v>430</v>
       </c>
@@ -15340,7 +15406,7 @@
         <v>926</v>
       </c>
     </row>
-    <row r="19" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="14" t="s">
         <v>430</v>
       </c>
@@ -15364,7 +15430,7 @@
         <v>927</v>
       </c>
     </row>
-    <row r="20" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="13" t="s">
         <v>442</v>
       </c>
@@ -15378,7 +15444,7 @@
       <c r="G20" s="13"/>
       <c r="H20" s="13"/>
     </row>
-    <row r="21" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="14" t="s">
         <v>442</v>
       </c>
@@ -15402,7 +15468,7 @@
         <v>916</v>
       </c>
     </row>
-    <row r="22" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="19" t="s">
         <v>442</v>
       </c>
@@ -15426,7 +15492,7 @@
         <v>925</v>
       </c>
     </row>
-    <row r="23" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="14" t="s">
         <v>442</v>
       </c>
@@ -15448,7 +15514,7 @@
       <c r="G23" s="16"/>
       <c r="H23" s="16"/>
     </row>
-    <row r="24" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="13" t="s">
         <v>450</v>
       </c>
@@ -15462,7 +15528,7 @@
       <c r="G24" s="13"/>
       <c r="H24" s="13"/>
     </row>
-    <row r="25" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="14" t="s">
         <v>450</v>
       </c>
@@ -15486,7 +15552,7 @@
         <v>924</v>
       </c>
     </row>
-    <row r="26" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="19" t="s">
         <v>450</v>
       </c>
@@ -15536,7 +15602,7 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
   <dimension ref="A1:H18"/>
-  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
@@ -15548,7 +15614,7 @@
     <col min="8" max="8" width="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="28.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:8" ht="28.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="12" t="s">
         <v>33</v>
       </c>
@@ -15574,7 +15640,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="13" t="s">
         <v>456</v>
       </c>
@@ -15588,7 +15654,7 @@
       <c r="G2" s="13"/>
       <c r="H2" s="13"/>
     </row>
-    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
         <v>456</v>
       </c>
@@ -15614,7 +15680,7 @@
         <v>1004</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="19" t="s">
         <v>456</v>
       </c>
@@ -15638,7 +15704,7 @@
         <v>903</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
         <v>456</v>
       </c>
@@ -15660,7 +15726,7 @@
       <c r="G5" s="16"/>
       <c r="H5" s="16"/>
     </row>
-    <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="19" t="s">
         <v>456</v>
       </c>
@@ -15682,7 +15748,7 @@
       <c r="G6" s="21"/>
       <c r="H6" s="21"/>
     </row>
-    <row r="7" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="13" t="s">
         <v>466</v>
       </c>
@@ -15696,7 +15762,7 @@
       <c r="G7" s="13"/>
       <c r="H7" s="13"/>
     </row>
-    <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="14" t="s">
         <v>466</v>
       </c>
@@ -15718,7 +15784,7 @@
       <c r="G8" s="16"/>
       <c r="H8" s="16"/>
     </row>
-    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="19" t="s">
         <v>466</v>
       </c>
@@ -15744,7 +15810,7 @@
         <v>1002</v>
       </c>
     </row>
-    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="14" t="s">
         <v>466</v>
       </c>
@@ -15768,7 +15834,7 @@
         <v>903</v>
       </c>
     </row>
-    <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="19" t="s">
         <v>466</v>
       </c>
@@ -15790,7 +15856,7 @@
       <c r="G11" s="21"/>
       <c r="H11" s="21"/>
     </row>
-    <row r="12" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="13" t="s">
         <v>476</v>
       </c>
@@ -15804,7 +15870,7 @@
       <c r="G12" s="13"/>
       <c r="H12" s="13"/>
     </row>
-    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="14" t="s">
         <v>476</v>
       </c>
@@ -15830,7 +15896,7 @@
         <v>1004</v>
       </c>
     </row>
-    <row r="14" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="19" t="s">
         <v>476</v>
       </c>
@@ -15852,7 +15918,7 @@
       <c r="G14" s="21"/>
       <c r="H14" s="21"/>
     </row>
-    <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="14" t="s">
         <v>476</v>
       </c>
@@ -15874,7 +15940,7 @@
       <c r="G15" s="16"/>
       <c r="H15" s="16"/>
     </row>
-    <row r="16" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="13" t="s">
         <v>484</v>
       </c>
@@ -15888,7 +15954,7 @@
       <c r="G16" s="13"/>
       <c r="H16" s="13"/>
     </row>
-    <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="14" t="s">
         <v>484</v>
       </c>
@@ -15912,7 +15978,7 @@
         <v>901</v>
       </c>
     </row>
-    <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="19" t="s">
         <v>484</v>
       </c>

</xml_diff>

<commit_message>
docs: updated asvs tracker
</commit_message>
<xml_diff>
--- a/Deliverables/Phase_1/ASVS_5.0_Tracker.xlsx
+++ b/Deliverables/Phase_1/ASVS_5.0_Tracker.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24332"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Utilizador\Desktop\DESOFS\desofs2026-thu_crr_2\Deliverables\Phase_1\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\KapaZete\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8DF1C60A-0940-4656-9DCF-B1F6AE87E08F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A518BBF2-6107-487A-9A66-2E9EB24F283E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="500" firstSheet="13" activeTab="13" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2278" uniqueCount="1021">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2285" uniqueCount="1029">
   <si>
     <t>OWASP ASVS 5.0 – Compliance Tracker</t>
   </si>
@@ -2805,9 +2805,6 @@
   </si>
   <si>
     <t>SR-06, SR-11</t>
-  </si>
-  <si>
-    <t>SR-01, SR06</t>
   </si>
   <si>
     <t>SR-08, SR-14</t>
@@ -3147,12 +3144,77 @@
   <si>
     <t>errorHandler loga UNHANDLED_ERROR com stack; httpLogger loga 5xx como error</t>
   </si>
+  <si>
+    <t>SR-08, (https://github.com/mei-desofs/desofs2026-thu_crr_2/pull/21)</t>
+  </si>
+  <si>
+    <t>https://github.com/mei-desofs/desofs2026-thu_crr_2/pull/21</t>
+  </si>
+  <si>
+    <t>SR-01, SR-08, https://github.com/mei-desofs/desofs2026-thu_crr_2/pull/21</t>
+  </si>
+  <si>
+    <t>"applicationDocumentParamSchema" em "common.validation.ts" força filename ao pattern ^[A-Za-z0-9._-]+$,  rejeita "/"," \", "..", e qualquer caracter especial. Aplicado via validate(schema, "params") em ApplicationRoutes.ts.</t>
+  </si>
+  <si>
+    <t>SR-01, SR06, https://github.com/mei-desofs/desofs2026-thu_crr_2/pull/21</t>
+  </si>
+  <si>
+    <t>"UserValidation.ts" usa "Joi.when()" para validar combinações: RefectoryManager exige refeitorioId, CanteenManager exige canteenId, outros roles rejeitam ambos.</t>
+  </si>
+  <si>
+    <r>
+      <t>Regras documentadas em "</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>Deliverables/Phase_2_pt2/D5-input-validation.md"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t>. Cada endpoint tem schema Joi declarativo em "</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>Backend/src/Schemas/"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <t>Todos os 23 routes aplicam "validate(schema)" antes do controller. Schemas usam abordagem positive/allowlist (campos e valores explicitamente permitidos e desconhecidos rejeitados).</t>
+  </si>
+  <si>
+    <t>"Joi .number().integer().positive( " aplicado em todos os IDs de path/body. Rejeita inputs fora de range, negativos, decimais e NaN antes de chegarem ao ORM.</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="12" x14ac:knownFonts="1">
+  <fonts count="14" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -3231,6 +3293,20 @@
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial Unicode MS"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="10">
@@ -3324,10 +3400,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -3402,6 +3479,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -3409,9 +3487,13 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hiperligação" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -3637,7 +3719,7 @@
                   <c:v>0.375</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.25</c:v>
+                  <c:v>0.75</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
@@ -3818,10 +3900,10 @@
                 <c:formatCode>0%</c:formatCode>
                 <c:ptCount val="17"/>
                 <c:pt idx="0">
-                  <c:v>0</c:v>
+                  <c:v>5.2631578947368418E-2</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0</c:v>
+                  <c:v>0.14285714285714285</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
@@ -3830,7 +3912,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0</c:v>
+                  <c:v>0.2</c:v>
                 </c:pt>
                 <c:pt idx="5">
                   <c:v>9.0909090909090912E-2</c:v>
@@ -4183,10 +4265,10 @@
                 <c:formatCode>0%</c:formatCode>
                 <c:ptCount val="17"/>
                 <c:pt idx="0">
-                  <c:v>0.1</c:v>
+                  <c:v>0.13333333333333333</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>7.6923076923076927E-2</c:v>
+                  <c:v>0.30769230769230771</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
@@ -4195,7 +4277,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.30769230769230771</c:v>
+                  <c:v>0.38461538461538464</c:v>
                 </c:pt>
                 <c:pt idx="5">
                   <c:v>0.1276595744680851</c:v>
@@ -4751,46 +4833,46 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="28" t="s">
+      <c r="A1" s="29" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="28"/>
-      <c r="C1" s="28"/>
-      <c r="D1" s="28"/>
-      <c r="E1" s="28"/>
-      <c r="F1" s="28"/>
-      <c r="G1" s="28"/>
-      <c r="H1" s="28"/>
-      <c r="I1" s="28"/>
-      <c r="J1" s="28"/>
-      <c r="K1" s="28"/>
-      <c r="L1" s="28"/>
-      <c r="M1" s="28"/>
-      <c r="N1" s="28"/>
-      <c r="O1" s="28"/>
-      <c r="P1" s="28"/>
+      <c r="B1" s="29"/>
+      <c r="C1" s="29"/>
+      <c r="D1" s="29"/>
+      <c r="E1" s="29"/>
+      <c r="F1" s="29"/>
+      <c r="G1" s="29"/>
+      <c r="H1" s="29"/>
+      <c r="I1" s="29"/>
+      <c r="J1" s="29"/>
+      <c r="K1" s="29"/>
+      <c r="L1" s="29"/>
+      <c r="M1" s="29"/>
+      <c r="N1" s="29"/>
+      <c r="O1" s="29"/>
+      <c r="P1" s="29"/>
     </row>
     <row r="2" spans="1:16" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="29"/>
-      <c r="B2" s="29"/>
-      <c r="C2" s="29"/>
-      <c r="D2" s="29"/>
-      <c r="E2" s="29"/>
-      <c r="F2" s="29"/>
-      <c r="G2" s="29"/>
-      <c r="H2" s="29"/>
-      <c r="I2" s="29"/>
-      <c r="J2" s="29"/>
-      <c r="K2" s="29"/>
-      <c r="L2" s="29"/>
-      <c r="M2" s="29"/>
-      <c r="N2" s="29"/>
-      <c r="O2" s="29"/>
-      <c r="P2" s="29"/>
+      <c r="A2" s="30"/>
+      <c r="B2" s="30"/>
+      <c r="C2" s="30"/>
+      <c r="D2" s="30"/>
+      <c r="E2" s="30"/>
+      <c r="F2" s="30"/>
+      <c r="G2" s="30"/>
+      <c r="H2" s="30"/>
+      <c r="I2" s="30"/>
+      <c r="J2" s="30"/>
+      <c r="K2" s="30"/>
+      <c r="L2" s="30"/>
+      <c r="M2" s="30"/>
+      <c r="N2" s="30"/>
+      <c r="O2" s="30"/>
+      <c r="P2" s="30"/>
     </row>
     <row r="3" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="30"/>
-      <c r="B3" s="30"/>
+      <c r="A3" s="31"/>
+      <c r="B3" s="31"/>
       <c r="C3" s="1"/>
       <c r="E3" s="1"/>
       <c r="G3" s="1"/>
@@ -4863,11 +4945,11 @@
       </c>
       <c r="G6" s="4">
         <f>COUNTIFS('V1 - Encoding and Sanitization'!$F$2:$F$36,"Compliant",'V1 - Encoding and Sanitization'!$E$2:$E$36,2)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H6" s="5">
         <f t="shared" ref="H6:H22" si="1">IF(F6=0,"",G6/F6)</f>
-        <v>0</v>
+        <v>5.2631578947368418E-2</v>
       </c>
       <c r="I6" s="4">
         <v>3</v>
@@ -4882,11 +4964,11 @@
       </c>
       <c r="L6" s="4">
         <f>COUNTIF('V1 - Encoding and Sanitization'!$F$2:$F$36,"Compliant")</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M6" s="5">
         <f t="shared" ref="M6:M22" si="3">IF(B6=0,"",L6/B6)</f>
-        <v>0.1</v>
+        <v>0.13333333333333333</v>
       </c>
     </row>
     <row r="7" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -4901,22 +4983,22 @@
       </c>
       <c r="D7" s="7">
         <f>COUNTIFS('V2 - Validation and Business Lo'!$F$2:$F$18,"Compliant",'V2 - Validation and Business Lo'!$E$2:$E$18,1)</f>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E7" s="8">
         <f t="shared" si="0"/>
-        <v>0.25</v>
+        <v>0.75</v>
       </c>
       <c r="F7" s="7">
         <v>7</v>
       </c>
       <c r="G7" s="7">
         <f>COUNTIFS('V2 - Validation and Business Lo'!$F$2:$F$18,"Compliant",'V2 - Validation and Business Lo'!$E$2:$E$18,2)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H7" s="8">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.14285714285714285</v>
       </c>
       <c r="I7" s="7">
         <v>2</v>
@@ -4931,11 +5013,11 @@
       </c>
       <c r="L7" s="7">
         <f>COUNTIF('V2 - Validation and Business Lo'!$F$2:$F$18,"Compliant")</f>
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="M7" s="8">
         <f t="shared" si="3"/>
-        <v>7.6923076923076927E-2</v>
+        <v>0.30769230769230771</v>
       </c>
     </row>
     <row r="8" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -5059,11 +5141,11 @@
       </c>
       <c r="G10" s="4">
         <f>COUNTIFS('V5 - File Handling'!$F$2:$F$18,"Compliant",'V5 - File Handling'!$E$2:$E$18,2)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H10" s="5">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="I10" s="4">
         <v>4</v>
@@ -5078,11 +5160,11 @@
       </c>
       <c r="L10" s="4">
         <f>COUNTIF('V5 - File Handling'!$F$2:$F$18,"Compliant")</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M10" s="5">
         <f t="shared" si="3"/>
-        <v>0.30769230769230771</v>
+        <v>0.38461538461538464</v>
       </c>
     </row>
     <row r="11" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -5681,11 +5763,11 @@
       </c>
       <c r="D23" s="10">
         <f>SUM(D6:D22)</f>
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="E23" s="11">
         <f>IFERROR(AVERAGE(E6:E22),"")</f>
-        <v>0.29551282051282057</v>
+        <v>0.32884615384615384</v>
       </c>
       <c r="F23" s="10">
         <f>SUM(F6:F22)</f>
@@ -5693,11 +5775,11 @@
       </c>
       <c r="G23" s="10">
         <f>SUM(G6:G22)</f>
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="H23" s="11">
         <f>IFERROR(AVERAGE(H6:H22),"")</f>
-        <v>6.2700534759358287E-2</v>
+        <v>8.5964577218447177E-2</v>
       </c>
       <c r="I23" s="10">
         <f>SUM(I6:I22)</f>
@@ -5713,11 +5795,11 @@
       </c>
       <c r="L23" s="10">
         <f>SUM(L6:L22)</f>
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="M23" s="11">
         <f>IFERROR(AVERAGE(M6:M22),"")</f>
-        <v>0.13957699586804467</v>
+        <v>0.15963732769308236</v>
       </c>
     </row>
   </sheetData>
@@ -5852,13 +5934,13 @@
         <v>1</v>
       </c>
       <c r="F3" s="18" t="s">
-        <v>981</v>
+        <v>980</v>
       </c>
       <c r="G3" s="16" t="s">
+        <v>1005</v>
+      </c>
+      <c r="H3" s="16" t="s">
         <v>1006</v>
-      </c>
-      <c r="H3" s="16" t="s">
-        <v>1007</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -5878,13 +5960,13 @@
         <v>1</v>
       </c>
       <c r="F4" s="18" t="s">
-        <v>981</v>
+        <v>980</v>
       </c>
       <c r="G4" s="21" t="s">
+        <v>1005</v>
+      </c>
+      <c r="H4" s="21" t="s">
         <v>1006</v>
-      </c>
-      <c r="H4" s="21" t="s">
-        <v>1007</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -5904,7 +5986,7 @@
         <v>1</v>
       </c>
       <c r="F5" s="18" t="s">
-        <v>981</v>
+        <v>980</v>
       </c>
       <c r="G5" s="16"/>
       <c r="H5" s="16"/>
@@ -5940,7 +6022,7 @@
         <v>1</v>
       </c>
       <c r="F7" s="18" t="s">
-        <v>980</v>
+        <v>979</v>
       </c>
       <c r="G7" s="16"/>
       <c r="H7" s="16"/>
@@ -5962,7 +6044,7 @@
         <v>2</v>
       </c>
       <c r="F8" s="18" t="s">
-        <v>980</v>
+        <v>979</v>
       </c>
       <c r="G8" s="21"/>
       <c r="H8" s="21" t="s">
@@ -5990,7 +6072,7 @@
       </c>
       <c r="G9" s="16"/>
       <c r="H9" s="16" t="s">
-        <v>916</v>
+        <v>915</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -6140,7 +6222,7 @@
       </c>
       <c r="G4" s="21"/>
       <c r="H4" s="21" t="s">
-        <v>928</v>
+        <v>927</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -6178,7 +6260,7 @@
       </c>
       <c r="G6" s="16"/>
       <c r="H6" s="16" t="s">
-        <v>921</v>
+        <v>920</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -6262,7 +6344,7 @@
       </c>
       <c r="G10" s="16"/>
       <c r="H10" s="16" t="s">
-        <v>916</v>
+        <v>915</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -6286,7 +6368,7 @@
       </c>
       <c r="G11" s="21"/>
       <c r="H11" s="21" t="s">
-        <v>916</v>
+        <v>915</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -6310,7 +6392,7 @@
       </c>
       <c r="G12" s="16"/>
       <c r="H12" s="16" t="s">
-        <v>929</v>
+        <v>928</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -6334,7 +6416,7 @@
       </c>
       <c r="G13" s="21"/>
       <c r="H13" s="21" t="s">
-        <v>916</v>
+        <v>915</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -6504,7 +6586,7 @@
       </c>
       <c r="G21" s="21"/>
       <c r="H21" s="21" t="s">
-        <v>921</v>
+        <v>920</v>
       </c>
     </row>
     <row r="22" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -6528,7 +6610,7 @@
       </c>
       <c r="G22" s="16"/>
       <c r="H22" s="16" t="s">
-        <v>930</v>
+        <v>929</v>
       </c>
     </row>
     <row r="23" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -6552,7 +6634,7 @@
       </c>
       <c r="G23" s="21"/>
       <c r="H23" s="21" t="s">
-        <v>931</v>
+        <v>930</v>
       </c>
     </row>
     <row r="24" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -6576,7 +6658,7 @@
       </c>
       <c r="G24" s="16"/>
       <c r="H24" s="16" t="s">
-        <v>925</v>
+        <v>924</v>
       </c>
     </row>
     <row r="25" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -6600,7 +6682,7 @@
       </c>
       <c r="G25" s="21"/>
       <c r="H25" s="21" t="s">
-        <v>916</v>
+        <v>915</v>
       </c>
     </row>
     <row r="26" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -6772,7 +6854,7 @@
       </c>
       <c r="G33" s="16"/>
       <c r="H33" s="16" t="s">
-        <v>919</v>
+        <v>918</v>
       </c>
     </row>
     <row r="34" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -6796,7 +6878,7 @@
       </c>
       <c r="G34" s="21"/>
       <c r="H34" s="21" t="s">
-        <v>929</v>
+        <v>928</v>
       </c>
     </row>
     <row r="35" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -6844,7 +6926,7 @@
       </c>
       <c r="G36" s="21"/>
       <c r="H36" s="21" t="s">
-        <v>916</v>
+        <v>915</v>
       </c>
     </row>
     <row r="37" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -6868,7 +6950,7 @@
       </c>
       <c r="G37" s="16"/>
       <c r="H37" s="16" t="s">
-        <v>919</v>
+        <v>918</v>
       </c>
     </row>
     <row r="38" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -6906,7 +6988,7 @@
       </c>
       <c r="G39" s="16"/>
       <c r="H39" s="16" t="s">
-        <v>928</v>
+        <v>927</v>
       </c>
     </row>
     <row r="40" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -6930,7 +7012,7 @@
       </c>
       <c r="G40" s="21"/>
       <c r="H40" s="21" t="s">
-        <v>927</v>
+        <v>926</v>
       </c>
     </row>
     <row r="41" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -6992,7 +7074,7 @@
       </c>
       <c r="G43" s="21"/>
       <c r="H43" s="21" t="s">
-        <v>932</v>
+        <v>931</v>
       </c>
     </row>
     <row r="44" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -7016,7 +7098,7 @@
       </c>
       <c r="G44" s="16"/>
       <c r="H44" s="16" t="s">
-        <v>925</v>
+        <v>924</v>
       </c>
     </row>
   </sheetData>
@@ -7118,7 +7200,7 @@
       </c>
       <c r="G3" s="16"/>
       <c r="H3" s="16" t="s">
-        <v>933</v>
+        <v>932</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -7142,7 +7224,7 @@
       </c>
       <c r="G4" s="21"/>
       <c r="H4" s="21" t="s">
-        <v>934</v>
+        <v>933</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -7220,11 +7302,11 @@
         <v>2</v>
       </c>
       <c r="F8" s="18" t="s">
-        <v>980</v>
+        <v>979</v>
       </c>
       <c r="G8" s="16"/>
       <c r="H8" s="16" t="s">
-        <v>934</v>
+        <v>933</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -7248,7 +7330,7 @@
       </c>
       <c r="G9" s="21"/>
       <c r="H9" s="21" t="s">
-        <v>934</v>
+        <v>933</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -7268,11 +7350,11 @@
         <v>2</v>
       </c>
       <c r="F10" s="18" t="s">
-        <v>980</v>
+        <v>979</v>
       </c>
       <c r="G10" s="16"/>
       <c r="H10" s="16" t="s">
-        <v>934</v>
+        <v>933</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -7476,7 +7558,7 @@
         <v>1</v>
       </c>
       <c r="F20" s="18" t="s">
-        <v>981</v>
+        <v>980</v>
       </c>
       <c r="G20" s="16"/>
       <c r="H20" s="16"/>
@@ -7498,11 +7580,11 @@
         <v>2</v>
       </c>
       <c r="F21" s="18" t="s">
-        <v>980</v>
+        <v>979</v>
       </c>
       <c r="G21" s="21"/>
       <c r="H21" s="21" t="s">
-        <v>935</v>
+        <v>934</v>
       </c>
     </row>
     <row r="22" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -7522,11 +7604,11 @@
         <v>2</v>
       </c>
       <c r="F22" s="18" t="s">
-        <v>980</v>
+        <v>979</v>
       </c>
       <c r="G22" s="16"/>
       <c r="H22" s="16" t="s">
-        <v>936</v>
+        <v>935</v>
       </c>
     </row>
     <row r="23" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -7546,11 +7628,11 @@
         <v>2</v>
       </c>
       <c r="F23" s="18" t="s">
-        <v>980</v>
+        <v>979</v>
       </c>
       <c r="G23" s="21"/>
       <c r="H23" s="21" t="s">
-        <v>935</v>
+        <v>934</v>
       </c>
     </row>
     <row r="24" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -7588,7 +7670,7 @@
       </c>
       <c r="G25" s="16"/>
       <c r="H25" s="16" t="s">
-        <v>918</v>
+        <v>917</v>
       </c>
     </row>
     <row r="26" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -7644,11 +7726,11 @@
         <v>2</v>
       </c>
       <c r="F28" s="18" t="s">
-        <v>980</v>
+        <v>979</v>
       </c>
       <c r="G28" s="16"/>
       <c r="H28" s="16" t="s">
-        <v>934</v>
+        <v>933</v>
       </c>
     </row>
     <row r="29" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -7852,7 +7934,7 @@
       </c>
       <c r="G4" s="21"/>
       <c r="H4" s="21" t="s">
-        <v>937</v>
+        <v>936</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -7876,7 +7958,7 @@
       </c>
       <c r="G5" s="16"/>
       <c r="H5" s="16" t="s">
-        <v>938</v>
+        <v>937</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -8016,7 +8098,7 @@
       </c>
       <c r="G12" s="16"/>
       <c r="H12" s="16" t="s">
-        <v>937</v>
+        <v>936</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -8040,7 +8122,7 @@
       </c>
       <c r="G13" s="21"/>
       <c r="H13" s="21" t="s">
-        <v>939</v>
+        <v>938</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -8064,7 +8146,7 @@
       </c>
       <c r="G14" s="16"/>
       <c r="H14" s="16" t="s">
-        <v>937</v>
+        <v>936</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -8088,7 +8170,7 @@
       </c>
       <c r="G15" s="21"/>
       <c r="H15" s="21" t="s">
-        <v>940</v>
+        <v>939</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -8212,7 +8294,7 @@
       </c>
       <c r="G3" s="16"/>
       <c r="H3" s="16" t="s">
-        <v>941</v>
+        <v>940</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -8312,11 +8394,11 @@
         <v>2</v>
       </c>
       <c r="F8" s="18" t="s">
-        <v>980</v>
+        <v>979</v>
       </c>
       <c r="G8" s="16"/>
       <c r="H8" s="16" t="s">
-        <v>942</v>
+        <v>941</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -8364,7 +8446,7 @@
       </c>
       <c r="G10" s="16"/>
       <c r="H10" s="16" t="s">
-        <v>943</v>
+        <v>942</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -8384,11 +8466,11 @@
         <v>2</v>
       </c>
       <c r="F11" s="18" t="s">
-        <v>980</v>
+        <v>979</v>
       </c>
       <c r="G11" s="21"/>
       <c r="H11" s="21" t="s">
-        <v>944</v>
+        <v>943</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -8412,7 +8494,7 @@
       </c>
       <c r="G12" s="16"/>
       <c r="H12" s="16" t="s">
-        <v>945</v>
+        <v>944</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -8472,7 +8554,7 @@
       </c>
       <c r="G15" s="16"/>
       <c r="H15" s="16" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -8496,7 +8578,7 @@
       </c>
       <c r="G16" s="21"/>
       <c r="H16" s="21" t="s">
-        <v>947</v>
+        <v>946</v>
       </c>
     </row>
     <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -8600,7 +8682,7 @@
       </c>
       <c r="G21" s="21"/>
       <c r="H21" s="21" t="s">
-        <v>934</v>
+        <v>933</v>
       </c>
     </row>
     <row r="22" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -8620,11 +8702,11 @@
         <v>2</v>
       </c>
       <c r="F22" s="18" t="s">
-        <v>980</v>
+        <v>979</v>
       </c>
       <c r="G22" s="16"/>
       <c r="H22" s="16" t="s">
-        <v>948</v>
+        <v>947</v>
       </c>
     </row>
     <row r="23" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -8648,7 +8730,7 @@
       </c>
       <c r="G23" s="21"/>
       <c r="H23" s="21" t="s">
-        <v>949</v>
+        <v>948</v>
       </c>
     </row>
     <row r="24" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -8672,7 +8754,7 @@
       </c>
       <c r="G24" s="16"/>
       <c r="H24" s="16" t="s">
-        <v>950</v>
+        <v>949</v>
       </c>
     </row>
     <row r="25" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -8814,11 +8896,11 @@
         <v>2</v>
       </c>
       <c r="F3" s="18" t="s">
-        <v>980</v>
+        <v>979</v>
       </c>
       <c r="G3" s="16"/>
       <c r="H3" s="16" t="s">
-        <v>941</v>
+        <v>940</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -8842,7 +8924,7 @@
       </c>
       <c r="G4" s="21"/>
       <c r="H4" s="21" t="s">
-        <v>951</v>
+        <v>950</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -8876,13 +8958,13 @@
         <v>1</v>
       </c>
       <c r="F6" s="18" t="s">
-        <v>981</v>
+        <v>980</v>
       </c>
       <c r="G6" s="16" t="s">
-        <v>992</v>
+        <v>991</v>
       </c>
       <c r="H6" s="16" t="s">
-        <v>1003</v>
+        <v>1002</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -8906,7 +8988,7 @@
       </c>
       <c r="G7" s="21"/>
       <c r="H7" s="21" t="s">
-        <v>952</v>
+        <v>951</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -8930,7 +9012,7 @@
       </c>
       <c r="G8" s="16"/>
       <c r="H8" s="16" t="s">
-        <v>953</v>
+        <v>952</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -8954,7 +9036,7 @@
       </c>
       <c r="G9" s="21"/>
       <c r="H9" s="21" t="s">
-        <v>954</v>
+        <v>953</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -9102,7 +9184,7 @@
       </c>
       <c r="G16" s="21"/>
       <c r="H16" s="21" t="s">
-        <v>955</v>
+        <v>954</v>
       </c>
     </row>
     <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -9126,7 +9208,7 @@
       </c>
       <c r="G17" s="16"/>
       <c r="H17" s="16" t="s">
-        <v>956</v>
+        <v>955</v>
       </c>
     </row>
   </sheetData>
@@ -9250,7 +9332,7 @@
       </c>
       <c r="G4" s="21"/>
       <c r="H4" s="21" t="s">
-        <v>957</v>
+        <v>956</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -9270,11 +9352,11 @@
         <v>2</v>
       </c>
       <c r="F5" s="18" t="s">
-        <v>980</v>
+        <v>979</v>
       </c>
       <c r="G5" s="16"/>
       <c r="H5" s="16" t="s">
-        <v>958</v>
+        <v>957</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -9374,13 +9456,13 @@
         <v>2</v>
       </c>
       <c r="F10" s="18" t="s">
-        <v>981</v>
+        <v>980</v>
       </c>
       <c r="G10" s="21" t="s">
-        <v>986</v>
+        <v>985</v>
       </c>
       <c r="H10" s="21" t="s">
-        <v>997</v>
+        <v>996</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -9400,11 +9482,11 @@
         <v>2</v>
       </c>
       <c r="F11" s="18" t="s">
-        <v>980</v>
+        <v>979</v>
       </c>
       <c r="G11" s="16"/>
       <c r="H11" s="16" t="s">
-        <v>959</v>
+        <v>958</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -9482,7 +9564,7 @@
         <v>1</v>
       </c>
       <c r="F15" s="18" t="s">
-        <v>980</v>
+        <v>979</v>
       </c>
       <c r="G15" s="16"/>
       <c r="H15" s="16"/>
@@ -9508,7 +9590,7 @@
       </c>
       <c r="G16" s="21"/>
       <c r="H16" s="21" t="s">
-        <v>960</v>
+        <v>959</v>
       </c>
     </row>
     <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -9528,11 +9610,11 @@
         <v>2</v>
       </c>
       <c r="F17" s="18" t="s">
-        <v>980</v>
+        <v>979</v>
       </c>
       <c r="G17" s="16"/>
       <c r="H17" s="16" t="s">
-        <v>961</v>
+        <v>960</v>
       </c>
     </row>
     <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -9556,7 +9638,7 @@
       </c>
       <c r="G18" s="21"/>
       <c r="H18" s="21" t="s">
-        <v>962</v>
+        <v>961</v>
       </c>
     </row>
     <row r="19" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -9576,11 +9658,11 @@
         <v>2</v>
       </c>
       <c r="F19" s="18" t="s">
-        <v>980</v>
+        <v>979</v>
       </c>
       <c r="G19" s="16"/>
       <c r="H19" s="16" t="s">
-        <v>963</v>
+        <v>962</v>
       </c>
     </row>
     <row r="20" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -9600,11 +9682,11 @@
         <v>2</v>
       </c>
       <c r="F20" s="18" t="s">
-        <v>980</v>
+        <v>979</v>
       </c>
       <c r="G20" s="21"/>
       <c r="H20" s="21" t="s">
-        <v>963</v>
+        <v>962</v>
       </c>
     </row>
     <row r="21" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -9628,7 +9710,7 @@
       </c>
       <c r="G21" s="16"/>
       <c r="H21" s="16" t="s">
-        <v>964</v>
+        <v>963</v>
       </c>
     </row>
     <row r="22" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -9828,11 +9910,11 @@
         <v>2</v>
       </c>
       <c r="F3" s="18" t="s">
-        <v>981</v>
+        <v>980</v>
       </c>
       <c r="G3" s="16"/>
       <c r="H3" s="16" t="s">
-        <v>965</v>
+        <v>964</v>
       </c>
     </row>
     <row r="4" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -9866,13 +9948,13 @@
         <v>2</v>
       </c>
       <c r="F5" s="18" t="s">
-        <v>981</v>
+        <v>980</v>
       </c>
       <c r="G5" s="16" t="s">
-        <v>1013</v>
+        <v>1012</v>
       </c>
       <c r="H5" s="16" t="s">
-        <v>966</v>
+        <v>965</v>
       </c>
     </row>
     <row r="6" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -9892,13 +9974,13 @@
         <v>2</v>
       </c>
       <c r="F6" s="18" t="s">
-        <v>981</v>
+        <v>980</v>
       </c>
       <c r="G6" s="21" t="s">
-        <v>1014</v>
+        <v>1013</v>
       </c>
       <c r="H6" s="21" t="s">
-        <v>967</v>
+        <v>966</v>
       </c>
       <c r="M6" s="25"/>
     </row>
@@ -9919,13 +10001,13 @@
         <v>2</v>
       </c>
       <c r="F7" s="18" t="s">
-        <v>981</v>
+        <v>980</v>
       </c>
       <c r="G7" s="16" t="s">
-        <v>1015</v>
+        <v>1014</v>
       </c>
       <c r="H7" s="16" t="s">
-        <v>968</v>
+        <v>967</v>
       </c>
     </row>
     <row r="8" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -9945,13 +10027,13 @@
         <v>2</v>
       </c>
       <c r="F8" s="18" t="s">
-        <v>981</v>
+        <v>980</v>
       </c>
       <c r="G8" t="s">
-        <v>1016</v>
+        <v>1015</v>
       </c>
       <c r="H8" s="21" t="s">
-        <v>966</v>
+        <v>965</v>
       </c>
     </row>
     <row r="9" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -9971,13 +10053,13 @@
         <v>2</v>
       </c>
       <c r="F9" s="18" t="s">
-        <v>981</v>
+        <v>980</v>
       </c>
       <c r="G9" s="16" t="s">
+        <v>1010</v>
+      </c>
+      <c r="H9" s="16" t="s">
         <v>1011</v>
-      </c>
-      <c r="H9" s="16" t="s">
-        <v>1012</v>
       </c>
     </row>
     <row r="10" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -10011,13 +10093,13 @@
         <v>2</v>
       </c>
       <c r="F11" s="18" t="s">
-        <v>981</v>
-      </c>
-      <c r="G11" s="31" t="s">
-        <v>1017</v>
+        <v>980</v>
+      </c>
+      <c r="G11" s="28" t="s">
+        <v>1016</v>
       </c>
       <c r="H11" s="16" t="s">
-        <v>969</v>
+        <v>968</v>
       </c>
     </row>
     <row r="12" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -10037,13 +10119,13 @@
         <v>2</v>
       </c>
       <c r="F12" s="18" t="s">
-        <v>981</v>
+        <v>980</v>
       </c>
       <c r="G12" s="21" t="s">
-        <v>1018</v>
+        <v>1017</v>
       </c>
       <c r="H12" s="21" t="s">
-        <v>970</v>
+        <v>969</v>
       </c>
     </row>
     <row r="13" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -10063,13 +10145,13 @@
         <v>2</v>
       </c>
       <c r="F13" s="18" t="s">
-        <v>981</v>
+        <v>980</v>
       </c>
       <c r="G13" s="16" t="s">
-        <v>1019</v>
+        <v>1018</v>
       </c>
       <c r="H13" s="16" t="s">
-        <v>971</v>
+        <v>970</v>
       </c>
     </row>
     <row r="14" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -10089,13 +10171,13 @@
         <v>2</v>
       </c>
       <c r="F14" s="18" t="s">
-        <v>981</v>
+        <v>980</v>
       </c>
       <c r="G14" s="21" t="s">
-        <v>1020</v>
+        <v>1019</v>
       </c>
       <c r="H14" s="21" t="s">
-        <v>972</v>
+        <v>971</v>
       </c>
     </row>
     <row r="15" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -10129,11 +10211,11 @@
         <v>2</v>
       </c>
       <c r="F16" s="18" t="s">
-        <v>981</v>
+        <v>980</v>
       </c>
       <c r="G16" s="16"/>
       <c r="H16" s="16" t="s">
-        <v>996</v>
+        <v>995</v>
       </c>
     </row>
     <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -10157,7 +10239,7 @@
       </c>
       <c r="G17" s="21"/>
       <c r="H17" s="21" t="s">
-        <v>973</v>
+        <v>972</v>
       </c>
     </row>
     <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -10181,7 +10263,7 @@
       </c>
       <c r="G18" s="16"/>
       <c r="H18" s="16" t="s">
-        <v>972</v>
+        <v>971</v>
       </c>
     </row>
     <row r="19" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -10215,13 +10297,13 @@
         <v>2</v>
       </c>
       <c r="F20" s="18" t="s">
+        <v>980</v>
+      </c>
+      <c r="G20" s="16" t="s">
         <v>981</v>
       </c>
-      <c r="G20" s="16" t="s">
-        <v>982</v>
-      </c>
       <c r="H20" s="16" t="s">
-        <v>994</v>
+        <v>993</v>
       </c>
     </row>
     <row r="21" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -10241,13 +10323,13 @@
         <v>2</v>
       </c>
       <c r="F21" s="18" t="s">
-        <v>981</v>
+        <v>980</v>
       </c>
       <c r="G21" s="16" t="s">
-        <v>983</v>
+        <v>982</v>
       </c>
       <c r="H21" s="21" t="s">
-        <v>993</v>
+        <v>992</v>
       </c>
     </row>
     <row r="22" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -10267,13 +10349,13 @@
         <v>2</v>
       </c>
       <c r="F22" s="18" t="s">
-        <v>981</v>
+        <v>980</v>
       </c>
       <c r="G22" s="16" t="s">
-        <v>984</v>
+        <v>983</v>
       </c>
       <c r="H22" s="16" t="s">
-        <v>974</v>
+        <v>973</v>
       </c>
     </row>
     <row r="23" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -10293,13 +10375,13 @@
         <v>3</v>
       </c>
       <c r="F23" s="18" t="s">
-        <v>981</v>
+        <v>980</v>
       </c>
       <c r="G23" s="16" t="s">
-        <v>985</v>
+        <v>984</v>
       </c>
       <c r="H23" s="21" t="s">
-        <v>995</v>
+        <v>994</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.25">
@@ -10407,7 +10489,7 @@
       </c>
       <c r="G3" s="16"/>
       <c r="H3" s="16" t="s">
-        <v>975</v>
+        <v>974</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -10467,7 +10549,7 @@
       </c>
       <c r="G6" s="16"/>
       <c r="H6" s="16" t="s">
-        <v>976</v>
+        <v>975</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -10491,7 +10573,7 @@
       </c>
       <c r="G7" s="21"/>
       <c r="H7" s="21" t="s">
-        <v>977</v>
+        <v>976</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -10515,7 +10597,7 @@
       </c>
       <c r="G8" s="16"/>
       <c r="H8" s="16" t="s">
-        <v>978</v>
+        <v>977</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -10539,7 +10621,7 @@
       </c>
       <c r="G9" s="21"/>
       <c r="H9" s="21" t="s">
-        <v>971</v>
+        <v>970</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -10665,7 +10747,7 @@
       </c>
       <c r="G15" s="16"/>
       <c r="H15" s="16" t="s">
-        <v>958</v>
+        <v>957</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -10689,7 +10771,7 @@
       </c>
       <c r="G16" s="21"/>
       <c r="H16" s="21" t="s">
-        <v>979</v>
+        <v>978</v>
       </c>
     </row>
   </sheetData>
@@ -10787,7 +10869,7 @@
         <v>2</v>
       </c>
       <c r="F3" s="18" t="s">
-        <v>980</v>
+        <v>979</v>
       </c>
       <c r="G3" s="16"/>
       <c r="H3" s="16"/>
@@ -10809,7 +10891,7 @@
         <v>2</v>
       </c>
       <c r="F4" s="18" t="s">
-        <v>980</v>
+        <v>979</v>
       </c>
       <c r="G4" s="21"/>
       <c r="H4" s="21"/>
@@ -10911,7 +10993,7 @@
         <v>1</v>
       </c>
       <c r="F9" s="18" t="s">
-        <v>981</v>
+        <v>980</v>
       </c>
       <c r="G9" s="21"/>
       <c r="H9" s="21"/>
@@ -10933,7 +11015,7 @@
         <v>1</v>
       </c>
       <c r="F10" s="18" t="s">
-        <v>981</v>
+        <v>980</v>
       </c>
       <c r="G10" s="16"/>
       <c r="H10" s="16"/>
@@ -11107,7 +11189,7 @@
         <v>1</v>
       </c>
       <c r="F18" s="18" t="s">
-        <v>981</v>
+        <v>980</v>
       </c>
       <c r="G18" s="21"/>
       <c r="H18" s="21"/>
@@ -11129,7 +11211,7 @@
         <v>2</v>
       </c>
       <c r="F19" s="18" t="s">
-        <v>980</v>
+        <v>979</v>
       </c>
       <c r="G19" s="16"/>
       <c r="H19" s="16" t="s">
@@ -11407,9 +11489,11 @@
       <c r="F31" s="18" t="s">
         <v>980</v>
       </c>
-      <c r="G31" s="21"/>
+      <c r="G31" s="32" t="s">
+        <v>1028</v>
+      </c>
       <c r="H31" s="21" t="s">
-        <v>893</v>
+        <v>1020</v>
       </c>
     </row>
     <row r="32" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -11489,7 +11573,7 @@
         <v>2</v>
       </c>
       <c r="F35" s="18" t="s">
-        <v>980</v>
+        <v>979</v>
       </c>
       <c r="G35" s="21"/>
       <c r="H35" s="21" t="s">
@@ -11537,7 +11621,7 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.51180555555555496" footer="0.51180555555555496"/>
-  <pageSetup firstPageNumber="0" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <pageSetup firstPageNumber="0" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -11615,8 +11699,12 @@
       <c r="F3" s="18" t="s">
         <v>980</v>
       </c>
-      <c r="G3" s="16"/>
-      <c r="H3" s="16"/>
+      <c r="G3" t="s">
+        <v>1026</v>
+      </c>
+      <c r="H3" s="33" t="s">
+        <v>1021</v>
+      </c>
     </row>
     <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="19" t="s">
@@ -11699,8 +11787,12 @@
       <c r="F7" s="18" t="s">
         <v>980</v>
       </c>
-      <c r="G7" s="16"/>
-      <c r="H7" s="16"/>
+      <c r="G7" s="16" t="s">
+        <v>1027</v>
+      </c>
+      <c r="H7" s="16" t="s">
+        <v>1021</v>
+      </c>
     </row>
     <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="19" t="s">
@@ -11719,7 +11811,7 @@
         <v>1</v>
       </c>
       <c r="F8" s="18" t="s">
-        <v>981</v>
+        <v>980</v>
       </c>
       <c r="G8" s="21"/>
       <c r="H8" s="21"/>
@@ -11743,9 +11835,11 @@
       <c r="F9" s="18" t="s">
         <v>980</v>
       </c>
-      <c r="G9" s="16"/>
+      <c r="G9" s="32" t="s">
+        <v>1025</v>
+      </c>
       <c r="H9" s="16" t="s">
-        <v>897</v>
+        <v>1022</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -11956,6 +12050,9 @@
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
+  <hyperlinks>
+    <hyperlink ref="H3" r:id="rId1" xr:uid="{131D9CD9-B617-4364-ABFB-55EC79404F8B}"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.51180555555555496" footer="0.51180555555555496"/>
   <pageSetup firstPageNumber="0" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
@@ -12301,7 +12398,7 @@
         <v>1</v>
       </c>
       <c r="F16" s="18" t="s">
-        <v>980</v>
+        <v>979</v>
       </c>
       <c r="G16" s="21"/>
       <c r="H16" s="21"/>
@@ -12477,7 +12574,7 @@
         <v>1</v>
       </c>
       <c r="F24" s="18" t="s">
-        <v>980</v>
+        <v>979</v>
       </c>
       <c r="G24" s="16"/>
       <c r="H24" s="16"/>
@@ -12499,7 +12596,7 @@
         <v>1</v>
       </c>
       <c r="F25" s="18" t="s">
-        <v>980</v>
+        <v>979</v>
       </c>
       <c r="G25" s="21"/>
       <c r="H25" s="21"/>
@@ -12521,7 +12618,7 @@
         <v>1</v>
       </c>
       <c r="F26" s="18" t="s">
-        <v>980</v>
+        <v>979</v>
       </c>
       <c r="G26" s="16"/>
       <c r="H26" s="16"/>
@@ -12543,7 +12640,7 @@
         <v>2</v>
       </c>
       <c r="F27" s="18" t="s">
-        <v>980</v>
+        <v>979</v>
       </c>
       <c r="G27" s="21"/>
       <c r="H27" s="21" t="s">
@@ -12899,7 +12996,7 @@
         <v>1</v>
       </c>
       <c r="F3" s="18" t="s">
-        <v>980</v>
+        <v>979</v>
       </c>
       <c r="G3" s="16"/>
       <c r="H3" s="16"/>
@@ -13027,7 +13124,7 @@
         <v>2</v>
       </c>
       <c r="F9" s="18" t="s">
-        <v>980</v>
+        <v>979</v>
       </c>
       <c r="G9" s="16"/>
       <c r="H9" s="16" t="s">
@@ -13153,7 +13250,7 @@
         <v>2</v>
       </c>
       <c r="F15" s="18" t="s">
-        <v>980</v>
+        <v>979</v>
       </c>
       <c r="G15" s="16"/>
       <c r="H15" s="16" t="s">
@@ -13387,7 +13484,7 @@
         <v>2</v>
       </c>
       <c r="F3" s="18" t="s">
-        <v>980</v>
+        <v>979</v>
       </c>
       <c r="G3" s="16"/>
       <c r="H3" s="16" t="s">
@@ -13425,13 +13522,13 @@
         <v>1</v>
       </c>
       <c r="F5" s="18" t="s">
-        <v>981</v>
+        <v>980</v>
       </c>
       <c r="G5" s="16" t="s">
-        <v>987</v>
+        <v>986</v>
       </c>
       <c r="H5" s="16" t="s">
-        <v>998</v>
+        <v>997</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -13451,13 +13548,13 @@
         <v>1</v>
       </c>
       <c r="F6" s="18" t="s">
-        <v>981</v>
+        <v>980</v>
       </c>
       <c r="G6" s="21" t="s">
-        <v>988</v>
+        <v>987</v>
       </c>
       <c r="H6" s="21" t="s">
-        <v>999</v>
+        <v>998</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -13581,13 +13678,13 @@
         <v>1</v>
       </c>
       <c r="F12" s="18" t="s">
-        <v>981</v>
+        <v>980</v>
       </c>
       <c r="G12" s="16" t="s">
-        <v>990</v>
+        <v>989</v>
       </c>
       <c r="H12" s="16" t="s">
-        <v>1001</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -13607,13 +13704,13 @@
         <v>1</v>
       </c>
       <c r="F13" s="18" t="s">
-        <v>981</v>
+        <v>980</v>
       </c>
       <c r="G13" s="21" t="s">
-        <v>989</v>
+        <v>988</v>
       </c>
       <c r="H13" s="21" t="s">
-        <v>1000</v>
+        <v>999</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -13671,9 +13768,11 @@
       <c r="F16" s="18" t="s">
         <v>980</v>
       </c>
-      <c r="G16" s="16"/>
+      <c r="G16" s="32" t="s">
+        <v>1023</v>
+      </c>
       <c r="H16" s="16" t="s">
-        <v>914</v>
+        <v>1024</v>
       </c>
     </row>
     <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -13819,13 +13918,13 @@
         <v>1</v>
       </c>
       <c r="F3" s="18" t="s">
-        <v>981</v>
+        <v>980</v>
       </c>
       <c r="G3" s="16" t="s">
-        <v>1009</v>
+        <v>1008</v>
       </c>
       <c r="H3" s="16" t="s">
-        <v>1008</v>
+        <v>1007</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -13849,7 +13948,7 @@
       </c>
       <c r="G4" s="21"/>
       <c r="H4" s="21" t="s">
-        <v>915</v>
+        <v>914</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -13873,7 +13972,7 @@
       </c>
       <c r="G5" s="16"/>
       <c r="H5" s="16" t="s">
-        <v>916</v>
+        <v>915</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -13995,7 +14094,7 @@
         <v>1</v>
       </c>
       <c r="F11" s="18" t="s">
-        <v>981</v>
+        <v>980</v>
       </c>
       <c r="G11" s="16"/>
       <c r="H11" s="16"/>
@@ -14061,7 +14160,7 @@
         <v>1</v>
       </c>
       <c r="F14" s="18" t="s">
-        <v>980</v>
+        <v>979</v>
       </c>
       <c r="G14" s="21"/>
       <c r="H14" s="21"/>
@@ -14083,7 +14182,7 @@
         <v>2</v>
       </c>
       <c r="F15" s="18" t="s">
-        <v>980</v>
+        <v>979</v>
       </c>
       <c r="G15" s="16"/>
       <c r="H15" s="16" t="s">
@@ -14107,11 +14206,11 @@
         <v>2</v>
       </c>
       <c r="F16" s="18" t="s">
-        <v>981</v>
+        <v>980</v>
       </c>
       <c r="G16" s="21"/>
       <c r="H16" s="21" t="s">
-        <v>917</v>
+        <v>916</v>
       </c>
     </row>
     <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -14135,7 +14234,7 @@
       </c>
       <c r="G17" s="16"/>
       <c r="H17" s="16" t="s">
-        <v>915</v>
+        <v>914</v>
       </c>
     </row>
     <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -14159,7 +14258,7 @@
       </c>
       <c r="G18" s="21"/>
       <c r="H18" s="21" t="s">
-        <v>918</v>
+        <v>917</v>
       </c>
     </row>
     <row r="19" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -14193,13 +14292,13 @@
         <v>1</v>
       </c>
       <c r="F20" s="18" t="s">
-        <v>981</v>
+        <v>980</v>
       </c>
       <c r="G20" s="27" t="s">
-        <v>1010</v>
+        <v>1009</v>
       </c>
       <c r="H20" s="16" t="s">
-        <v>1008</v>
+        <v>1007</v>
       </c>
     </row>
     <row r="21" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -14219,7 +14318,7 @@
         <v>1</v>
       </c>
       <c r="F21" s="18" t="s">
-        <v>980</v>
+        <v>979</v>
       </c>
       <c r="G21" s="21"/>
       <c r="H21" s="21"/>
@@ -14245,7 +14344,7 @@
       </c>
       <c r="G22" s="16"/>
       <c r="H22" s="16" t="s">
-        <v>916</v>
+        <v>915</v>
       </c>
     </row>
     <row r="23" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -14265,11 +14364,11 @@
         <v>2</v>
       </c>
       <c r="F23" s="18" t="s">
-        <v>981</v>
+        <v>980</v>
       </c>
       <c r="G23" s="21"/>
       <c r="H23" s="21" t="s">
-        <v>916</v>
+        <v>915</v>
       </c>
     </row>
     <row r="24" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -14413,7 +14512,7 @@
         <v>1</v>
       </c>
       <c r="F30" s="18" t="s">
-        <v>981</v>
+        <v>980</v>
       </c>
       <c r="G30" s="21"/>
       <c r="H30" s="21"/>
@@ -14439,7 +14538,7 @@
       </c>
       <c r="G31" s="16"/>
       <c r="H31" s="16" t="s">
-        <v>919</v>
+        <v>918</v>
       </c>
     </row>
     <row r="32" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -14463,7 +14562,7 @@
       </c>
       <c r="G32" s="21"/>
       <c r="H32" s="21" t="s">
-        <v>920</v>
+        <v>919</v>
       </c>
     </row>
     <row r="33" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -14545,7 +14644,7 @@
       </c>
       <c r="G36" s="16"/>
       <c r="H36" s="16" t="s">
-        <v>919</v>
+        <v>918</v>
       </c>
     </row>
     <row r="37" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -14569,7 +14668,7 @@
       </c>
       <c r="G37" s="21"/>
       <c r="H37" s="21" t="s">
-        <v>917</v>
+        <v>916</v>
       </c>
     </row>
     <row r="38" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -14593,7 +14692,7 @@
       </c>
       <c r="G38" s="16"/>
       <c r="H38" s="16" t="s">
-        <v>918</v>
+        <v>917</v>
       </c>
     </row>
     <row r="39" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -14617,7 +14716,7 @@
       </c>
       <c r="G39" s="21"/>
       <c r="H39" s="21" t="s">
-        <v>918</v>
+        <v>917</v>
       </c>
     </row>
     <row r="40" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -14641,7 +14740,7 @@
       </c>
       <c r="G40" s="16"/>
       <c r="H40" s="16" t="s">
-        <v>921</v>
+        <v>920</v>
       </c>
     </row>
     <row r="41" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -14745,7 +14844,7 @@
       </c>
       <c r="G45" s="16"/>
       <c r="H45" s="16" t="s">
-        <v>916</v>
+        <v>915</v>
       </c>
     </row>
     <row r="46" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -14769,7 +14868,7 @@
       </c>
       <c r="G46" s="21"/>
       <c r="H46" s="21" t="s">
-        <v>919</v>
+        <v>918</v>
       </c>
     </row>
     <row r="47" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -14793,7 +14892,7 @@
       </c>
       <c r="G47" s="16"/>
       <c r="H47" s="16" t="s">
-        <v>922</v>
+        <v>921</v>
       </c>
     </row>
     <row r="48" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -14931,11 +15030,11 @@
         <v>2</v>
       </c>
       <c r="F54" s="18" t="s">
-        <v>980</v>
+        <v>979</v>
       </c>
       <c r="G54" s="21"/>
       <c r="H54" s="21" t="s">
-        <v>919</v>
+        <v>918</v>
       </c>
     </row>
     <row r="55" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -14959,7 +15058,7 @@
       </c>
       <c r="G55" s="16"/>
       <c r="H55" s="16" t="s">
-        <v>919</v>
+        <v>918</v>
       </c>
     </row>
     <row r="56" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -14983,7 +15082,7 @@
       </c>
       <c r="G56" s="21"/>
       <c r="H56" s="21" t="s">
-        <v>916</v>
+        <v>915</v>
       </c>
     </row>
   </sheetData>
@@ -15085,7 +15184,7 @@
       </c>
       <c r="G3" s="16"/>
       <c r="H3" s="16" t="s">
-        <v>919</v>
+        <v>918</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -15109,7 +15208,7 @@
       </c>
       <c r="G4" s="21"/>
       <c r="H4" s="21" t="s">
-        <v>923</v>
+        <v>922</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -15133,7 +15232,7 @@
       </c>
       <c r="G5" s="16"/>
       <c r="H5" s="16" t="s">
-        <v>924</v>
+        <v>923</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -15167,7 +15266,7 @@
         <v>1</v>
       </c>
       <c r="F7" s="18" t="s">
-        <v>980</v>
+        <v>979</v>
       </c>
       <c r="G7" s="16"/>
       <c r="H7" s="16"/>
@@ -15189,7 +15288,7 @@
         <v>1</v>
       </c>
       <c r="F8" s="18" t="s">
-        <v>981</v>
+        <v>980</v>
       </c>
       <c r="G8" s="21"/>
       <c r="H8" s="21"/>
@@ -15273,7 +15372,7 @@
       </c>
       <c r="G12" s="16"/>
       <c r="H12" s="16" t="s">
-        <v>919</v>
+        <v>918</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -15293,11 +15392,11 @@
         <v>2</v>
       </c>
       <c r="F13" s="18" t="s">
-        <v>980</v>
+        <v>979</v>
       </c>
       <c r="G13" s="21"/>
       <c r="H13" s="21" t="s">
-        <v>919</v>
+        <v>918</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -15379,7 +15478,7 @@
       </c>
       <c r="G17" s="16"/>
       <c r="H17" s="16" t="s">
-        <v>925</v>
+        <v>924</v>
       </c>
     </row>
     <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -15403,7 +15502,7 @@
       </c>
       <c r="G18" s="21"/>
       <c r="H18" s="21" t="s">
-        <v>926</v>
+        <v>925</v>
       </c>
     </row>
     <row r="19" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -15427,7 +15526,7 @@
       </c>
       <c r="G19" s="16"/>
       <c r="H19" s="16" t="s">
-        <v>927</v>
+        <v>926</v>
       </c>
     </row>
     <row r="20" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -15465,7 +15564,7 @@
       </c>
       <c r="G21" s="16"/>
       <c r="H21" s="16" t="s">
-        <v>916</v>
+        <v>915</v>
       </c>
     </row>
     <row r="22" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -15489,7 +15588,7 @@
       </c>
       <c r="G22" s="21"/>
       <c r="H22" s="21" t="s">
-        <v>925</v>
+        <v>924</v>
       </c>
     </row>
     <row r="23" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -15549,7 +15648,7 @@
       </c>
       <c r="G25" s="16"/>
       <c r="H25" s="16" t="s">
-        <v>924</v>
+        <v>923</v>
       </c>
     </row>
     <row r="26" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -15569,7 +15668,7 @@
         <v>2</v>
       </c>
       <c r="F26" s="18" t="s">
-        <v>980</v>
+        <v>979</v>
       </c>
       <c r="G26" s="21"/>
       <c r="H26" s="21" t="s">
@@ -15671,13 +15770,13 @@
         <v>1</v>
       </c>
       <c r="F3" s="18" t="s">
-        <v>981</v>
+        <v>980</v>
       </c>
       <c r="G3" s="16" t="s">
-        <v>1005</v>
+        <v>1004</v>
       </c>
       <c r="H3" s="16" t="s">
-        <v>1004</v>
+        <v>1003</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -15801,13 +15900,13 @@
         <v>1</v>
       </c>
       <c r="F9" s="18" t="s">
-        <v>981</v>
+        <v>980</v>
       </c>
       <c r="G9" s="21" t="s">
-        <v>991</v>
+        <v>990</v>
       </c>
       <c r="H9" s="21" t="s">
-        <v>1002</v>
+        <v>1001</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -15887,13 +15986,13 @@
         <v>1</v>
       </c>
       <c r="F13" s="18" t="s">
-        <v>981</v>
+        <v>980</v>
       </c>
       <c r="G13" s="16" t="s">
-        <v>1005</v>
+        <v>1004</v>
       </c>
       <c r="H13" s="16" t="s">
-        <v>1004</v>
+        <v>1003</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">

</xml_diff>